<commit_message>
update LNG import emissions from USA
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
+++ b/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79324A41-8810-43F9-948A-307EBB6089FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A619179-851B-422F-BAFA-D75492A89AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BAA9D55F-0FEB-4558-AFDF-92239B956412}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="71">
   <si>
     <t>AL</t>
   </si>
@@ -196,6 +196,60 @@
   </si>
   <si>
     <t>Node</t>
+  </si>
+  <si>
+    <t>USA_LNG</t>
+  </si>
+  <si>
+    <t>BE_LNG</t>
+  </si>
+  <si>
+    <t>FR_LNG</t>
+  </si>
+  <si>
+    <t>EL_LNG</t>
+  </si>
+  <si>
+    <t>IT_LNG</t>
+  </si>
+  <si>
+    <t>HR_LNG</t>
+  </si>
+  <si>
+    <t>LT_LNG</t>
+  </si>
+  <si>
+    <t>NL_LNG</t>
+  </si>
+  <si>
+    <t>PL_LNG</t>
+  </si>
+  <si>
+    <t>PT_LNG</t>
+  </si>
+  <si>
+    <t>ES_LNG</t>
+  </si>
+  <si>
+    <t>TR_LNG</t>
+  </si>
+  <si>
+    <t>UK_LNG</t>
+  </si>
+  <si>
+    <t>EE_LNG</t>
+  </si>
+  <si>
+    <t>FI_LNG</t>
+  </si>
+  <si>
+    <t>DE_LNG</t>
+  </si>
+  <si>
+    <t>IE_LNG</t>
+  </si>
+  <si>
+    <t>LV_LNG</t>
   </si>
 </sst>
 </file>
@@ -567,10 +621,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6177B6A9-4CD7-49C9-8407-62B26396811D}">
-  <dimension ref="A1:Q37"/>
+  <dimension ref="A1:AA37"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="26" max="26" width="11.81640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>52</v>
       </c>
@@ -622,8 +679,15 @@
       <c r="Q1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="T1">
+        <v>3600000</v>
+      </c>
+      <c r="U1">
+        <f>1000*1000</f>
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -631,52 +695,64 @@
         <v>0</v>
       </c>
       <c r="C2">
-        <v>50</v>
+        <v>81.639529411764684</v>
       </c>
       <c r="D2">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E2">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F2">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G2">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H2">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I2">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J2">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K2">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L2">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M2">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N2">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O2">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P2">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+      <c r="S2">
+        <f>22.6-2.1</f>
+        <v>20.5</v>
+      </c>
+      <c r="T2">
+        <f>S2*T1</f>
+        <v>73800000</v>
+      </c>
+      <c r="U2">
+        <f>T2/U1</f>
+        <v>73.8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -684,52 +760,52 @@
         <v>1</v>
       </c>
       <c r="C3">
-        <v>50</v>
+        <v>81.639529411764684</v>
       </c>
       <c r="D3">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E3">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F3">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G3">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H3">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I3">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J3">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K3">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L3">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M3">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N3">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O3">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P3">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q3">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -737,52 +813,55 @@
         <v>1</v>
       </c>
       <c r="C4">
-        <v>50</v>
+        <v>81.028026845637584</v>
       </c>
       <c r="D4">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E4">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F4">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G4">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H4">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I4">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J4">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K4">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L4">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M4">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N4">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O4">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P4">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+      <c r="S4">
+        <v>20.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -790,52 +869,55 @@
         <v>0</v>
       </c>
       <c r="C5">
-        <v>50</v>
+        <v>81.639529411764684</v>
       </c>
       <c r="D5">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E5">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F5">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G5">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H5">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I5">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J5">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K5">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L5">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M5">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N5">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O5">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P5">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+      <c r="S5">
+        <v>18.7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -843,52 +925,56 @@
         <v>1</v>
       </c>
       <c r="C6">
-        <v>50</v>
+        <v>81.639529411764684</v>
       </c>
       <c r="D6">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E6">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F6">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G6">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H6">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I6">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J6">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K6">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L6">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M6">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N6">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O6">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P6">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q6">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+      <c r="S6">
+        <f>(S5+S4)/2</f>
+        <v>19.600000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -896,52 +982,52 @@
         <v>1</v>
       </c>
       <c r="C7">
-        <v>50</v>
+        <v>83.048859060402691</v>
       </c>
       <c r="D7">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E7">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F7">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G7">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H7">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I7">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J7">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K7">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L7">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M7">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N7">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O7">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P7">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -949,52 +1035,79 @@
         <v>1</v>
       </c>
       <c r="C8">
-        <v>50</v>
+        <v>81.639529411764684</v>
       </c>
       <c r="D8">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E8">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F8">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G8">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H8">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I8">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J8">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K8">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L8">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M8">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N8">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O8">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P8">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q8">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+      <c r="R8">
+        <f>AA8</f>
+        <v>81.028026845637584</v>
+      </c>
+      <c r="S8" t="s">
+        <v>53</v>
+      </c>
+      <c r="T8" t="s">
+        <v>54</v>
+      </c>
+      <c r="W8">
+        <v>0</v>
+      </c>
+      <c r="X8">
+        <v>4986</v>
+      </c>
+      <c r="Y8">
+        <v>8024.1916664923037</v>
+      </c>
+      <c r="Z8">
+        <f>(((2.1/$Y$22)*Y8)*$T$1)/$U$1</f>
+        <v>7.2280268456375838</v>
+      </c>
+      <c r="AA8">
+        <f>Z8+$U$2</f>
+        <v>81.028026845637584</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -1002,52 +1115,79 @@
         <v>1</v>
       </c>
       <c r="C9">
-        <v>50</v>
+        <v>81.639529411764684</v>
       </c>
       <c r="D9">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E9">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F9">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G9">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H9">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I9">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J9">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K9">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L9">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M9">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N9">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O9">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P9">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q9">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+      <c r="R9">
+        <f>AA9</f>
+        <v>80.987436241610737</v>
+      </c>
+      <c r="S9" t="s">
+        <v>53</v>
+      </c>
+      <c r="T9" t="s">
+        <v>55</v>
+      </c>
+      <c r="W9">
+        <v>0</v>
+      </c>
+      <c r="X9">
+        <v>4958</v>
+      </c>
+      <c r="Y9">
+        <v>7979.1300205513126</v>
+      </c>
+      <c r="Z9">
+        <f t="shared" ref="Z9:Z24" si="0">(((2.1/$Y$22)*Y9)*$T$1)/$U$1</f>
+        <v>7.1874362416107402</v>
+      </c>
+      <c r="AA9">
+        <f t="shared" ref="AA9:AA24" si="1">Z9+$U$2</f>
+        <v>80.987436241610737</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1055,52 +1195,79 @@
         <v>1</v>
       </c>
       <c r="C10">
-        <v>50</v>
+        <v>82.274738255033554</v>
       </c>
       <c r="D10">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E10">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F10">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G10">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H10">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I10">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J10">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K10">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L10">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M10">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N10">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O10">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P10">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+      <c r="R10">
+        <f>AA10</f>
+        <v>82.867651006711412</v>
+      </c>
+      <c r="S10" t="s">
+        <v>53</v>
+      </c>
+      <c r="T10" t="s">
+        <v>56</v>
+      </c>
+      <c r="W10">
+        <v>0</v>
+      </c>
+      <c r="X10">
+        <v>6255</v>
+      </c>
+      <c r="Y10">
+        <v>10066.449834317962</v>
+      </c>
+      <c r="Z10">
+        <f t="shared" si="0"/>
+        <v>9.0676510067114116</v>
+      </c>
+      <c r="AA10">
+        <f t="shared" si="1"/>
+        <v>82.867651006711412</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1108,52 +1275,79 @@
         <v>1</v>
       </c>
       <c r="C11">
-        <v>50</v>
+        <v>82.274738255033554</v>
       </c>
       <c r="D11">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E11">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F11">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G11">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H11">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I11">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J11">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K11">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L11">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M11">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N11">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O11">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P11">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q11">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+      <c r="R11">
+        <f>AA11</f>
+        <v>81.963060402684562</v>
+      </c>
+      <c r="S11" t="s">
+        <v>53</v>
+      </c>
+      <c r="T11" t="s">
+        <v>57</v>
+      </c>
+      <c r="W11">
+        <v>0</v>
+      </c>
+      <c r="X11">
+        <v>5631</v>
+      </c>
+      <c r="Y11">
+        <v>9062.2188676330043</v>
+      </c>
+      <c r="Z11">
+        <f t="shared" si="0"/>
+        <v>8.1630604026845646</v>
+      </c>
+      <c r="AA11">
+        <f t="shared" si="1"/>
+        <v>81.963060402684562</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1161,52 +1355,79 @@
         <v>1</v>
       </c>
       <c r="C12">
-        <v>50</v>
+        <v>80.987436241610737</v>
       </c>
       <c r="D12">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E12">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F12">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G12">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H12">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I12">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J12">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K12">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L12">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M12">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N12">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O12">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P12">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q12">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+      <c r="R12">
+        <f>AA12</f>
+        <v>83.048859060402691</v>
+      </c>
+      <c r="S12" t="s">
+        <v>53</v>
+      </c>
+      <c r="T12" t="s">
+        <v>58</v>
+      </c>
+      <c r="W12">
+        <v>0</v>
+      </c>
+      <c r="X12">
+        <v>6380</v>
+      </c>
+      <c r="Y12">
+        <v>10267.617896554533</v>
+      </c>
+      <c r="Z12">
+        <f t="shared" si="0"/>
+        <v>9.2488590604026868</v>
+      </c>
+      <c r="AA12">
+        <f t="shared" si="1"/>
+        <v>83.048859060402691</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -1214,52 +1435,79 @@
         <v>1</v>
       </c>
       <c r="C13">
-        <v>50</v>
+        <v>81.36</v>
       </c>
       <c r="D13">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E13">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F13">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G13">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H13">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I13">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J13">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K13">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L13">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M13">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N13">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O13">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P13">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q13">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+      <c r="R13">
+        <f>AA13</f>
+        <v>81.967409395973149</v>
+      </c>
+      <c r="S13" t="s">
+        <v>53</v>
+      </c>
+      <c r="T13" t="s">
+        <v>59</v>
+      </c>
+      <c r="W13">
+        <v>0</v>
+      </c>
+      <c r="X13">
+        <v>5634</v>
+      </c>
+      <c r="Y13">
+        <v>9067.0469011266832</v>
+      </c>
+      <c r="Z13">
+        <f t="shared" si="0"/>
+        <v>8.1674093959731557</v>
+      </c>
+      <c r="AA13">
+        <f t="shared" si="1"/>
+        <v>81.967409395973149</v>
+      </c>
+    </row>
+    <row r="14" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -1267,52 +1515,79 @@
         <v>1</v>
       </c>
       <c r="C14">
-        <v>50</v>
+        <v>82.867651006711412</v>
       </c>
       <c r="D14">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E14">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F14">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G14">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H14">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I14">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J14">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K14">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L14">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M14">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N14">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O14">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P14">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q14">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+      <c r="R14">
+        <f>AA14</f>
+        <v>81.123704697986582</v>
+      </c>
+      <c r="S14" t="s">
+        <v>53</v>
+      </c>
+      <c r="T14" t="s">
+        <v>60</v>
+      </c>
+      <c r="W14">
+        <v>0</v>
+      </c>
+      <c r="X14">
+        <v>5052</v>
+      </c>
+      <c r="Y14">
+        <v>8130.4084033532126</v>
+      </c>
+      <c r="Z14">
+        <f t="shared" si="0"/>
+        <v>7.323704697986579</v>
+      </c>
+      <c r="AA14">
+        <f t="shared" si="1"/>
+        <v>81.123704697986582</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -1320,52 +1595,79 @@
         <v>1</v>
       </c>
       <c r="C15">
-        <v>50</v>
+        <v>81.639529411764684</v>
       </c>
       <c r="D15">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E15">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F15">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G15">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H15">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I15">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J15">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K15">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L15">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M15">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N15">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O15">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P15">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q15">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+      <c r="R15">
+        <f>AA15</f>
+        <v>81.690523489932886</v>
+      </c>
+      <c r="S15" t="s">
+        <v>53</v>
+      </c>
+      <c r="T15" t="s">
+        <v>61</v>
+      </c>
+      <c r="W15">
+        <v>0</v>
+      </c>
+      <c r="X15">
+        <v>5443</v>
+      </c>
+      <c r="Y15">
+        <v>8759.6621020292041</v>
+      </c>
+      <c r="Z15">
+        <f t="shared" si="0"/>
+        <v>7.8905234899328871</v>
+      </c>
+      <c r="AA15">
+        <f t="shared" si="1"/>
+        <v>81.690523489932886</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -1373,52 +1675,79 @@
         <v>1</v>
       </c>
       <c r="C16">
-        <v>50</v>
+        <v>80.416268456375832</v>
       </c>
       <c r="D16">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E16">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F16">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G16">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H16">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I16">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J16">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K16">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L16">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M16">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N16">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O16">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P16">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q16">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+      <c r="R16">
+        <f>AA16</f>
+        <v>80.417718120805375</v>
+      </c>
+      <c r="S16" t="s">
+        <v>53</v>
+      </c>
+      <c r="T16" t="s">
+        <v>62</v>
+      </c>
+      <c r="W16">
+        <v>0</v>
+      </c>
+      <c r="X16">
+        <v>4565</v>
+      </c>
+      <c r="Y16">
+        <v>7346.6576328795363</v>
+      </c>
+      <c r="Z16">
+        <f t="shared" si="0"/>
+        <v>6.617718120805371</v>
+      </c>
+      <c r="AA16">
+        <f t="shared" si="1"/>
+        <v>80.417718120805375</v>
+      </c>
+    </row>
+    <row r="17" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -1426,52 +1755,79 @@
         <v>1</v>
       </c>
       <c r="C17">
-        <v>50</v>
+        <v>81.963060402684562</v>
       </c>
       <c r="D17">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E17">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F17">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G17">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H17">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I17">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J17">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K17">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L17">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M17">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N17">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O17">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P17">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q17">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+      <c r="R17">
+        <f>AA17</f>
+        <v>80.609073825503359</v>
+      </c>
+      <c r="S17" t="s">
+        <v>53</v>
+      </c>
+      <c r="T17" t="s">
+        <v>63</v>
+      </c>
+      <c r="W17">
+        <v>0</v>
+      </c>
+      <c r="X17">
+        <v>4697</v>
+      </c>
+      <c r="Y17">
+        <v>7559.0911066013541</v>
+      </c>
+      <c r="Z17">
+        <f t="shared" si="0"/>
+        <v>6.8090738255033578</v>
+      </c>
+      <c r="AA17">
+        <f t="shared" si="1"/>
+        <v>80.609073825503359</v>
+      </c>
+    </row>
+    <row r="18" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -1479,52 +1835,79 @@
         <v>1</v>
       </c>
       <c r="C18">
-        <v>50</v>
+        <v>82.187758389261745</v>
       </c>
       <c r="D18">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E18">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F18">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G18">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H18">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I18">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J18">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K18">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L18">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M18">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N18">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O18">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P18">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q18">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+      <c r="R18">
+        <f>AA18</f>
+        <v>83.090899328859052</v>
+      </c>
+      <c r="S18" t="s">
+        <v>53</v>
+      </c>
+      <c r="T18" t="s">
+        <v>64</v>
+      </c>
+      <c r="W18">
+        <v>0</v>
+      </c>
+      <c r="X18">
+        <v>6409</v>
+      </c>
+      <c r="Y18">
+        <v>10314.288886993416</v>
+      </c>
+      <c r="Z18">
+        <f t="shared" si="0"/>
+        <v>9.2908993288590622</v>
+      </c>
+      <c r="AA18">
+        <f t="shared" si="1"/>
+        <v>83.090899328859052</v>
+      </c>
+    </row>
+    <row r="19" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>17</v>
       </c>
@@ -1532,52 +1915,79 @@
         <v>1</v>
       </c>
       <c r="C19">
-        <v>50</v>
+        <v>81.967409395973149</v>
       </c>
       <c r="D19">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E19">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F19">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G19">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H19">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I19">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J19">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K19">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L19">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M19">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N19">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O19">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P19">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q19">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+      <c r="R19">
+        <f>AA19</f>
+        <v>80.564134228187925</v>
+      </c>
+      <c r="S19" t="s">
+        <v>53</v>
+      </c>
+      <c r="T19" t="s">
+        <v>65</v>
+      </c>
+      <c r="W19">
+        <v>0</v>
+      </c>
+      <c r="X19">
+        <v>4666</v>
+      </c>
+      <c r="Y19">
+        <v>7509.2014271666849</v>
+      </c>
+      <c r="Z19">
+        <f t="shared" si="0"/>
+        <v>6.7641342281879213</v>
+      </c>
+      <c r="AA19">
+        <f t="shared" si="1"/>
+        <v>80.564134228187925</v>
+      </c>
+    </row>
+    <row r="20" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>18</v>
       </c>
@@ -1585,52 +1995,79 @@
         <v>1</v>
       </c>
       <c r="C20">
-        <v>50</v>
+        <v>81.639529411764684</v>
       </c>
       <c r="D20">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E20">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F20">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G20">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H20">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I20">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J20">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K20">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L20">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M20">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N20">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O20">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P20">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q20">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+      <c r="R20">
+        <f>AA20</f>
+        <v>82.274738255033554</v>
+      </c>
+      <c r="S20" t="s">
+        <v>53</v>
+      </c>
+      <c r="T20" t="s">
+        <v>66</v>
+      </c>
+      <c r="W20">
+        <v>0</v>
+      </c>
+      <c r="X20">
+        <v>5846</v>
+      </c>
+      <c r="Y20">
+        <v>9408.227934679906</v>
+      </c>
+      <c r="Z20">
+        <f t="shared" si="0"/>
+        <v>8.4747382550335608</v>
+      </c>
+      <c r="AA20">
+        <f t="shared" si="1"/>
+        <v>82.274738255033554</v>
+      </c>
+    </row>
+    <row r="21" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -1638,52 +2075,79 @@
         <v>0</v>
       </c>
       <c r="C21">
-        <v>50</v>
+        <v>81.639529411764684</v>
       </c>
       <c r="D21">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E21">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F21">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G21">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H21">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I21">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J21">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K21">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L21">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M21">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N21">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O21">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P21">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q21">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+      <c r="R21">
+        <f>AA21</f>
+        <v>82.274738255033554</v>
+      </c>
+      <c r="S21" t="s">
+        <v>53</v>
+      </c>
+      <c r="T21" t="s">
+        <v>67</v>
+      </c>
+      <c r="W21">
+        <v>0</v>
+      </c>
+      <c r="X21">
+        <v>5846</v>
+      </c>
+      <c r="Y21">
+        <v>9408.227934679906</v>
+      </c>
+      <c r="Z21">
+        <f t="shared" si="0"/>
+        <v>8.4747382550335608</v>
+      </c>
+      <c r="AA21">
+        <f t="shared" si="1"/>
+        <v>82.274738255033554</v>
+      </c>
+    </row>
+    <row r="22" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -1691,52 +2155,79 @@
         <v>1</v>
       </c>
       <c r="C22">
-        <v>50</v>
+        <v>81.123704697986582</v>
       </c>
       <c r="D22">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E22">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F22">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G22">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H22">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I22">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J22">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K22">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L22">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M22">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N22">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O22">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P22">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q22">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+      <c r="R22">
+        <f>AA22</f>
+        <v>81.36</v>
+      </c>
+      <c r="S22" t="s">
+        <v>53</v>
+      </c>
+      <c r="T22" t="s">
+        <v>68</v>
+      </c>
+      <c r="W22">
+        <v>0</v>
+      </c>
+      <c r="X22">
+        <v>5215</v>
+      </c>
+      <c r="Y22">
+        <v>8392.7315565096997</v>
+      </c>
+      <c r="Z22">
+        <f t="shared" si="0"/>
+        <v>7.56</v>
+      </c>
+      <c r="AA22">
+        <f t="shared" si="1"/>
+        <v>81.36</v>
+      </c>
+    </row>
+    <row r="23" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -1744,52 +2235,79 @@
         <v>0</v>
       </c>
       <c r="C23">
-        <v>50</v>
+        <v>81.639529411764684</v>
       </c>
       <c r="D23">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E23">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F23">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G23">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H23">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I23">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J23">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K23">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L23">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M23">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N23">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O23">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P23">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q23">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+      <c r="R23">
+        <f>AA23</f>
+        <v>80.416268456375832</v>
+      </c>
+      <c r="S23" t="s">
+        <v>53</v>
+      </c>
+      <c r="T23" t="s">
+        <v>69</v>
+      </c>
+      <c r="W23">
+        <v>0</v>
+      </c>
+      <c r="X23">
+        <v>4564</v>
+      </c>
+      <c r="Y23">
+        <v>7345.0482883816439</v>
+      </c>
+      <c r="Z23">
+        <f t="shared" si="0"/>
+        <v>6.61626845637584</v>
+      </c>
+      <c r="AA23">
+        <f t="shared" si="1"/>
+        <v>80.416268456375832</v>
+      </c>
+    </row>
+    <row r="24" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>22</v>
       </c>
@@ -1797,52 +2315,79 @@
         <v>0</v>
       </c>
       <c r="C24">
-        <v>50</v>
+        <v>81.639529411764684</v>
       </c>
       <c r="D24">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E24">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F24">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G24">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H24">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I24">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J24">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K24">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L24">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M24">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N24">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O24">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P24">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q24">
+        <v>9.36</v>
+      </c>
+      <c r="R24">
+        <f>AA24</f>
+        <v>82.187758389261745</v>
+      </c>
+      <c r="S24" t="s">
+        <v>53</v>
+      </c>
+      <c r="T24" t="s">
+        <v>70</v>
+      </c>
+      <c r="W24">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="X24">
+        <v>5786</v>
+      </c>
+      <c r="Y24">
+        <v>9311.6672648063523</v>
+      </c>
+      <c r="Z24">
+        <f t="shared" si="0"/>
+        <v>8.3877583892617462</v>
+      </c>
+      <c r="AA24">
+        <f t="shared" si="1"/>
+        <v>82.187758389261745</v>
+      </c>
+    </row>
+    <row r="25" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -1850,52 +2395,56 @@
         <v>1</v>
       </c>
       <c r="C25">
-        <v>50</v>
+        <v>81.690523489932886</v>
       </c>
       <c r="D25">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E25">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F25">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G25">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H25">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I25">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J25">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K25">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L25">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M25">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N25">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O25">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P25">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q25">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+      <c r="R25">
+        <f>AVERAGE(R8:R24)</f>
+        <v>81.639529411764684</v>
+      </c>
+    </row>
+    <row r="26" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>24</v>
       </c>
@@ -1903,52 +2452,52 @@
         <v>1</v>
       </c>
       <c r="C26">
-        <v>50</v>
+        <v>80.417718120805375</v>
       </c>
       <c r="D26">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E26">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F26">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G26">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H26">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I26">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J26">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K26">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L26">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M26">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N26">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O26">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P26">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q26">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+    </row>
+    <row r="27" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>25</v>
       </c>
@@ -1956,52 +2505,52 @@
         <v>1</v>
       </c>
       <c r="C27">
-        <v>50</v>
+        <v>81.639529411764684</v>
       </c>
       <c r="D27">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E27">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F27">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G27">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H27">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I27">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J27">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K27">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L27">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M27">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N27">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O27">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P27">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q27">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+    </row>
+    <row r="28" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>26</v>
       </c>
@@ -2009,52 +2558,52 @@
         <v>0</v>
       </c>
       <c r="C28">
-        <v>50</v>
+        <v>81.639529411764684</v>
       </c>
       <c r="D28">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E28">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F28">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G28">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H28">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I28">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J28">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K28">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L28">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M28">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N28">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O28">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P28">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q28">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+    </row>
+    <row r="29" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>27</v>
       </c>
@@ -2062,52 +2611,52 @@
         <v>0</v>
       </c>
       <c r="C29">
-        <v>50</v>
+        <v>81.639529411764684</v>
       </c>
       <c r="D29">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E29">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F29">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G29">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H29">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I29">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J29">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K29">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L29">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M29">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N29">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O29">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P29">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q29">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+    </row>
+    <row r="30" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>28</v>
       </c>
@@ -2115,52 +2664,52 @@
         <v>1</v>
       </c>
       <c r="C30">
-        <v>50</v>
+        <v>81.639529411764684</v>
       </c>
       <c r="D30">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E30">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F30">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G30">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H30">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I30">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J30">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K30">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L30">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M30">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N30">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O30">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P30">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q30">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+    </row>
+    <row r="31" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>29</v>
       </c>
@@ -2168,52 +2717,52 @@
         <v>1</v>
       </c>
       <c r="C31">
-        <v>50</v>
+        <v>81.639529411764684</v>
       </c>
       <c r="D31">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E31">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F31">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G31">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H31">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I31">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J31">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K31">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L31">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M31">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N31">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O31">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P31">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q31">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.35">
+        <v>9.36</v>
+      </c>
+    </row>
+    <row r="32" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>30</v>
       </c>
@@ -2221,49 +2770,49 @@
         <v>1</v>
       </c>
       <c r="C32">
-        <v>50</v>
+        <v>80.609073825503359</v>
       </c>
       <c r="D32">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E32">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F32">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G32">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H32">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I32">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J32">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K32">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L32">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M32">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N32">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O32">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P32">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q32">
-        <v>3</v>
+        <v>9.36</v>
       </c>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.35">
@@ -2274,49 +2823,49 @@
         <v>1</v>
       </c>
       <c r="C33">
-        <v>50</v>
+        <v>81.639529411764684</v>
       </c>
       <c r="D33">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E33">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F33">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G33">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H33">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I33">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J33">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K33">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L33">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M33">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N33">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O33">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P33">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q33">
-        <v>3</v>
+        <v>9.36</v>
       </c>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.35">
@@ -2327,49 +2876,49 @@
         <v>0</v>
       </c>
       <c r="C34">
-        <v>50</v>
+        <v>81.639529411764684</v>
       </c>
       <c r="D34">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E34">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F34">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G34">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H34">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I34">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J34">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K34">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L34">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M34">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N34">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O34">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P34">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q34">
-        <v>3</v>
+        <v>9.36</v>
       </c>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.35">
@@ -2380,49 +2929,49 @@
         <v>0</v>
       </c>
       <c r="C35">
-        <v>50</v>
+        <v>83.090899328859052</v>
       </c>
       <c r="D35">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E35">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F35">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G35">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H35">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I35">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J35">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K35">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L35">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M35">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N35">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O35">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P35">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q35">
-        <v>3</v>
+        <v>9.36</v>
       </c>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.35">
@@ -2433,49 +2982,49 @@
         <v>0</v>
       </c>
       <c r="C36">
-        <v>50</v>
+        <v>80.564134228187925</v>
       </c>
       <c r="D36">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E36">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F36">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G36">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H36">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I36">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J36">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K36">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L36">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M36">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N36">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O36">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P36">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q36">
-        <v>3</v>
+        <v>9.36</v>
       </c>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.35">
@@ -2486,49 +3035,49 @@
         <v>0</v>
       </c>
       <c r="C37">
-        <v>50</v>
+        <v>81.639529411764684</v>
       </c>
       <c r="D37">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E37">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="F37">
-        <v>30</v>
+        <v>63.72</v>
       </c>
       <c r="G37">
-        <v>20</v>
+        <v>74.52</v>
       </c>
       <c r="H37">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I37">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="J37">
-        <v>6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="K37">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="L37">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="M37">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="N37">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="O37">
-        <v>5</v>
+        <v>72.72</v>
       </c>
       <c r="P37">
-        <v>40</v>
+        <v>70.56</v>
       </c>
       <c r="Q37">
-        <v>3</v>
+        <v>9.36</v>
       </c>
     </row>
   </sheetData>
@@ -2554,7 +3103,7 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -2562,7 +3111,7 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -2570,7 +3119,7 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -2578,7 +3127,7 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
@@ -2586,7 +3135,7 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -2594,7 +3143,7 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -2602,7 +3151,7 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
@@ -2610,7 +3159,7 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
@@ -2618,7 +3167,7 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
@@ -2626,7 +3175,7 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
@@ -2634,7 +3183,7 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
@@ -2642,7 +3191,7 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
@@ -2650,7 +3199,7 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
@@ -2658,7 +3207,7 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
@@ -2666,7 +3215,7 @@
         <v>14</v>
       </c>
       <c r="B16">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
@@ -2674,7 +3223,7 @@
         <v>15</v>
       </c>
       <c r="B17">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
@@ -2682,7 +3231,7 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
@@ -2690,7 +3239,7 @@
         <v>17</v>
       </c>
       <c r="B19">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -2698,7 +3247,7 @@
         <v>18</v>
       </c>
       <c r="B20">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
@@ -2706,7 +3255,7 @@
         <v>19</v>
       </c>
       <c r="B21">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
@@ -2714,7 +3263,7 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>3</v>
+        <v>8.64</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
@@ -2722,7 +3271,7 @@
         <v>21</v>
       </c>
       <c r="B23">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
@@ -2730,7 +3279,7 @@
         <v>22</v>
       </c>
       <c r="B24">
-        <v>3</v>
+        <v>7.9200000000000008</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
@@ -2738,7 +3287,7 @@
         <v>23</v>
       </c>
       <c r="B25">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
@@ -2746,7 +3295,7 @@
         <v>24</v>
       </c>
       <c r="B26">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
@@ -2754,7 +3303,7 @@
         <v>25</v>
       </c>
       <c r="B27">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.35">
@@ -2762,7 +3311,7 @@
         <v>26</v>
       </c>
       <c r="B28">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.35">
@@ -2770,7 +3319,7 @@
         <v>27</v>
       </c>
       <c r="B29">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.35">
@@ -2778,7 +3327,7 @@
         <v>28</v>
       </c>
       <c r="B30">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.35">
@@ -2786,7 +3335,7 @@
         <v>29</v>
       </c>
       <c r="B31">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.35">
@@ -2794,7 +3343,7 @@
         <v>30</v>
       </c>
       <c r="B32">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.35">
@@ -2802,7 +3351,7 @@
         <v>31</v>
       </c>
       <c r="B33">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.35">
@@ -2810,7 +3359,7 @@
         <v>32</v>
       </c>
       <c r="B34">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.35">
@@ -2818,7 +3367,7 @@
         <v>33</v>
       </c>
       <c r="B35">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.35">
@@ -2826,7 +3375,7 @@
         <v>34</v>
       </c>
       <c r="B36">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.35">
@@ -2834,7 +3383,7 @@
         <v>35</v>
       </c>
       <c r="B37">
-        <v>3</v>
+        <v>23.04</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update emission factors for imports from QA
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
+++ b/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A619179-851B-422F-BAFA-D75492A89AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0E8D1F3-74C5-4280-A375-F2494D6D72C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BAA9D55F-0FEB-4558-AFDF-92239B956412}"/>
   </bookViews>
@@ -198,9 +198,6 @@
     <t>Node</t>
   </si>
   <si>
-    <t>USA_LNG</t>
-  </si>
-  <si>
     <t>BE_LNG</t>
   </si>
   <si>
@@ -250,6 +247,9 @@
   </si>
   <si>
     <t>LV_LNG</t>
+  </si>
+  <si>
+    <t>QA_LNG</t>
   </si>
 </sst>
 </file>
@@ -701,10 +701,10 @@
         <v>70</v>
       </c>
       <c r="E2">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="F2">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="G2">
         <v>74.52</v>
@@ -740,16 +740,16 @@
         <v>9.36</v>
       </c>
       <c r="S2">
-        <f>22.6-2.1</f>
-        <v>20.5</v>
+        <f>U5-U4</f>
+        <v>15.1</v>
       </c>
       <c r="T2">
         <f>S2*T1</f>
-        <v>73800000</v>
+        <v>54360000</v>
       </c>
       <c r="U2">
         <f>T2/U1</f>
-        <v>73.8</v>
+        <v>54.36</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.35">
@@ -766,10 +766,10 @@
         <v>70</v>
       </c>
       <c r="E3">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="F3">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="G3">
         <v>74.52</v>
@@ -819,10 +819,10 @@
         <v>70</v>
       </c>
       <c r="E4">
-        <v>63.72</v>
+        <v>63.343596330275233</v>
       </c>
       <c r="F4">
-        <v>63.72</v>
+        <v>63.343596330275233</v>
       </c>
       <c r="G4">
         <v>74.52</v>
@@ -859,6 +859,9 @@
       </c>
       <c r="S4">
         <v>20.5</v>
+      </c>
+      <c r="U4">
+        <v>2.6</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.35">
@@ -875,10 +878,10 @@
         <v>70</v>
       </c>
       <c r="E5">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="F5">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="G5">
         <v>74.52</v>
@@ -915,6 +918,9 @@
       </c>
       <c r="S5">
         <v>18.7</v>
+      </c>
+      <c r="U5">
+        <v>17.7</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.35">
@@ -931,10 +937,10 @@
         <v>70</v>
       </c>
       <c r="E6">
-        <v>63.72</v>
+        <v>61.615981651376146</v>
       </c>
       <c r="F6">
-        <v>63.72</v>
+        <v>61.615981651376146</v>
       </c>
       <c r="G6">
         <v>74.52</v>
@@ -988,10 +994,10 @@
         <v>70</v>
       </c>
       <c r="E7">
-        <v>63.72</v>
+        <v>60.552770642201835</v>
       </c>
       <c r="F7">
-        <v>63.72</v>
+        <v>60.552770642201835</v>
       </c>
       <c r="G7">
         <v>74.52</v>
@@ -1041,10 +1047,10 @@
         <v>70</v>
       </c>
       <c r="E8">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="F8">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="G8">
         <v>74.52</v>
@@ -1080,31 +1086,31 @@
         <v>9.36</v>
       </c>
       <c r="R8">
-        <f>AA8</f>
-        <v>81.028026845637584</v>
+        <f t="shared" ref="R8:R24" si="0">AA8</f>
+        <v>63.343596330275233</v>
       </c>
       <c r="S8" t="s">
+        <v>70</v>
+      </c>
+      <c r="T8" t="s">
         <v>53</v>
-      </c>
-      <c r="T8" t="s">
-        <v>54</v>
       </c>
       <c r="W8">
         <v>0</v>
       </c>
       <c r="X8">
-        <v>4986</v>
+        <v>6277</v>
       </c>
       <c r="Y8">
-        <v>8024.1916664923037</v>
+        <v>10101.855413271598</v>
       </c>
       <c r="Z8">
-        <f>(((2.1/$Y$22)*Y8)*$T$1)/$U$1</f>
-        <v>7.2280268456375838</v>
+        <f>((($U$4/$Y$22)*Y8)*$T$1)/$U$1</f>
+        <v>8.9835963302752297</v>
       </c>
       <c r="AA8">
         <f>Z8+$U$2</f>
-        <v>81.028026845637584</v>
+        <v>63.343596330275233</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.35">
@@ -1121,10 +1127,10 @@
         <v>70</v>
       </c>
       <c r="E9">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="F9">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="G9">
         <v>74.52</v>
@@ -1160,31 +1166,31 @@
         <v>9.36</v>
       </c>
       <c r="R9">
-        <f>AA9</f>
-        <v>80.987436241610737</v>
+        <f t="shared" si="0"/>
+        <v>60.916293577981648</v>
       </c>
       <c r="S9" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="T9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="W9">
         <v>0</v>
       </c>
       <c r="X9">
-        <v>4958</v>
+        <v>4581</v>
       </c>
       <c r="Y9">
-        <v>7979.1300205513126</v>
+        <v>7372.4071448458171</v>
       </c>
       <c r="Z9">
-        <f t="shared" ref="Z9:Z24" si="0">(((2.1/$Y$22)*Y9)*$T$1)/$U$1</f>
-        <v>7.1874362416107402</v>
+        <f t="shared" ref="Z9:Z24" si="1">((($U$4/$Y$22)*Y9)*$T$1)/$U$1</f>
+        <v>6.556293577981652</v>
       </c>
       <c r="AA9">
-        <f t="shared" ref="AA9:AA24" si="1">Z9+$U$2</f>
-        <v>80.987436241610737</v>
+        <f t="shared" ref="AA9:AA24" si="2">Z9+$U$2</f>
+        <v>60.916293577981648</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.35">
@@ -1201,10 +1207,10 @@
         <v>70</v>
       </c>
       <c r="E10">
-        <v>63.72</v>
+        <v>64.983743119266052</v>
       </c>
       <c r="F10">
-        <v>63.72</v>
+        <v>64.983743119266052</v>
       </c>
       <c r="G10">
         <v>74.52</v>
@@ -1240,31 +1246,31 @@
         <v>9.36</v>
       </c>
       <c r="R10">
-        <f>AA10</f>
-        <v>82.867651006711412</v>
+        <f t="shared" si="0"/>
+        <v>59.609614678899085</v>
       </c>
       <c r="S10" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="T10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="W10">
         <v>0</v>
       </c>
       <c r="X10">
-        <v>6255</v>
+        <v>3668</v>
       </c>
       <c r="Y10">
-        <v>10066.449834317962</v>
+        <v>5903.0756182699097</v>
       </c>
       <c r="Z10">
-        <f t="shared" si="0"/>
-        <v>9.0676510067114116</v>
+        <f t="shared" si="1"/>
+        <v>5.249614678899083</v>
       </c>
       <c r="AA10">
-        <f t="shared" si="1"/>
-        <v>82.867651006711412</v>
+        <f t="shared" si="2"/>
+        <v>59.609614678899085</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.35">
@@ -1281,10 +1287,10 @@
         <v>70</v>
       </c>
       <c r="E11">
-        <v>63.72</v>
+        <v>64.983743119266052</v>
       </c>
       <c r="F11">
-        <v>63.72</v>
+        <v>64.983743119266052</v>
       </c>
       <c r="G11">
         <v>74.52</v>
@@ -1320,31 +1326,31 @@
         <v>9.36</v>
       </c>
       <c r="R11">
-        <f>AA11</f>
-        <v>81.963060402684562</v>
+        <f t="shared" si="0"/>
+        <v>60.62862385321101</v>
       </c>
       <c r="S11" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="T11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="W11">
         <v>0</v>
       </c>
       <c r="X11">
-        <v>5631</v>
+        <v>4380</v>
       </c>
       <c r="Y11">
-        <v>9062.2188676330043</v>
+        <v>7048.9289007694124</v>
       </c>
       <c r="Z11">
-        <f t="shared" si="0"/>
-        <v>8.1630604026845646</v>
+        <f t="shared" si="1"/>
+        <v>6.2686238532110092</v>
       </c>
       <c r="AA11">
-        <f t="shared" si="1"/>
-        <v>81.963060402684562</v>
+        <f t="shared" si="2"/>
+        <v>60.62862385321101</v>
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.35">
@@ -1361,10 +1367,10 @@
         <v>70</v>
       </c>
       <c r="E12">
-        <v>63.72</v>
+        <v>60.916293577981648</v>
       </c>
       <c r="F12">
-        <v>63.72</v>
+        <v>60.916293577981648</v>
       </c>
       <c r="G12">
         <v>74.52</v>
@@ -1400,31 +1406,31 @@
         <v>9.36</v>
       </c>
       <c r="R12">
-        <f>AA12</f>
-        <v>83.048859060402691</v>
+        <f t="shared" si="0"/>
+        <v>60.552770642201835</v>
       </c>
       <c r="S12" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="T12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="W12">
         <v>0</v>
       </c>
       <c r="X12">
-        <v>6380</v>
+        <v>4327</v>
       </c>
       <c r="Y12">
-        <v>10267.617896554533</v>
+        <v>6963.6336423811072</v>
       </c>
       <c r="Z12">
-        <f t="shared" si="0"/>
-        <v>9.2488590604026868</v>
+        <f t="shared" si="1"/>
+        <v>6.192770642201836</v>
       </c>
       <c r="AA12">
-        <f t="shared" si="1"/>
-        <v>83.048859060402691</v>
+        <f t="shared" si="2"/>
+        <v>60.552770642201835</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.35">
@@ -1480,31 +1486,31 @@
         <v>9.36</v>
       </c>
       <c r="R13">
-        <f>AA13</f>
-        <v>81.967409395973149</v>
+        <f t="shared" si="0"/>
+        <v>64.680330275229352</v>
       </c>
       <c r="S13" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="T13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="W13">
         <v>0</v>
       </c>
       <c r="X13">
-        <v>5634</v>
+        <v>7211</v>
       </c>
       <c r="Y13">
-        <v>9067.0469011266832</v>
+        <v>11604.98317430325</v>
       </c>
       <c r="Z13">
-        <f t="shared" si="0"/>
-        <v>8.1674093959731557</v>
+        <f t="shared" si="1"/>
+        <v>10.32033027522936</v>
       </c>
       <c r="AA13">
-        <f t="shared" si="1"/>
-        <v>81.967409395973149</v>
+        <f t="shared" si="2"/>
+        <v>64.680330275229352</v>
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.35">
@@ -1521,10 +1527,10 @@
         <v>70</v>
       </c>
       <c r="E14">
-        <v>63.72</v>
+        <v>59.609614678899085</v>
       </c>
       <c r="F14">
-        <v>63.72</v>
+        <v>59.609614678899085</v>
       </c>
       <c r="G14">
         <v>74.52</v>
@@ -1560,31 +1566,31 @@
         <v>9.36</v>
       </c>
       <c r="R14">
-        <f>AA14</f>
-        <v>81.123704697986582</v>
+        <f t="shared" si="0"/>
+        <v>63.442348623853213</v>
       </c>
       <c r="S14" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="T14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="W14">
         <v>0</v>
       </c>
       <c r="X14">
-        <v>5052</v>
+        <v>6346</v>
       </c>
       <c r="Y14">
-        <v>8130.4084033532126</v>
+        <v>10212.900183626185</v>
       </c>
       <c r="Z14">
-        <f t="shared" si="0"/>
-        <v>7.323704697986579</v>
+        <f t="shared" si="1"/>
+        <v>9.0823486238532123</v>
       </c>
       <c r="AA14">
-        <f t="shared" si="1"/>
-        <v>81.123704697986582</v>
+        <f t="shared" si="2"/>
+        <v>63.442348623853213</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.35">
@@ -1601,10 +1607,10 @@
         <v>70</v>
       </c>
       <c r="E15">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="F15">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="G15">
         <v>74.52</v>
@@ -1640,31 +1646,31 @@
         <v>9.36</v>
       </c>
       <c r="R15">
-        <f>AA15</f>
-        <v>81.690523489932886</v>
+        <f t="shared" si="0"/>
+        <v>64.406972477064215</v>
       </c>
       <c r="S15" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="T15" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="W15">
         <v>0</v>
       </c>
       <c r="X15">
-        <v>5443</v>
+        <v>7020</v>
       </c>
       <c r="Y15">
-        <v>8759.6621020292041</v>
+        <v>11297.598375205771</v>
       </c>
       <c r="Z15">
-        <f t="shared" si="0"/>
-        <v>7.8905234899328871</v>
+        <f t="shared" si="1"/>
+        <v>10.046972477064221</v>
       </c>
       <c r="AA15">
-        <f t="shared" si="1"/>
-        <v>81.690523489932886</v>
+        <f t="shared" si="2"/>
+        <v>64.406972477064215</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.35">
@@ -1681,10 +1687,10 @@
         <v>70</v>
       </c>
       <c r="E16">
-        <v>63.72</v>
+        <v>63.05878899082569</v>
       </c>
       <c r="F16">
-        <v>63.72</v>
+        <v>63.05878899082569</v>
       </c>
       <c r="G16">
         <v>74.52</v>
@@ -1720,31 +1726,31 @@
         <v>9.36</v>
       </c>
       <c r="R16">
-        <f>AA16</f>
-        <v>80.417718120805375</v>
+        <f t="shared" si="0"/>
+        <v>61.896660550458719</v>
       </c>
       <c r="S16" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="T16" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="W16">
         <v>0</v>
       </c>
       <c r="X16">
-        <v>4565</v>
+        <v>5266</v>
       </c>
       <c r="Y16">
-        <v>7346.6576328795363</v>
+        <v>8474.8081259022201</v>
       </c>
       <c r="Z16">
-        <f t="shared" si="0"/>
-        <v>6.617718120805371</v>
+        <f t="shared" si="1"/>
+        <v>7.5366605504587163</v>
       </c>
       <c r="AA16">
-        <f t="shared" si="1"/>
-        <v>80.417718120805375</v>
+        <f t="shared" si="2"/>
+        <v>61.896660550458719</v>
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.35">
@@ -1761,10 +1767,10 @@
         <v>70</v>
       </c>
       <c r="E17">
-        <v>63.72</v>
+        <v>60.62862385321101</v>
       </c>
       <c r="F17">
-        <v>63.72</v>
+        <v>60.62862385321101</v>
       </c>
       <c r="G17">
         <v>74.52</v>
@@ -1800,31 +1806,31 @@
         <v>9.36</v>
       </c>
       <c r="R17">
-        <f>AA17</f>
-        <v>80.609073825503359</v>
+        <f t="shared" si="0"/>
+        <v>61.025064220183488</v>
       </c>
       <c r="S17" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="T17" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="W17">
         <v>0</v>
       </c>
       <c r="X17">
-        <v>4697</v>
+        <v>4657</v>
       </c>
       <c r="Y17">
-        <v>7559.0911066013541</v>
+        <v>7494.7173266856516</v>
       </c>
       <c r="Z17">
-        <f t="shared" si="0"/>
-        <v>6.8090738255033578</v>
+        <f t="shared" si="1"/>
+        <v>6.6650642201834858</v>
       </c>
       <c r="AA17">
-        <f t="shared" si="1"/>
-        <v>80.609073825503359</v>
+        <f t="shared" si="2"/>
+        <v>61.025064220183488</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.35">
@@ -1841,10 +1847,10 @@
         <v>70</v>
       </c>
       <c r="E18">
-        <v>63.72</v>
+        <v>64.897871559633032</v>
       </c>
       <c r="F18">
-        <v>63.72</v>
+        <v>64.897871559633032</v>
       </c>
       <c r="G18">
         <v>74.52</v>
@@ -1880,31 +1886,31 @@
         <v>9.36</v>
       </c>
       <c r="R18">
-        <f>AA18</f>
-        <v>83.090899328859052</v>
+        <f t="shared" si="0"/>
+        <v>59.608183486238531</v>
       </c>
       <c r="S18" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="T18" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="W18">
         <v>0</v>
       </c>
       <c r="X18">
-        <v>6409</v>
+        <v>3667</v>
       </c>
       <c r="Y18">
-        <v>10314.288886993416</v>
+        <v>5901.4662737720173</v>
       </c>
       <c r="Z18">
-        <f t="shared" si="0"/>
-        <v>9.2908993288590622</v>
+        <f t="shared" si="1"/>
+        <v>5.248183486238533</v>
       </c>
       <c r="AA18">
-        <f t="shared" si="1"/>
-        <v>83.090899328859052</v>
+        <f t="shared" si="2"/>
+        <v>59.608183486238531</v>
       </c>
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.35">
@@ -1921,10 +1927,10 @@
         <v>70</v>
       </c>
       <c r="E19">
-        <v>63.72</v>
+        <v>64.680330275229352</v>
       </c>
       <c r="F19">
-        <v>63.72</v>
+        <v>64.680330275229352</v>
       </c>
       <c r="G19">
         <v>74.52</v>
@@ -1960,31 +1966,31 @@
         <v>9.36</v>
       </c>
       <c r="R19">
-        <f>AA19</f>
-        <v>80.564134228187925</v>
+        <f t="shared" si="0"/>
+        <v>63.077394495412847</v>
       </c>
       <c r="S19" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="T19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="W19">
         <v>0</v>
       </c>
       <c r="X19">
-        <v>4666</v>
+        <v>6091</v>
       </c>
       <c r="Y19">
-        <v>7509.2014271666849</v>
+        <v>9802.5173366635827</v>
       </c>
       <c r="Z19">
-        <f t="shared" si="0"/>
-        <v>6.7641342281879213</v>
+        <f t="shared" si="1"/>
+        <v>8.7173944954128455</v>
       </c>
       <c r="AA19">
-        <f t="shared" si="1"/>
-        <v>80.564134228187925</v>
+        <f t="shared" si="2"/>
+        <v>63.077394495412847</v>
       </c>
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.35">
@@ -2001,10 +2007,10 @@
         <v>70</v>
       </c>
       <c r="E20">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="F20">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="G20">
         <v>74.52</v>
@@ -2040,31 +2046,31 @@
         <v>9.36</v>
       </c>
       <c r="R20">
-        <f>AA20</f>
-        <v>82.274738255033554</v>
+        <f t="shared" si="0"/>
+        <v>64.983743119266052</v>
       </c>
       <c r="S20" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="T20" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="W20">
         <v>0</v>
       </c>
       <c r="X20">
-        <v>5846</v>
+        <v>7423</v>
       </c>
       <c r="Y20">
-        <v>9408.227934679906</v>
+        <v>11946.164207856473</v>
       </c>
       <c r="Z20">
-        <f t="shared" si="0"/>
-        <v>8.4747382550335608</v>
+        <f t="shared" si="1"/>
+        <v>10.623743119266056</v>
       </c>
       <c r="AA20">
-        <f t="shared" si="1"/>
-        <v>82.274738255033554</v>
+        <f t="shared" si="2"/>
+        <v>64.983743119266052</v>
       </c>
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.35">
@@ -2081,10 +2087,10 @@
         <v>70</v>
       </c>
       <c r="E21">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="F21">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="G21">
         <v>74.52</v>
@@ -2120,31 +2126,31 @@
         <v>9.36</v>
       </c>
       <c r="R21">
-        <f>AA21</f>
-        <v>82.274738255033554</v>
+        <f t="shared" si="0"/>
+        <v>64.983743119266052</v>
       </c>
       <c r="S21" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="T21" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="W21">
         <v>0</v>
       </c>
       <c r="X21">
-        <v>5846</v>
+        <v>7423</v>
       </c>
       <c r="Y21">
-        <v>9408.227934679906</v>
+        <v>11946.164207856473</v>
       </c>
       <c r="Z21">
-        <f t="shared" si="0"/>
-        <v>8.4747382550335608</v>
+        <f t="shared" si="1"/>
+        <v>10.623743119266056</v>
       </c>
       <c r="AA21">
-        <f t="shared" si="1"/>
-        <v>82.274738255033554</v>
+        <f t="shared" si="2"/>
+        <v>64.983743119266052</v>
       </c>
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.35">
@@ -2161,70 +2167,70 @@
         <v>70</v>
       </c>
       <c r="E22">
+        <v>63.442348623853213</v>
+      </c>
+      <c r="F22">
+        <v>63.442348623853213</v>
+      </c>
+      <c r="G22">
+        <v>74.52</v>
+      </c>
+      <c r="H22">
+        <v>90</v>
+      </c>
+      <c r="I22">
+        <v>37.799999999999997</v>
+      </c>
+      <c r="J22">
+        <v>37.799999999999997</v>
+      </c>
+      <c r="K22">
+        <v>72.72</v>
+      </c>
+      <c r="L22">
+        <v>72.72</v>
+      </c>
+      <c r="M22">
+        <v>72.72</v>
+      </c>
+      <c r="N22">
+        <v>72.72</v>
+      </c>
+      <c r="O22">
+        <v>72.72</v>
+      </c>
+      <c r="P22">
+        <v>70.56</v>
+      </c>
+      <c r="Q22">
+        <v>9.36</v>
+      </c>
+      <c r="R22">
+        <f t="shared" si="0"/>
         <v>63.72</v>
       </c>
-      <c r="F22">
-        <v>63.72</v>
-      </c>
-      <c r="G22">
-        <v>74.52</v>
-      </c>
-      <c r="H22">
-        <v>90</v>
-      </c>
-      <c r="I22">
-        <v>37.799999999999997</v>
-      </c>
-      <c r="J22">
-        <v>37.799999999999997</v>
-      </c>
-      <c r="K22">
-        <v>72.72</v>
-      </c>
-      <c r="L22">
-        <v>72.72</v>
-      </c>
-      <c r="M22">
-        <v>72.72</v>
-      </c>
-      <c r="N22">
-        <v>72.72</v>
-      </c>
-      <c r="O22">
-        <v>72.72</v>
-      </c>
-      <c r="P22">
-        <v>70.56</v>
-      </c>
-      <c r="Q22">
-        <v>9.36</v>
-      </c>
-      <c r="R22">
-        <f>AA22</f>
-        <v>81.36</v>
-      </c>
       <c r="S22" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="T22" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="W22">
         <v>0</v>
       </c>
       <c r="X22">
-        <v>5215</v>
+        <v>6540</v>
       </c>
       <c r="Y22">
-        <v>8392.7315565096997</v>
+        <v>10525.113016217341</v>
       </c>
       <c r="Z22">
-        <f t="shared" si="0"/>
-        <v>7.56</v>
+        <f t="shared" si="1"/>
+        <v>9.36</v>
       </c>
       <c r="AA22">
-        <f t="shared" si="1"/>
-        <v>81.36</v>
+        <f t="shared" si="2"/>
+        <v>63.72</v>
       </c>
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.35">
@@ -2241,10 +2247,10 @@
         <v>70</v>
       </c>
       <c r="E23">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="F23">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="G23">
         <v>74.52</v>
@@ -2280,31 +2286,31 @@
         <v>9.36</v>
       </c>
       <c r="R23">
-        <f>AA23</f>
-        <v>80.416268456375832</v>
+        <f t="shared" si="0"/>
+        <v>63.05878899082569</v>
       </c>
       <c r="S23" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="T23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="W23">
         <v>0</v>
       </c>
       <c r="X23">
-        <v>4564</v>
+        <v>6078</v>
       </c>
       <c r="Y23">
-        <v>7345.0482883816439</v>
+        <v>9781.5958581909799</v>
       </c>
       <c r="Z23">
-        <f t="shared" si="0"/>
-        <v>6.61626845637584</v>
+        <f t="shared" si="1"/>
+        <v>8.6987889908256903</v>
       </c>
       <c r="AA23">
-        <f t="shared" si="1"/>
-        <v>80.416268456375832</v>
+        <f t="shared" si="2"/>
+        <v>63.05878899082569</v>
       </c>
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.35">
@@ -2321,10 +2327,10 @@
         <v>70</v>
       </c>
       <c r="E24">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="F24">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="G24">
         <v>74.52</v>
@@ -2360,31 +2366,31 @@
         <v>9.36</v>
       </c>
       <c r="R24">
-        <f>AA24</f>
-        <v>82.187758389261745</v>
+        <f t="shared" si="0"/>
+        <v>64.897871559633032</v>
       </c>
       <c r="S24" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="T24" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="W24">
         <v>0</v>
       </c>
       <c r="X24">
-        <v>5786</v>
+        <v>7363</v>
       </c>
       <c r="Y24">
-        <v>9311.6672648063523</v>
+        <v>11849.603537982919</v>
       </c>
       <c r="Z24">
-        <f t="shared" si="0"/>
-        <v>8.3877583892617462</v>
+        <f t="shared" si="1"/>
+        <v>10.537871559633027</v>
       </c>
       <c r="AA24">
-        <f t="shared" si="1"/>
-        <v>82.187758389261745</v>
+        <f t="shared" si="2"/>
+        <v>64.897871559633032</v>
       </c>
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.35">
@@ -2401,10 +2407,10 @@
         <v>70</v>
       </c>
       <c r="E25">
-        <v>63.72</v>
+        <v>64.406972477064215</v>
       </c>
       <c r="F25">
-        <v>63.72</v>
+        <v>64.406972477064215</v>
       </c>
       <c r="G25">
         <v>74.52</v>
@@ -2441,7 +2447,7 @@
       </c>
       <c r="R25">
         <f>AVERAGE(R8:R24)</f>
-        <v>81.639529411764684</v>
+        <v>62.637176470588244</v>
       </c>
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.35">
@@ -2458,10 +2464,10 @@
         <v>70</v>
       </c>
       <c r="E26">
-        <v>63.72</v>
+        <v>61.896660550458719</v>
       </c>
       <c r="F26">
-        <v>63.72</v>
+        <v>61.896660550458719</v>
       </c>
       <c r="G26">
         <v>74.52</v>
@@ -2511,10 +2517,10 @@
         <v>70</v>
       </c>
       <c r="E27">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="F27">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="G27">
         <v>74.52</v>
@@ -2564,10 +2570,10 @@
         <v>70</v>
       </c>
       <c r="E28">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="F28">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="G28">
         <v>74.52</v>
@@ -2617,10 +2623,10 @@
         <v>70</v>
       </c>
       <c r="E29">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="F29">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="G29">
         <v>74.52</v>
@@ -2670,10 +2676,10 @@
         <v>70</v>
       </c>
       <c r="E30">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="F30">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="G30">
         <v>74.52</v>
@@ -2723,10 +2729,10 @@
         <v>70</v>
       </c>
       <c r="E31">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="F31">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="G31">
         <v>74.52</v>
@@ -2776,10 +2782,10 @@
         <v>70</v>
       </c>
       <c r="E32">
-        <v>63.72</v>
+        <v>61.025064220183488</v>
       </c>
       <c r="F32">
-        <v>63.72</v>
+        <v>61.025064220183488</v>
       </c>
       <c r="G32">
         <v>74.52</v>
@@ -2829,10 +2835,10 @@
         <v>70</v>
       </c>
       <c r="E33">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="F33">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="G33">
         <v>74.52</v>
@@ -2882,10 +2888,10 @@
         <v>70</v>
       </c>
       <c r="E34">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="F34">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="G34">
         <v>74.52</v>
@@ -2935,10 +2941,10 @@
         <v>70</v>
       </c>
       <c r="E35">
-        <v>63.72</v>
+        <v>59.608183486238531</v>
       </c>
       <c r="F35">
-        <v>63.72</v>
+        <v>59.608183486238531</v>
       </c>
       <c r="G35">
         <v>74.52</v>
@@ -2988,10 +2994,10 @@
         <v>70</v>
       </c>
       <c r="E36">
-        <v>63.72</v>
+        <v>63.077394495412847</v>
       </c>
       <c r="F36">
-        <v>63.72</v>
+        <v>63.077394495412847</v>
       </c>
       <c r="G36">
         <v>74.52</v>
@@ -3041,10 +3047,10 @@
         <v>70</v>
       </c>
       <c r="E37">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="F37">
-        <v>63.72</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="G37">
         <v>74.52</v>

</xml_diff>

<commit_message>
update LNG import emissions from ME
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
+++ b/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0E8D1F3-74C5-4280-A375-F2494D6D72C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{098E60FB-05B5-4CD2-B5DF-51A63E6759A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BAA9D55F-0FEB-4558-AFDF-92239B956412}"/>
   </bookViews>
@@ -249,7 +249,7 @@
     <t>LV_LNG</t>
   </si>
   <si>
-    <t>QA_LNG</t>
+    <t>ME_LNG</t>
   </si>
 </sst>
 </file>
@@ -701,7 +701,7 @@
         <v>70</v>
       </c>
       <c r="E2">
-        <v>62.637176470588244</v>
+        <v>62.773291046064649</v>
       </c>
       <c r="F2">
         <v>62.637176470588244</v>
@@ -766,7 +766,7 @@
         <v>70</v>
       </c>
       <c r="E3">
-        <v>62.637176470588244</v>
+        <v>62.773291046064649</v>
       </c>
       <c r="F3">
         <v>62.637176470588244</v>
@@ -819,7 +819,7 @@
         <v>70</v>
       </c>
       <c r="E4">
-        <v>63.343596330275233</v>
+        <v>63.33970029352696</v>
       </c>
       <c r="F4">
         <v>63.343596330275233</v>
@@ -878,7 +878,7 @@
         <v>70</v>
       </c>
       <c r="E5">
-        <v>62.637176470588244</v>
+        <v>62.773291046064649</v>
       </c>
       <c r="F5">
         <v>62.637176470588244</v>
@@ -937,10 +937,10 @@
         <v>70</v>
       </c>
       <c r="E6">
-        <v>61.615981651376146</v>
+        <v>62.773291046064649</v>
       </c>
       <c r="F6">
-        <v>61.615981651376146</v>
+        <v>62.637176470588244</v>
       </c>
       <c r="G6">
         <v>74.52</v>
@@ -994,7 +994,7 @@
         <v>70</v>
       </c>
       <c r="E7">
-        <v>60.552770642201835</v>
+        <v>60.519987640970186</v>
       </c>
       <c r="F7">
         <v>60.552770642201835</v>
@@ -1047,7 +1047,7 @@
         <v>70</v>
       </c>
       <c r="E8">
-        <v>62.637176470588244</v>
+        <v>62.773291046064649</v>
       </c>
       <c r="F8">
         <v>62.637176470588244</v>
@@ -1087,7 +1087,7 @@
       </c>
       <c r="R8">
         <f t="shared" ref="R8:R24" si="0">AA8</f>
-        <v>63.343596330275233</v>
+        <v>63.33970029352696</v>
       </c>
       <c r="S8" t="s">
         <v>70</v>
@@ -1099,18 +1099,18 @@
         <v>0</v>
       </c>
       <c r="X8">
-        <v>6277</v>
+        <v>6210</v>
       </c>
       <c r="Y8">
-        <v>10101.855413271598</v>
+        <v>9994.0293319127977</v>
       </c>
       <c r="Z8">
         <f>((($U$4/$Y$22)*Y8)*$T$1)/$U$1</f>
-        <v>8.9835963302752297</v>
+        <v>8.9797002935269568</v>
       </c>
       <c r="AA8">
         <f>Z8+$U$2</f>
-        <v>63.343596330275233</v>
+        <v>63.33970029352696</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.35">
@@ -1127,7 +1127,7 @@
         <v>70</v>
       </c>
       <c r="E9">
-        <v>62.637176470588244</v>
+        <v>62.773291046064649</v>
       </c>
       <c r="F9">
         <v>62.637176470588244</v>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="R9">
         <f t="shared" si="0"/>
-        <v>60.916293577981648</v>
+        <v>63.291982079406765</v>
       </c>
       <c r="S9" t="s">
         <v>70</v>
@@ -1179,18 +1179,18 @@
         <v>0</v>
       </c>
       <c r="X9">
-        <v>4581</v>
+        <v>6177</v>
       </c>
       <c r="Y9">
-        <v>7372.4071448458171</v>
+        <v>9940.9209634823437</v>
       </c>
       <c r="Z9">
         <f t="shared" ref="Z9:Z24" si="1">((($U$4/$Y$22)*Y9)*$T$1)/$U$1</f>
-        <v>6.556293577981652</v>
+        <v>8.9319820794067688</v>
       </c>
       <c r="AA9">
         <f t="shared" ref="AA9:AA24" si="2">Z9+$U$2</f>
-        <v>60.916293577981648</v>
+        <v>63.291982079406765</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.35">
@@ -1207,7 +1207,7 @@
         <v>70</v>
       </c>
       <c r="E10">
-        <v>64.983743119266052</v>
+        <v>64.996823729337251</v>
       </c>
       <c r="F10">
         <v>64.983743119266052</v>
@@ -1247,7 +1247,7 @@
       </c>
       <c r="R10">
         <f t="shared" si="0"/>
-        <v>59.609614678899085</v>
+        <v>59.567069365054842</v>
       </c>
       <c r="S10" t="s">
         <v>70</v>
@@ -1259,18 +1259,18 @@
         <v>0</v>
       </c>
       <c r="X10">
-        <v>3668</v>
+        <v>3601</v>
       </c>
       <c r="Y10">
-        <v>5903.0756182699097</v>
+        <v>5795.2495369111084</v>
       </c>
       <c r="Z10">
         <f t="shared" si="1"/>
-        <v>5.249614678899083</v>
+        <v>5.207069365054843</v>
       </c>
       <c r="AA10">
         <f t="shared" si="2"/>
-        <v>59.609614678899085</v>
+        <v>59.567069365054842</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.35">
@@ -1287,7 +1287,7 @@
         <v>70</v>
       </c>
       <c r="E11">
-        <v>64.983743119266052</v>
+        <v>64.996823729337251</v>
       </c>
       <c r="F11">
         <v>64.983743119266052</v>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="R11">
         <f t="shared" si="0"/>
-        <v>60.62862385321101</v>
+        <v>60.700738452031516</v>
       </c>
       <c r="S11" t="s">
         <v>70</v>
@@ -1339,18 +1339,18 @@
         <v>0</v>
       </c>
       <c r="X11">
-        <v>4380</v>
+        <v>4385</v>
       </c>
       <c r="Y11">
-        <v>7048.9289007694124</v>
+        <v>7056.9756232588752</v>
       </c>
       <c r="Z11">
         <f t="shared" si="1"/>
-        <v>6.2686238532110092</v>
+        <v>6.3407384520315153</v>
       </c>
       <c r="AA11">
         <f t="shared" si="2"/>
-        <v>60.62862385321101</v>
+        <v>60.700738452031516</v>
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.35">
@@ -1367,7 +1367,7 @@
         <v>70</v>
       </c>
       <c r="E12">
-        <v>60.916293577981648</v>
+        <v>63.291982079406765</v>
       </c>
       <c r="F12">
         <v>60.916293577981648</v>
@@ -1407,7 +1407,7 @@
       </c>
       <c r="R12">
         <f t="shared" si="0"/>
-        <v>60.552770642201835</v>
+        <v>60.519987640970186</v>
       </c>
       <c r="S12" t="s">
         <v>70</v>
@@ -1419,18 +1419,18 @@
         <v>0</v>
       </c>
       <c r="X12">
-        <v>4327</v>
+        <v>4260</v>
       </c>
       <c r="Y12">
-        <v>6963.6336423811072</v>
+        <v>6855.807561022305</v>
       </c>
       <c r="Z12">
         <f t="shared" si="1"/>
-        <v>6.192770642201836</v>
+        <v>6.1599876409701837</v>
       </c>
       <c r="AA12">
         <f t="shared" si="2"/>
-        <v>60.552770642201835</v>
+        <v>60.519987640970186</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.35">
@@ -1487,7 +1487,7 @@
       </c>
       <c r="R13">
         <f t="shared" si="0"/>
-        <v>64.680330275229352</v>
+        <v>64.690270353777223</v>
       </c>
       <c r="S13" t="s">
         <v>70</v>
@@ -1499,18 +1499,18 @@
         <v>0</v>
       </c>
       <c r="X13">
-        <v>7211</v>
+        <v>7144</v>
       </c>
       <c r="Y13">
-        <v>11604.98317430325</v>
+        <v>11497.157092944448</v>
       </c>
       <c r="Z13">
         <f t="shared" si="1"/>
-        <v>10.32033027522936</v>
+        <v>10.330270353777228</v>
       </c>
       <c r="AA13">
         <f t="shared" si="2"/>
-        <v>64.680330275229352</v>
+        <v>64.690270353777223</v>
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.35">
@@ -1527,7 +1527,7 @@
         <v>70</v>
       </c>
       <c r="E14">
-        <v>59.609614678899085</v>
+        <v>59.567069365054842</v>
       </c>
       <c r="F14">
         <v>59.609614678899085</v>
@@ -1567,7 +1567,7 @@
       </c>
       <c r="R14">
         <f t="shared" si="0"/>
-        <v>63.442348623853213</v>
+        <v>63.435136721767336</v>
       </c>
       <c r="S14" t="s">
         <v>70</v>
@@ -1579,18 +1579,18 @@
         <v>0</v>
       </c>
       <c r="X14">
-        <v>6346</v>
+        <v>6276</v>
       </c>
       <c r="Y14">
-        <v>10212.900183626185</v>
+        <v>10100.246068773706</v>
       </c>
       <c r="Z14">
         <f t="shared" si="1"/>
-        <v>9.0823486238532123</v>
+        <v>9.0751367217673398</v>
       </c>
       <c r="AA14">
         <f t="shared" si="2"/>
-        <v>63.442348623853213</v>
+        <v>63.435136721767336</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.35">
@@ -1607,7 +1607,7 @@
         <v>70</v>
       </c>
       <c r="E15">
-        <v>62.637176470588244</v>
+        <v>62.773291046064649</v>
       </c>
       <c r="F15">
         <v>62.637176470588244</v>
@@ -1647,7 +1647,7 @@
       </c>
       <c r="R15">
         <f t="shared" si="0"/>
-        <v>64.406972477064215</v>
+        <v>64.414083114475517</v>
       </c>
       <c r="S15" t="s">
         <v>70</v>
@@ -1659,18 +1659,18 @@
         <v>0</v>
       </c>
       <c r="X15">
-        <v>7020</v>
+        <v>6953</v>
       </c>
       <c r="Y15">
-        <v>11297.598375205771</v>
+        <v>11189.772293846969</v>
       </c>
       <c r="Z15">
         <f t="shared" si="1"/>
-        <v>10.046972477064221</v>
+        <v>10.054083114475512</v>
       </c>
       <c r="AA15">
         <f t="shared" si="2"/>
-        <v>64.406972477064215</v>
+        <v>64.414083114475517</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.35">
@@ -1687,7 +1687,7 @@
         <v>70</v>
       </c>
       <c r="E16">
-        <v>63.05878899082569</v>
+        <v>63.051945002317318</v>
       </c>
       <c r="F16">
         <v>63.05878899082569</v>
@@ -1727,7 +1727,7 @@
       </c>
       <c r="R16">
         <f t="shared" si="0"/>
-        <v>61.896660550458719</v>
+        <v>61.877787733662906</v>
       </c>
       <c r="S16" t="s">
         <v>70</v>
@@ -1739,18 +1739,18 @@
         <v>0</v>
       </c>
       <c r="X16">
-        <v>5266</v>
+        <v>5199</v>
       </c>
       <c r="Y16">
-        <v>8474.8081259022201</v>
+        <v>8366.9820445434198</v>
       </c>
       <c r="Z16">
         <f t="shared" si="1"/>
-        <v>7.5366605504587163</v>
+        <v>7.5177877336629066</v>
       </c>
       <c r="AA16">
         <f t="shared" si="2"/>
-        <v>61.896660550458719</v>
+        <v>61.877787733662906</v>
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.35">
@@ -1767,7 +1767,7 @@
         <v>70</v>
       </c>
       <c r="E17">
-        <v>60.62862385321101</v>
+        <v>60.700738452031516</v>
       </c>
       <c r="F17">
         <v>60.62862385321101</v>
@@ -1807,7 +1807,7 @@
       </c>
       <c r="R17">
         <f t="shared" si="0"/>
-        <v>61.025064220183488</v>
+        <v>60.997169782172101</v>
       </c>
       <c r="S17" t="s">
         <v>70</v>
@@ -1819,18 +1819,18 @@
         <v>0</v>
       </c>
       <c r="X17">
-        <v>4657</v>
+        <v>4590</v>
       </c>
       <c r="Y17">
-        <v>7494.7173266856516</v>
+        <v>7386.8912453268504</v>
       </c>
       <c r="Z17">
         <f t="shared" si="1"/>
-        <v>6.6650642201834858</v>
+        <v>6.6371697821720996</v>
       </c>
       <c r="AA17">
         <f t="shared" si="2"/>
-        <v>61.025064220183488</v>
+        <v>60.997169782172101</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.35">
@@ -1847,7 +1847,7 @@
         <v>70</v>
       </c>
       <c r="E18">
-        <v>64.897871559633032</v>
+        <v>64.910063340027804</v>
       </c>
       <c r="F18">
         <v>64.897871559633032</v>
@@ -1887,7 +1887,7 @@
       </c>
       <c r="R18">
         <f t="shared" si="0"/>
-        <v>59.608183486238531</v>
+        <v>59.565623358566349</v>
       </c>
       <c r="S18" t="s">
         <v>70</v>
@@ -1899,18 +1899,18 @@
         <v>0</v>
       </c>
       <c r="X18">
-        <v>3667</v>
+        <v>3600</v>
       </c>
       <c r="Y18">
-        <v>5901.4662737720173</v>
+        <v>5793.640192413216</v>
       </c>
       <c r="Z18">
         <f t="shared" si="1"/>
-        <v>5.248183486238533</v>
+        <v>5.2056233585663518</v>
       </c>
       <c r="AA18">
         <f t="shared" si="2"/>
-        <v>59.608183486238531</v>
+        <v>59.565623358566349</v>
       </c>
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.35">
@@ -1927,7 +1927,7 @@
         <v>70</v>
       </c>
       <c r="E19">
-        <v>64.680330275229352</v>
+        <v>64.690270353777223</v>
       </c>
       <c r="F19">
         <v>64.680330275229352</v>
@@ -1967,7 +1967,7 @@
       </c>
       <c r="R19">
         <f t="shared" si="0"/>
-        <v>63.077394495412847</v>
+        <v>63.070743086667697</v>
       </c>
       <c r="S19" t="s">
         <v>70</v>
@@ -1979,18 +1979,18 @@
         <v>0</v>
       </c>
       <c r="X19">
-        <v>6091</v>
+        <v>6024</v>
       </c>
       <c r="Y19">
-        <v>9802.5173366635827</v>
+        <v>9694.6912553047805</v>
       </c>
       <c r="Z19">
         <f t="shared" si="1"/>
-        <v>8.7173944954128455</v>
+        <v>8.710743086667696</v>
       </c>
       <c r="AA19">
         <f t="shared" si="2"/>
-        <v>63.077394495412847</v>
+        <v>63.070743086667697</v>
       </c>
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.35">
@@ -2007,7 +2007,7 @@
         <v>70</v>
       </c>
       <c r="E20">
-        <v>62.637176470588244</v>
+        <v>62.773291046064649</v>
       </c>
       <c r="F20">
         <v>62.637176470588244</v>
@@ -2047,7 +2047,7 @@
       </c>
       <c r="R20">
         <f t="shared" si="0"/>
-        <v>64.983743119266052</v>
+        <v>64.996823729337251</v>
       </c>
       <c r="S20" t="s">
         <v>70</v>
@@ -2059,18 +2059,18 @@
         <v>0</v>
       </c>
       <c r="X20">
-        <v>7423</v>
+        <v>7356</v>
       </c>
       <c r="Y20">
-        <v>11946.164207856473</v>
+        <v>11838.338126497671</v>
       </c>
       <c r="Z20">
         <f t="shared" si="1"/>
-        <v>10.623743119266056</v>
+        <v>10.636823729337245</v>
       </c>
       <c r="AA20">
         <f t="shared" si="2"/>
-        <v>64.983743119266052</v>
+        <v>64.996823729337251</v>
       </c>
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.35">
@@ -2087,7 +2087,7 @@
         <v>70</v>
       </c>
       <c r="E21">
-        <v>62.637176470588244</v>
+        <v>62.773291046064649</v>
       </c>
       <c r="F21">
         <v>62.637176470588244</v>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="R21">
         <f t="shared" si="0"/>
-        <v>64.983743119266052</v>
+        <v>64.996823729337251</v>
       </c>
       <c r="S21" t="s">
         <v>70</v>
@@ -2139,18 +2139,18 @@
         <v>0</v>
       </c>
       <c r="X21">
-        <v>7423</v>
+        <v>7356</v>
       </c>
       <c r="Y21">
-        <v>11946.164207856473</v>
+        <v>11838.338126497671</v>
       </c>
       <c r="Z21">
         <f t="shared" si="1"/>
-        <v>10.623743119266056</v>
+        <v>10.636823729337245</v>
       </c>
       <c r="AA21">
         <f t="shared" si="2"/>
-        <v>64.983743119266052</v>
+        <v>64.996823729337251</v>
       </c>
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.35">
@@ -2167,7 +2167,7 @@
         <v>70</v>
       </c>
       <c r="E22">
-        <v>63.442348623853213</v>
+        <v>63.435136721767336</v>
       </c>
       <c r="F22">
         <v>63.442348623853213</v>
@@ -2219,10 +2219,10 @@
         <v>0</v>
       </c>
       <c r="X22">
-        <v>6540</v>
+        <v>6473</v>
       </c>
       <c r="Y22">
-        <v>10525.113016217341</v>
+        <v>10417.286934858541</v>
       </c>
       <c r="Z22">
         <f t="shared" si="1"/>
@@ -2247,7 +2247,7 @@
         <v>70</v>
       </c>
       <c r="E23">
-        <v>62.637176470588244</v>
+        <v>62.773291046064649</v>
       </c>
       <c r="F23">
         <v>62.637176470588244</v>
@@ -2287,7 +2287,7 @@
       </c>
       <c r="R23">
         <f t="shared" si="0"/>
-        <v>63.05878899082569</v>
+        <v>63.051945002317318</v>
       </c>
       <c r="S23" t="s">
         <v>70</v>
@@ -2299,18 +2299,18 @@
         <v>0</v>
       </c>
       <c r="X23">
-        <v>6078</v>
+        <v>6011</v>
       </c>
       <c r="Y23">
-        <v>9781.5958581909799</v>
+        <v>9673.7697768321777</v>
       </c>
       <c r="Z23">
         <f t="shared" si="1"/>
-        <v>8.6987889908256903</v>
+        <v>8.6919450023173184</v>
       </c>
       <c r="AA23">
         <f t="shared" si="2"/>
-        <v>63.05878899082569</v>
+        <v>63.051945002317318</v>
       </c>
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.35">
@@ -2327,7 +2327,7 @@
         <v>70</v>
       </c>
       <c r="E24">
-        <v>62.637176470588244</v>
+        <v>62.773291046064649</v>
       </c>
       <c r="F24">
         <v>62.637176470588244</v>
@@ -2367,7 +2367,7 @@
       </c>
       <c r="R24">
         <f t="shared" si="0"/>
-        <v>64.897871559633032</v>
+        <v>64.910063340027804</v>
       </c>
       <c r="S24" t="s">
         <v>70</v>
@@ -2379,18 +2379,18 @@
         <v>0</v>
       </c>
       <c r="X24">
-        <v>7363</v>
+        <v>7296</v>
       </c>
       <c r="Y24">
-        <v>11849.603537982919</v>
+        <v>11741.777456624117</v>
       </c>
       <c r="Z24">
         <f t="shared" si="1"/>
-        <v>10.537871559633027</v>
+        <v>10.550063340027807</v>
       </c>
       <c r="AA24">
         <f t="shared" si="2"/>
-        <v>64.897871559633032</v>
+        <v>64.910063340027804</v>
       </c>
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.35">
@@ -2407,7 +2407,7 @@
         <v>70</v>
       </c>
       <c r="E25">
-        <v>64.406972477064215</v>
+        <v>64.414083114475517</v>
       </c>
       <c r="F25">
         <v>64.406972477064215</v>
@@ -2447,7 +2447,7 @@
       </c>
       <c r="R25">
         <f>AVERAGE(R8:R24)</f>
-        <v>62.637176470588244</v>
+        <v>62.773291046064649</v>
       </c>
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.35">
@@ -2464,7 +2464,7 @@
         <v>70</v>
       </c>
       <c r="E26">
-        <v>61.896660550458719</v>
+        <v>61.877787733662906</v>
       </c>
       <c r="F26">
         <v>61.896660550458719</v>
@@ -2517,7 +2517,7 @@
         <v>70</v>
       </c>
       <c r="E27">
-        <v>62.637176470588244</v>
+        <v>62.773291046064649</v>
       </c>
       <c r="F27">
         <v>62.637176470588244</v>
@@ -2570,7 +2570,7 @@
         <v>70</v>
       </c>
       <c r="E28">
-        <v>62.637176470588244</v>
+        <v>62.773291046064649</v>
       </c>
       <c r="F28">
         <v>62.637176470588244</v>
@@ -2623,7 +2623,7 @@
         <v>70</v>
       </c>
       <c r="E29">
-        <v>62.637176470588244</v>
+        <v>62.773291046064649</v>
       </c>
       <c r="F29">
         <v>62.637176470588244</v>
@@ -2676,7 +2676,7 @@
         <v>70</v>
       </c>
       <c r="E30">
-        <v>62.637176470588244</v>
+        <v>62.773291046064649</v>
       </c>
       <c r="F30">
         <v>62.637176470588244</v>
@@ -2729,7 +2729,7 @@
         <v>70</v>
       </c>
       <c r="E31">
-        <v>62.637176470588244</v>
+        <v>62.773291046064649</v>
       </c>
       <c r="F31">
         <v>62.637176470588244</v>
@@ -2782,7 +2782,7 @@
         <v>70</v>
       </c>
       <c r="E32">
-        <v>61.025064220183488</v>
+        <v>60.997169782172101</v>
       </c>
       <c r="F32">
         <v>61.025064220183488</v>
@@ -2835,7 +2835,7 @@
         <v>70</v>
       </c>
       <c r="E33">
-        <v>62.637176470588244</v>
+        <v>62.773291046064649</v>
       </c>
       <c r="F33">
         <v>62.637176470588244</v>
@@ -2888,7 +2888,7 @@
         <v>70</v>
       </c>
       <c r="E34">
-        <v>62.637176470588244</v>
+        <v>62.773291046064649</v>
       </c>
       <c r="F34">
         <v>62.637176470588244</v>
@@ -2941,7 +2941,7 @@
         <v>70</v>
       </c>
       <c r="E35">
-        <v>59.608183486238531</v>
+        <v>59.565623358566349</v>
       </c>
       <c r="F35">
         <v>59.608183486238531</v>
@@ -2994,7 +2994,7 @@
         <v>70</v>
       </c>
       <c r="E36">
-        <v>63.077394495412847</v>
+        <v>63.070743086667697</v>
       </c>
       <c r="F36">
         <v>63.077394495412847</v>
@@ -3047,7 +3047,7 @@
         <v>70</v>
       </c>
       <c r="E37">
-        <v>62.637176470588244</v>
+        <v>62.773291046064649</v>
       </c>
       <c r="F37">
         <v>62.637176470588244</v>

</xml_diff>

<commit_message>
update LNG import emissions from DZ
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
+++ b/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{098E60FB-05B5-4CD2-B5DF-51A63E6759A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D7F5A4B-6650-494D-804D-0AAA844F0D29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BAA9D55F-0FEB-4558-AFDF-92239B956412}"/>
   </bookViews>
@@ -719,7 +719,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K2">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L2">
         <v>72.72</v>
@@ -741,15 +741,15 @@
       </c>
       <c r="S2">
         <f>U5-U4</f>
-        <v>15.1</v>
+        <v>18.2</v>
       </c>
       <c r="T2">
         <f>S2*T1</f>
-        <v>54360000</v>
+        <v>65520000</v>
       </c>
       <c r="U2">
         <f>T2/U1</f>
-        <v>54.36</v>
+        <v>65.52</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.35">
@@ -784,7 +784,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K3">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L3">
         <v>72.72</v>
@@ -837,7 +837,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K4">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L4">
         <v>72.72</v>
@@ -861,7 +861,7 @@
         <v>20.5</v>
       </c>
       <c r="U4">
-        <v>2.6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.35">
@@ -896,7 +896,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K5">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L5">
         <v>72.72</v>
@@ -920,7 +920,7 @@
         <v>18.7</v>
       </c>
       <c r="U5">
-        <v>17.7</v>
+        <v>19.2</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.35">
@@ -955,7 +955,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K6">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L6">
         <v>72.72</v>
@@ -1012,7 +1012,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K7">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L7">
         <v>72.72</v>
@@ -1065,7 +1065,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K8">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L8">
         <v>72.72</v>
@@ -1087,7 +1087,7 @@
       </c>
       <c r="R8">
         <f t="shared" ref="R8:R24" si="0">AA8</f>
-        <v>63.33970029352696</v>
+        <v>68.97373088212575</v>
       </c>
       <c r="S8" t="s">
         <v>70</v>
@@ -1106,11 +1106,11 @@
       </c>
       <c r="Z8">
         <f>((($U$4/$Y$22)*Y8)*$T$1)/$U$1</f>
-        <v>8.9797002935269568</v>
+        <v>3.4537308821257531</v>
       </c>
       <c r="AA8">
         <f>Z8+$U$2</f>
-        <v>63.33970029352696</v>
+        <v>68.97373088212575</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.35">
@@ -1145,7 +1145,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K9">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L9">
         <v>72.72</v>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="R9">
         <f t="shared" si="0"/>
-        <v>63.291982079406765</v>
+        <v>68.955377722848752</v>
       </c>
       <c r="S9" t="s">
         <v>70</v>
@@ -1186,11 +1186,11 @@
       </c>
       <c r="Z9">
         <f t="shared" ref="Z9:Z24" si="1">((($U$4/$Y$22)*Y9)*$T$1)/$U$1</f>
-        <v>8.9319820794067688</v>
+        <v>3.4353777228487563</v>
       </c>
       <c r="AA9">
         <f t="shared" ref="AA9:AA24" si="2">Z9+$U$2</f>
-        <v>63.291982079406765</v>
+        <v>68.955377722848752</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.35">
@@ -1225,7 +1225,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K10">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L10">
         <v>72.72</v>
@@ -1247,7 +1247,7 @@
       </c>
       <c r="R10">
         <f t="shared" si="0"/>
-        <v>59.567069365054842</v>
+        <v>67.522718986559553</v>
       </c>
       <c r="S10" t="s">
         <v>70</v>
@@ -1266,11 +1266,11 @@
       </c>
       <c r="Z10">
         <f t="shared" si="1"/>
-        <v>5.207069365054843</v>
+        <v>2.0027189865595547</v>
       </c>
       <c r="AA10">
         <f t="shared" si="2"/>
-        <v>59.567069365054842</v>
+        <v>67.522718986559553</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.35">
@@ -1305,7 +1305,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K11">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L11">
         <v>72.72</v>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="R11">
         <f t="shared" si="0"/>
-        <v>60.700738452031516</v>
+        <v>67.958745558473652</v>
       </c>
       <c r="S11" t="s">
         <v>70</v>
@@ -1339,18 +1339,18 @@
         <v>0</v>
       </c>
       <c r="X11">
-        <v>4385</v>
+        <v>1496.9745220516984</v>
       </c>
       <c r="Y11">
         <v>7056.9756232588752</v>
       </c>
       <c r="Z11">
         <f t="shared" si="1"/>
-        <v>6.3407384520315153</v>
+        <v>2.4387455584736597</v>
       </c>
       <c r="AA11">
         <f t="shared" si="2"/>
-        <v>60.700738452031516</v>
+        <v>67.958745558473652</v>
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.35">
@@ -1385,7 +1385,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K12">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L12">
         <v>72.72</v>
@@ -1407,7 +1407,7 @@
       </c>
       <c r="R12">
         <f t="shared" si="0"/>
-        <v>60.519987640970186</v>
+        <v>67.889226015757757</v>
       </c>
       <c r="S12" t="s">
         <v>70</v>
@@ -1426,11 +1426,11 @@
       </c>
       <c r="Z12">
         <f t="shared" si="1"/>
-        <v>6.1599876409701837</v>
+        <v>2.3692260157577629</v>
       </c>
       <c r="AA12">
         <f t="shared" si="2"/>
-        <v>60.519987640970186</v>
+        <v>67.889226015757757</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.35">
@@ -1465,7 +1465,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K13">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L13">
         <v>72.72</v>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="R13">
         <f t="shared" si="0"/>
-        <v>64.690270353777223</v>
+        <v>69.493180905298928</v>
       </c>
       <c r="S13" t="s">
         <v>70</v>
@@ -1506,11 +1506,11 @@
       </c>
       <c r="Z13">
         <f t="shared" si="1"/>
-        <v>10.330270353777228</v>
+        <v>3.9731809052989338</v>
       </c>
       <c r="AA13">
         <f t="shared" si="2"/>
-        <v>64.690270353777223</v>
+        <v>69.493180905298928</v>
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.35">
@@ -1545,7 +1545,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K14">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L14">
         <v>72.72</v>
@@ -1567,7 +1567,7 @@
       </c>
       <c r="R14">
         <f t="shared" si="0"/>
-        <v>63.435136721767336</v>
+        <v>69.010437200679746</v>
       </c>
       <c r="S14" t="s">
         <v>70</v>
@@ -1586,11 +1586,11 @@
       </c>
       <c r="Z14">
         <f t="shared" si="1"/>
-        <v>9.0751367217673398</v>
+        <v>3.4904372006797462</v>
       </c>
       <c r="AA14">
         <f t="shared" si="2"/>
-        <v>63.435136721767336</v>
+        <v>69.010437200679746</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.35">
@@ -1625,7 +1625,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K15">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L15">
         <v>72.72</v>
@@ -1647,7 +1647,7 @@
       </c>
       <c r="R15">
         <f t="shared" si="0"/>
-        <v>64.414083114475517</v>
+        <v>69.386955044029037</v>
       </c>
       <c r="S15" t="s">
         <v>70</v>
@@ -1666,11 +1666,11 @@
       </c>
       <c r="Z15">
         <f t="shared" si="1"/>
-        <v>10.054083114475512</v>
+        <v>3.866955044029043</v>
       </c>
       <c r="AA15">
         <f t="shared" si="2"/>
-        <v>64.414083114475517</v>
+        <v>69.386955044029037</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.35">
@@ -1705,7 +1705,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K16">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L16">
         <v>72.72</v>
@@ -1727,7 +1727,7 @@
       </c>
       <c r="R16">
         <f t="shared" si="0"/>
-        <v>61.877787733662906</v>
+        <v>68.411456820639572</v>
       </c>
       <c r="S16" t="s">
         <v>70</v>
@@ -1746,11 +1746,11 @@
       </c>
       <c r="Z16">
         <f t="shared" si="1"/>
-        <v>7.5177877336629066</v>
+        <v>2.8914568206395801</v>
       </c>
       <c r="AA16">
         <f t="shared" si="2"/>
-        <v>61.877787733662906</v>
+        <v>68.411456820639572</v>
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.35">
@@ -1785,7 +1785,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K17">
-        <v>72.72</v>
+        <v>67.958745558473652</v>
       </c>
       <c r="L17">
         <v>72.72</v>
@@ -1807,7 +1807,7 @@
       </c>
       <c r="R17">
         <f t="shared" si="0"/>
-        <v>60.997169782172101</v>
+        <v>68.072757608527724</v>
       </c>
       <c r="S17" t="s">
         <v>70</v>
@@ -1819,18 +1819,18 @@
         <v>0</v>
       </c>
       <c r="X17">
-        <v>4590</v>
+        <v>1477.9000485607401</v>
       </c>
       <c r="Y17">
         <v>7386.8912453268504</v>
       </c>
       <c r="Z17">
         <f t="shared" si="1"/>
-        <v>6.6371697821720996</v>
+        <v>2.5527576085277301</v>
       </c>
       <c r="AA17">
         <f t="shared" si="2"/>
-        <v>60.997169782172101</v>
+        <v>68.072757608527724</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.35">
@@ -1865,7 +1865,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K18">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L18">
         <v>72.72</v>
@@ -1887,7 +1887,7 @@
       </c>
       <c r="R18">
         <f t="shared" si="0"/>
-        <v>59.565623358566349</v>
+        <v>67.522162830217823</v>
       </c>
       <c r="S18" t="s">
         <v>70</v>
@@ -1906,11 +1906,11 @@
       </c>
       <c r="Z18">
         <f t="shared" si="1"/>
-        <v>5.2056233585663518</v>
+        <v>2.002162830217828</v>
       </c>
       <c r="AA18">
         <f t="shared" si="2"/>
-        <v>59.565623358566349</v>
+        <v>67.522162830217823</v>
       </c>
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.35">
@@ -1945,7 +1945,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K19">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L19">
         <v>72.72</v>
@@ -1967,7 +1967,7 @@
       </c>
       <c r="R19">
         <f t="shared" si="0"/>
-        <v>63.070743086667697</v>
+        <v>68.870285802564496</v>
       </c>
       <c r="S19" t="s">
         <v>70</v>
@@ -1986,11 +1986,11 @@
       </c>
       <c r="Z19">
         <f t="shared" si="1"/>
-        <v>8.710743086667696</v>
+        <v>3.3502858025644979</v>
       </c>
       <c r="AA19">
         <f t="shared" si="2"/>
-        <v>63.070743086667697</v>
+        <v>68.870285802564496</v>
       </c>
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.35">
@@ -2025,7 +2025,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K20">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L20">
         <v>72.72</v>
@@ -2047,7 +2047,7 @@
       </c>
       <c r="R20">
         <f t="shared" si="0"/>
-        <v>64.996823729337251</v>
+        <v>69.611086049745097</v>
       </c>
       <c r="S20" t="s">
         <v>70</v>
@@ -2066,11 +2066,11 @@
       </c>
       <c r="Z20">
         <f t="shared" si="1"/>
-        <v>10.636823729337245</v>
+        <v>4.091086049745094</v>
       </c>
       <c r="AA20">
         <f t="shared" si="2"/>
-        <v>64.996823729337251</v>
+        <v>69.611086049745097</v>
       </c>
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.35">
@@ -2105,7 +2105,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K21">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L21">
         <v>72.72</v>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="R21">
         <f t="shared" si="0"/>
-        <v>64.996823729337251</v>
+        <v>69.611086049745097</v>
       </c>
       <c r="S21" t="s">
         <v>70</v>
@@ -2146,11 +2146,11 @@
       </c>
       <c r="Z21">
         <f t="shared" si="1"/>
-        <v>10.636823729337245</v>
+        <v>4.091086049745094</v>
       </c>
       <c r="AA21">
         <f t="shared" si="2"/>
-        <v>64.996823729337251</v>
+        <v>69.611086049745097</v>
       </c>
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.35">
@@ -2185,7 +2185,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K22">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L22">
         <v>72.72</v>
@@ -2207,7 +2207,7 @@
       </c>
       <c r="R22">
         <f t="shared" si="0"/>
-        <v>63.72</v>
+        <v>69.11999999999999</v>
       </c>
       <c r="S22" t="s">
         <v>70</v>
@@ -2219,18 +2219,18 @@
         <v>0</v>
       </c>
       <c r="X22">
-        <v>6473</v>
+        <v>3083.6821009103123</v>
       </c>
       <c r="Y22">
         <v>10417.286934858541</v>
       </c>
       <c r="Z22">
         <f t="shared" si="1"/>
-        <v>9.36</v>
+        <v>3.6</v>
       </c>
       <c r="AA22">
         <f t="shared" si="2"/>
-        <v>63.72</v>
+        <v>69.11999999999999</v>
       </c>
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.35">
@@ -2265,7 +2265,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K23">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L23">
         <v>72.72</v>
@@ -2287,7 +2287,7 @@
       </c>
       <c r="R23">
         <f t="shared" si="0"/>
-        <v>63.051945002317318</v>
+        <v>68.863055770122045</v>
       </c>
       <c r="S23" t="s">
         <v>70</v>
@@ -2306,11 +2306,11 @@
       </c>
       <c r="Z23">
         <f t="shared" si="1"/>
-        <v>8.6919450023173184</v>
+        <v>3.3430557701220454</v>
       </c>
       <c r="AA23">
         <f t="shared" si="2"/>
-        <v>63.051945002317318</v>
+        <v>68.863055770122045</v>
       </c>
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.35">
@@ -2345,7 +2345,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K24">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L24">
         <v>72.72</v>
@@ -2367,7 +2367,7 @@
       </c>
       <c r="R24">
         <f t="shared" si="0"/>
-        <v>64.910063340027804</v>
+        <v>69.577716669241454</v>
       </c>
       <c r="S24" t="s">
         <v>70</v>
@@ -2386,11 +2386,11 @@
       </c>
       <c r="Z24">
         <f t="shared" si="1"/>
-        <v>10.550063340027807</v>
+        <v>4.0577166692414641</v>
       </c>
       <c r="AA24">
         <f t="shared" si="2"/>
-        <v>64.910063340027804</v>
+        <v>69.577716669241454</v>
       </c>
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.35">
@@ -2425,7 +2425,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K25">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L25">
         <v>72.72</v>
@@ -2447,7 +2447,7 @@
       </c>
       <c r="R25">
         <f>AVERAGE(R8:R24)</f>
-        <v>62.773291046064649</v>
+        <v>68.755881171563317</v>
       </c>
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.35">
@@ -2482,7 +2482,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K26">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L26">
         <v>72.72</v>
@@ -2535,7 +2535,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K27">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L27">
         <v>72.72</v>
@@ -2554,6 +2554,9 @@
       </c>
       <c r="Q27">
         <v>9.36</v>
+      </c>
+      <c r="U27">
+        <v>964.8646999038657</v>
       </c>
     </row>
     <row r="28" spans="1:27" x14ac:dyDescent="0.35">
@@ -2588,7 +2591,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K28">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L28">
         <v>72.72</v>
@@ -2607,6 +2610,9 @@
       </c>
       <c r="Q28">
         <v>9.36</v>
+      </c>
+      <c r="U28">
+        <v>532.10982214783257</v>
       </c>
     </row>
     <row r="29" spans="1:27" x14ac:dyDescent="0.35">
@@ -2641,7 +2647,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K29">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L29">
         <v>72.72</v>
@@ -2694,7 +2700,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K30">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L30">
         <v>72.72</v>
@@ -2747,7 +2753,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K31">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L31">
         <v>72.72</v>
@@ -2766,6 +2772,14 @@
       </c>
       <c r="Q31">
         <v>9.36</v>
+      </c>
+      <c r="S31">
+        <f>(K32+K17)/2</f>
+        <v>68.015751583500688</v>
+      </c>
+      <c r="U31">
+        <f>SUM(U27:U29)</f>
+        <v>1496.9745220516984</v>
       </c>
     </row>
     <row r="32" spans="1:27" x14ac:dyDescent="0.35">
@@ -2800,7 +2814,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K32">
-        <v>72.72</v>
+        <v>68.072757608527724</v>
       </c>
       <c r="L32">
         <v>72.72</v>
@@ -2853,7 +2867,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K33">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L33">
         <v>72.72</v>
@@ -2906,7 +2920,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K34">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L34">
         <v>72.72</v>
@@ -2959,7 +2973,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K35">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L35">
         <v>72.72</v>
@@ -3012,7 +3026,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K36">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L36">
         <v>72.72</v>
@@ -3065,7 +3079,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="K37">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="L37">
         <v>72.72</v>

</xml_diff>

<commit_message>
update LNG import emissions from IM
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
+++ b/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D7F5A4B-6650-494D-804D-0AAA844F0D29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{164DB5F0-6DE7-4435-AA5B-766BA8DD57F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BAA9D55F-0FEB-4558-AFDF-92239B956412}"/>
   </bookViews>
@@ -249,7 +249,7 @@
     <t>LV_LNG</t>
   </si>
   <si>
-    <t>ME_LNG</t>
+    <t>IM_LNG</t>
   </si>
 </sst>
 </file>
@@ -734,22 +734,22 @@
         <v>72.72</v>
       </c>
       <c r="P2">
-        <v>70.56</v>
+        <v>69.650954303405584</v>
       </c>
       <c r="Q2">
         <v>9.36</v>
       </c>
       <c r="S2">
         <f>U5-U4</f>
-        <v>18.2</v>
+        <v>16</v>
       </c>
       <c r="T2">
         <f>S2*T1</f>
-        <v>65520000</v>
+        <v>57600000</v>
       </c>
       <c r="U2">
         <f>T2/U1</f>
-        <v>65.52</v>
+        <v>57.6</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.35">
@@ -799,7 +799,7 @@
         <v>72.72</v>
       </c>
       <c r="P3">
-        <v>70.56</v>
+        <v>69.650954303405584</v>
       </c>
       <c r="Q3">
         <v>9.36</v>
@@ -852,7 +852,7 @@
         <v>72.72</v>
       </c>
       <c r="P4">
-        <v>70.56</v>
+        <v>70.201212631578954</v>
       </c>
       <c r="Q4">
         <v>9.36</v>
@@ -861,7 +861,8 @@
         <v>20.5</v>
       </c>
       <c r="U4">
-        <v>1</v>
+        <f>(3.7+3.5)/2</f>
+        <v>3.6</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.35">
@@ -911,7 +912,7 @@
         <v>72.72</v>
       </c>
       <c r="P5">
-        <v>70.56</v>
+        <v>69.650954303405584</v>
       </c>
       <c r="Q5">
         <v>9.36</v>
@@ -920,7 +921,8 @@
         <v>18.7</v>
       </c>
       <c r="U5">
-        <v>19.2</v>
+        <f>(20.5+18.7)/2</f>
+        <v>19.600000000000001</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.35">
@@ -970,7 +972,7 @@
         <v>72.72</v>
       </c>
       <c r="P6">
-        <v>70.56</v>
+        <v>69.650954303405584</v>
       </c>
       <c r="Q6">
         <v>9.36</v>
@@ -1027,7 +1029,7 @@
         <v>72.72</v>
       </c>
       <c r="P7">
-        <v>70.56</v>
+        <v>67.541002105263161</v>
       </c>
       <c r="Q7">
         <v>9.36</v>
@@ -1080,14 +1082,14 @@
         <v>72.72</v>
       </c>
       <c r="P8">
-        <v>70.56</v>
+        <v>69.650954303405584</v>
       </c>
       <c r="Q8">
         <v>9.36</v>
       </c>
       <c r="R8">
-        <f t="shared" ref="R8:R24" si="0">AA8</f>
-        <v>68.97373088212575</v>
+        <f t="shared" ref="P6:R24" si="0">AA8</f>
+        <v>70.201212631578954</v>
       </c>
       <c r="S8" t="s">
         <v>70</v>
@@ -1099,18 +1101,18 @@
         <v>0</v>
       </c>
       <c r="X8">
-        <v>6210</v>
+        <v>9237</v>
       </c>
       <c r="Y8">
-        <v>9994.0293319127977</v>
+        <v>14865.515127033575</v>
       </c>
       <c r="Z8">
         <f>((($U$4/$Y$22)*Y8)*$T$1)/$U$1</f>
-        <v>3.4537308821257531</v>
+        <v>12.601212631578948</v>
       </c>
       <c r="AA8">
         <f>Z8+$U$2</f>
-        <v>68.97373088212575</v>
+        <v>70.201212631578954</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.35">
@@ -1160,14 +1162,14 @@
         <v>72.72</v>
       </c>
       <c r="P9">
-        <v>70.56</v>
+        <v>69.650954303405584</v>
       </c>
       <c r="Q9">
         <v>9.36</v>
       </c>
       <c r="R9">
         <f t="shared" si="0"/>
-        <v>68.955377722848752</v>
+        <v>69.737381052631576</v>
       </c>
       <c r="S9" t="s">
         <v>70</v>
@@ -1179,18 +1181,18 @@
         <v>0</v>
       </c>
       <c r="X9">
-        <v>6177</v>
+        <v>8897</v>
       </c>
       <c r="Y9">
-        <v>9940.9209634823437</v>
+        <v>14318.337997750106</v>
       </c>
       <c r="Z9">
         <f t="shared" ref="Z9:Z24" si="1">((($U$4/$Y$22)*Y9)*$T$1)/$U$1</f>
-        <v>3.4353777228487563</v>
+        <v>12.13738105263158</v>
       </c>
       <c r="AA9">
         <f t="shared" ref="AA9:AA24" si="2">Z9+$U$2</f>
-        <v>68.955377722848752</v>
+        <v>69.737381052631576</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.35">
@@ -1240,14 +1242,14 @@
         <v>72.72</v>
       </c>
       <c r="P10">
-        <v>70.56</v>
+        <v>71.764597894736838</v>
       </c>
       <c r="Q10">
         <v>9.36</v>
       </c>
       <c r="R10">
         <f t="shared" si="0"/>
-        <v>67.522718986559553</v>
+        <v>66.790686315789472</v>
       </c>
       <c r="S10" t="s">
         <v>70</v>
@@ -1259,18 +1261,18 @@
         <v>0</v>
       </c>
       <c r="X10">
-        <v>3601</v>
+        <v>6737</v>
       </c>
       <c r="Y10">
-        <v>5795.2495369111084</v>
+        <v>10842.153882302176</v>
       </c>
       <c r="Z10">
         <f t="shared" si="1"/>
-        <v>2.0027189865595547</v>
+        <v>9.190686315789474</v>
       </c>
       <c r="AA10">
         <f t="shared" si="2"/>
-        <v>67.522718986559553</v>
+        <v>66.790686315789472</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.35">
@@ -1320,14 +1322,14 @@
         <v>72.72</v>
       </c>
       <c r="P11">
-        <v>70.56</v>
+        <v>71.764597894736838</v>
       </c>
       <c r="Q11">
         <v>9.36</v>
       </c>
       <c r="R11">
         <f t="shared" si="0"/>
-        <v>67.958745558473652</v>
+        <v>67.711528421052634</v>
       </c>
       <c r="S11" t="s">
         <v>70</v>
@@ -1339,18 +1341,18 @@
         <v>0</v>
       </c>
       <c r="X11">
-        <v>1496.9745220516984</v>
+        <v>7412</v>
       </c>
       <c r="Y11">
-        <v>7056.9756232588752</v>
+        <v>11928.461418379655</v>
       </c>
       <c r="Z11">
         <f t="shared" si="1"/>
-        <v>2.4387455584736597</v>
+        <v>10.111528421052633</v>
       </c>
       <c r="AA11">
         <f t="shared" si="2"/>
-        <v>67.958745558473652</v>
+        <v>67.711528421052634</v>
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.35">
@@ -1400,14 +1402,14 @@
         <v>72.72</v>
       </c>
       <c r="P12">
-        <v>70.56</v>
+        <v>69.737381052631576</v>
       </c>
       <c r="Q12">
         <v>9.36</v>
       </c>
       <c r="R12">
         <f t="shared" si="0"/>
-        <v>67.889226015757757</v>
+        <v>67.541002105263161</v>
       </c>
       <c r="S12" t="s">
         <v>70</v>
@@ -1419,18 +1421,18 @@
         <v>0</v>
       </c>
       <c r="X12">
-        <v>4260</v>
+        <v>7287</v>
       </c>
       <c r="Y12">
-        <v>6855.807561022305</v>
+        <v>11727.293356143084</v>
       </c>
       <c r="Z12">
         <f t="shared" si="1"/>
-        <v>2.3692260157577629</v>
+        <v>9.9410021052631592</v>
       </c>
       <c r="AA12">
         <f t="shared" si="2"/>
-        <v>67.889226015757757</v>
+        <v>67.541002105263161</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.35">
@@ -1487,7 +1489,7 @@
       </c>
       <c r="R13">
         <f t="shared" si="0"/>
-        <v>69.493180905298928</v>
+        <v>71.475385263157904</v>
       </c>
       <c r="S13" t="s">
         <v>70</v>
@@ -1499,18 +1501,18 @@
         <v>0</v>
       </c>
       <c r="X13">
-        <v>7144</v>
+        <v>10171</v>
       </c>
       <c r="Y13">
-        <v>11497.157092944448</v>
+        <v>16368.642888065227</v>
       </c>
       <c r="Z13">
         <f t="shared" si="1"/>
-        <v>3.9731809052989338</v>
+        <v>13.875385263157895</v>
       </c>
       <c r="AA13">
         <f t="shared" si="2"/>
-        <v>69.493180905298928</v>
+        <v>71.475385263157904</v>
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.35">
@@ -1560,14 +1562,14 @@
         <v>72.72</v>
       </c>
       <c r="P14">
-        <v>70.56</v>
+        <v>66.790686315789472</v>
       </c>
       <c r="Q14">
         <v>9.36</v>
       </c>
       <c r="R14">
         <f t="shared" si="0"/>
-        <v>69.010437200679746</v>
+        <v>70.291250526315793</v>
       </c>
       <c r="S14" t="s">
         <v>70</v>
@@ -1579,18 +1581,18 @@
         <v>0</v>
       </c>
       <c r="X14">
-        <v>6276</v>
+        <v>9303</v>
       </c>
       <c r="Y14">
-        <v>10100.246068773706</v>
+        <v>14971.731863894485</v>
       </c>
       <c r="Z14">
         <f t="shared" si="1"/>
-        <v>3.4904372006797462</v>
+        <v>12.691250526315789</v>
       </c>
       <c r="AA14">
         <f t="shared" si="2"/>
-        <v>69.010437200679746</v>
+        <v>70.291250526315793</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.35">
@@ -1640,14 +1642,14 @@
         <v>72.72</v>
       </c>
       <c r="P15">
-        <v>70.56</v>
+        <v>69.650954303405584</v>
       </c>
       <c r="Q15">
         <v>9.36</v>
       </c>
       <c r="R15">
         <f t="shared" si="0"/>
-        <v>69.386955044029037</v>
+        <v>71.214821052631578</v>
       </c>
       <c r="S15" t="s">
         <v>70</v>
@@ -1659,18 +1661,18 @@
         <v>0</v>
       </c>
       <c r="X15">
-        <v>6953</v>
+        <v>9980</v>
       </c>
       <c r="Y15">
-        <v>11189.772293846969</v>
+        <v>16061.258088967748</v>
       </c>
       <c r="Z15">
         <f t="shared" si="1"/>
-        <v>3.866955044029043</v>
+        <v>13.61482105263158</v>
       </c>
       <c r="AA15">
         <f t="shared" si="2"/>
-        <v>69.386955044029037</v>
+        <v>71.214821052631578</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.35">
@@ -1720,14 +1722,14 @@
         <v>72.72</v>
       </c>
       <c r="P16">
-        <v>70.56</v>
+        <v>69.929734736842107</v>
       </c>
       <c r="Q16">
         <v>9.36</v>
       </c>
       <c r="R16">
         <f t="shared" si="0"/>
-        <v>68.411456820639572</v>
+        <v>68.821995789473689</v>
       </c>
       <c r="S16" t="s">
         <v>70</v>
@@ -1739,18 +1741,18 @@
         <v>0</v>
       </c>
       <c r="X16">
-        <v>5199</v>
+        <v>8226</v>
       </c>
       <c r="Y16">
-        <v>8366.9820445434198</v>
+        <v>13238.467839664198</v>
       </c>
       <c r="Z16">
         <f t="shared" si="1"/>
-        <v>2.8914568206395801</v>
+        <v>11.221995789473684</v>
       </c>
       <c r="AA16">
         <f t="shared" si="2"/>
-        <v>68.411456820639572</v>
+        <v>68.821995789473689</v>
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.35">
@@ -1800,14 +1802,14 @@
         <v>72.72</v>
       </c>
       <c r="P17">
-        <v>70.56</v>
+        <v>71.475385263157904</v>
       </c>
       <c r="Q17">
         <v>9.36</v>
       </c>
       <c r="R17">
         <f t="shared" si="0"/>
-        <v>68.072757608527724</v>
+        <v>67.991191578947365</v>
       </c>
       <c r="S17" t="s">
         <v>70</v>
@@ -1819,18 +1821,18 @@
         <v>0</v>
       </c>
       <c r="X17">
-        <v>1477.9000485607401</v>
+        <v>7617</v>
       </c>
       <c r="Y17">
-        <v>7386.8912453268504</v>
+        <v>12258.377040447629</v>
       </c>
       <c r="Z17">
         <f t="shared" si="1"/>
-        <v>2.5527576085277301</v>
+        <v>10.391191578947371</v>
       </c>
       <c r="AA17">
         <f t="shared" si="2"/>
-        <v>68.072757608527724</v>
+        <v>67.991191578947365</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.35">
@@ -1880,14 +1882,14 @@
         <v>72.72</v>
       </c>
       <c r="P18">
-        <v>70.56</v>
+        <v>71.682745263157898</v>
       </c>
       <c r="Q18">
         <v>9.36</v>
       </c>
       <c r="R18">
         <f t="shared" si="0"/>
-        <v>67.522162830217823</v>
+        <v>66.640623157894737</v>
       </c>
       <c r="S18" t="s">
         <v>70</v>
@@ -1899,18 +1901,18 @@
         <v>0</v>
       </c>
       <c r="X18">
-        <v>3600</v>
+        <v>6627</v>
       </c>
       <c r="Y18">
-        <v>5793.640192413216</v>
+        <v>10665.125987533995</v>
       </c>
       <c r="Z18">
         <f t="shared" si="1"/>
-        <v>2.002162830217828</v>
+        <v>9.0406231578947374</v>
       </c>
       <c r="AA18">
         <f t="shared" si="2"/>
-        <v>67.522162830217823</v>
+        <v>66.640623157894737</v>
       </c>
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.35">
@@ -1960,14 +1962,14 @@
         <v>72.72</v>
       </c>
       <c r="P19">
-        <v>70.56</v>
+        <v>69.650954303405584</v>
       </c>
       <c r="Q19">
         <v>9.36</v>
       </c>
       <c r="R19">
         <f t="shared" si="0"/>
-        <v>68.870285802564496</v>
+        <v>69.947469473684208</v>
       </c>
       <c r="S19" t="s">
         <v>70</v>
@@ -1979,18 +1981,18 @@
         <v>0</v>
       </c>
       <c r="X19">
-        <v>6024</v>
+        <v>9051</v>
       </c>
       <c r="Y19">
-        <v>9694.6912553047805</v>
+        <v>14566.17705042556</v>
       </c>
       <c r="Z19">
         <f t="shared" si="1"/>
-        <v>3.3502858025644979</v>
+        <v>12.347469473684212</v>
       </c>
       <c r="AA19">
         <f t="shared" si="2"/>
-        <v>68.870285802564496</v>
+        <v>69.947469473684208</v>
       </c>
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.35">
@@ -2040,14 +2042,14 @@
         <v>72.72</v>
       </c>
       <c r="P20">
-        <v>70.56</v>
+        <v>69.650954303405584</v>
       </c>
       <c r="Q20">
         <v>9.36</v>
       </c>
       <c r="R20">
         <f t="shared" si="0"/>
-        <v>69.611086049745097</v>
+        <v>71.764597894736838</v>
       </c>
       <c r="S20" t="s">
         <v>70</v>
@@ -2059,18 +2061,18 @@
         <v>0</v>
       </c>
       <c r="X20">
-        <v>7356</v>
+        <v>10383</v>
       </c>
       <c r="Y20">
-        <v>11838.338126497671</v>
+        <v>16709.823921618448</v>
       </c>
       <c r="Z20">
         <f t="shared" si="1"/>
-        <v>4.091086049745094</v>
+        <v>14.164597894736842</v>
       </c>
       <c r="AA20">
         <f t="shared" si="2"/>
-        <v>69.611086049745097</v>
+        <v>71.764597894736838</v>
       </c>
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.35">
@@ -2120,14 +2122,14 @@
         <v>72.72</v>
       </c>
       <c r="P21">
-        <v>70.56</v>
+        <v>69.650954303405584</v>
       </c>
       <c r="Q21">
         <v>9.36</v>
       </c>
       <c r="R21">
         <f t="shared" si="0"/>
-        <v>69.611086049745097</v>
+        <v>71.764597894736838</v>
       </c>
       <c r="S21" t="s">
         <v>70</v>
@@ -2139,18 +2141,18 @@
         <v>0</v>
       </c>
       <c r="X21">
-        <v>7356</v>
+        <v>10383</v>
       </c>
       <c r="Y21">
-        <v>11838.338126497671</v>
+        <v>16709.823921618448</v>
       </c>
       <c r="Z21">
         <f t="shared" si="1"/>
-        <v>4.091086049745094</v>
+        <v>14.164597894736842</v>
       </c>
       <c r="AA21">
         <f t="shared" si="2"/>
-        <v>69.611086049745097</v>
+        <v>71.764597894736838</v>
       </c>
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.35">
@@ -2200,14 +2202,14 @@
         <v>72.72</v>
       </c>
       <c r="P22">
-        <v>70.56</v>
+        <v>70.291250526315793</v>
       </c>
       <c r="Q22">
         <v>9.36</v>
       </c>
       <c r="R22">
         <f t="shared" si="0"/>
-        <v>69.11999999999999</v>
+        <v>70.56</v>
       </c>
       <c r="S22" t="s">
         <v>70</v>
@@ -2219,18 +2221,18 @@
         <v>0</v>
       </c>
       <c r="X22">
-        <v>3083.6821009103123</v>
+        <v>9500</v>
       </c>
       <c r="Y22">
-        <v>10417.286934858541</v>
+        <v>15288.772729979319</v>
       </c>
       <c r="Z22">
         <f t="shared" si="1"/>
-        <v>3.6</v>
+        <v>12.96</v>
       </c>
       <c r="AA22">
         <f t="shared" si="2"/>
-        <v>69.11999999999999</v>
+        <v>70.56</v>
       </c>
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.35">
@@ -2280,14 +2282,14 @@
         <v>72.72</v>
       </c>
       <c r="P23">
-        <v>70.56</v>
+        <v>69.650954303405584</v>
       </c>
       <c r="Q23">
         <v>9.36</v>
       </c>
       <c r="R23">
         <f t="shared" si="0"/>
-        <v>68.863055770122045</v>
+        <v>69.929734736842107</v>
       </c>
       <c r="S23" t="s">
         <v>70</v>
@@ -2299,18 +2301,18 @@
         <v>0</v>
       </c>
       <c r="X23">
-        <v>6011</v>
+        <v>9038</v>
       </c>
       <c r="Y23">
-        <v>9673.7697768321777</v>
+        <v>14545.255571952957</v>
       </c>
       <c r="Z23">
         <f t="shared" si="1"/>
-        <v>3.3430557701220454</v>
+        <v>12.329734736842108</v>
       </c>
       <c r="AA23">
         <f t="shared" si="2"/>
-        <v>68.863055770122045</v>
+        <v>69.929734736842107</v>
       </c>
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.35">
@@ -2360,14 +2362,14 @@
         <v>72.72</v>
       </c>
       <c r="P24">
-        <v>70.56</v>
+        <v>69.650954303405584</v>
       </c>
       <c r="Q24">
         <v>9.36</v>
       </c>
       <c r="R24">
         <f t="shared" si="0"/>
-        <v>69.577716669241454</v>
+        <v>71.682745263157898</v>
       </c>
       <c r="S24" t="s">
         <v>70</v>
@@ -2379,18 +2381,18 @@
         <v>0</v>
       </c>
       <c r="X24">
-        <v>7296</v>
+        <v>10323</v>
       </c>
       <c r="Y24">
-        <v>11741.777456624117</v>
+        <v>16613.263251744895</v>
       </c>
       <c r="Z24">
         <f t="shared" si="1"/>
-        <v>4.0577166692414641</v>
+        <v>14.082745263157895</v>
       </c>
       <c r="AA24">
         <f t="shared" si="2"/>
-        <v>69.577716669241454</v>
+        <v>71.682745263157898</v>
       </c>
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.35">
@@ -2440,14 +2442,14 @@
         <v>72.72</v>
       </c>
       <c r="P25">
-        <v>70.56</v>
+        <v>71.214821052631578</v>
       </c>
       <c r="Q25">
         <v>9.36</v>
       </c>
       <c r="R25">
         <f>AVERAGE(R8:R24)</f>
-        <v>68.755881171563317</v>
+        <v>69.650954303405584</v>
       </c>
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.35">
@@ -2497,7 +2499,7 @@
         <v>72.72</v>
       </c>
       <c r="P26">
-        <v>70.56</v>
+        <v>68.821995789473689</v>
       </c>
       <c r="Q26">
         <v>9.36</v>
@@ -2550,7 +2552,7 @@
         <v>72.72</v>
       </c>
       <c r="P27">
-        <v>70.56</v>
+        <v>69.650954303405584</v>
       </c>
       <c r="Q27">
         <v>9.36</v>
@@ -2606,7 +2608,7 @@
         <v>72.72</v>
       </c>
       <c r="P28">
-        <v>70.56</v>
+        <v>69.650954303405584</v>
       </c>
       <c r="Q28">
         <v>9.36</v>
@@ -2662,7 +2664,7 @@
         <v>72.72</v>
       </c>
       <c r="P29">
-        <v>70.56</v>
+        <v>69.650954303405584</v>
       </c>
       <c r="Q29">
         <v>9.36</v>
@@ -2715,7 +2717,7 @@
         <v>72.72</v>
       </c>
       <c r="P30">
-        <v>70.56</v>
+        <v>69.650954303405584</v>
       </c>
       <c r="Q30">
         <v>9.36</v>
@@ -2768,7 +2770,7 @@
         <v>72.72</v>
       </c>
       <c r="P31">
-        <v>70.56</v>
+        <v>69.650954303405584</v>
       </c>
       <c r="Q31">
         <v>9.36</v>
@@ -2829,7 +2831,7 @@
         <v>72.72</v>
       </c>
       <c r="P32">
-        <v>70.56</v>
+        <v>67.991191578947365</v>
       </c>
       <c r="Q32">
         <v>9.36</v>
@@ -2882,7 +2884,7 @@
         <v>72.72</v>
       </c>
       <c r="P33">
-        <v>70.56</v>
+        <v>69.650954303405584</v>
       </c>
       <c r="Q33">
         <v>9.36</v>
@@ -2935,7 +2937,7 @@
         <v>72.72</v>
       </c>
       <c r="P34">
-        <v>70.56</v>
+        <v>69.650954303405584</v>
       </c>
       <c r="Q34">
         <v>9.36</v>
@@ -2988,7 +2990,7 @@
         <v>72.72</v>
       </c>
       <c r="P35">
-        <v>70.56</v>
+        <v>66.640623157894737</v>
       </c>
       <c r="Q35">
         <v>9.36</v>
@@ -3041,7 +3043,7 @@
         <v>72.72</v>
       </c>
       <c r="P36">
-        <v>70.56</v>
+        <v>69.947469473684208</v>
       </c>
       <c r="Q36">
         <v>9.36</v>
@@ -3094,7 +3096,7 @@
         <v>72.72</v>
       </c>
       <c r="P37">
-        <v>70.56</v>
+        <v>69.650954303405584</v>
       </c>
       <c r="Q37">
         <v>9.36</v>

</xml_diff>

<commit_message>
update LNG import emissions from RU and CR
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
+++ b/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{164DB5F0-6DE7-4435-AA5B-766BA8DD57F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD679743-7103-470C-84DC-12B613816F5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BAA9D55F-0FEB-4558-AFDF-92239B956412}"/>
   </bookViews>
@@ -713,43 +713,43 @@
         <v>90</v>
       </c>
       <c r="I2">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J2">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K2">
         <v>68.015751583500688</v>
       </c>
       <c r="L2">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M2">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N2">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O2">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P2">
         <v>69.650954303405584</v>
       </c>
       <c r="Q2">
-        <v>9.36</v>
+        <v>1</v>
       </c>
       <c r="S2">
         <f>U5-U4</f>
-        <v>16</v>
+        <v>1.5</v>
       </c>
       <c r="T2">
         <f>S2*T1</f>
-        <v>57600000</v>
+        <v>5400000</v>
       </c>
       <c r="U2">
         <f>T2/U1</f>
-        <v>57.6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.35">
@@ -778,31 +778,31 @@
         <v>90</v>
       </c>
       <c r="I3">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J3">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K3">
         <v>68.015751583500688</v>
       </c>
       <c r="L3">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M3">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N3">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O3">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P3">
         <v>69.650954303405584</v>
       </c>
       <c r="Q3">
-        <v>9.36</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.35">
@@ -831,38 +831,34 @@
         <v>90</v>
       </c>
       <c r="I4">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J4">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K4">
         <v>68.015751583500688</v>
       </c>
       <c r="L4">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M4">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N4">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O4">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P4">
         <v>70.201212631578954</v>
       </c>
       <c r="Q4">
-        <v>9.36</v>
-      </c>
-      <c r="S4">
-        <v>20.5</v>
+        <v>1</v>
       </c>
       <c r="U4">
-        <f>(3.7+3.5)/2</f>
-        <v>3.6</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.35">
@@ -891,38 +887,34 @@
         <v>90</v>
       </c>
       <c r="I5">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J5">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K5">
         <v>68.015751583500688</v>
       </c>
       <c r="L5">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M5">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N5">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O5">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P5">
         <v>69.650954303405584</v>
       </c>
       <c r="Q5">
-        <v>9.36</v>
-      </c>
-      <c r="S5">
-        <v>18.7</v>
+        <v>1</v>
       </c>
       <c r="U5">
-        <f>(20.5+18.7)/2</f>
-        <v>19.600000000000001</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.35">
@@ -951,35 +943,31 @@
         <v>90</v>
       </c>
       <c r="I6">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J6">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K6">
         <v>68.015751583500688</v>
       </c>
       <c r="L6">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M6">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N6">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O6">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P6">
         <v>69.650954303405584</v>
       </c>
       <c r="Q6">
-        <v>9.36</v>
-      </c>
-      <c r="S6">
-        <f>(S5+S4)/2</f>
-        <v>19.600000000000001</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.35">
@@ -1008,31 +996,31 @@
         <v>90</v>
       </c>
       <c r="I7">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J7">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K7">
         <v>68.015751583500688</v>
       </c>
       <c r="L7">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M7">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N7">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O7">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P7">
         <v>67.541002105263161</v>
       </c>
       <c r="Q7">
-        <v>9.36</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.35">
@@ -1061,35 +1049,35 @@
         <v>90</v>
       </c>
       <c r="I8">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J8">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K8">
         <v>68.015751583500688</v>
       </c>
       <c r="L8">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M8">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N8">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O8">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P8">
         <v>69.650954303405584</v>
       </c>
       <c r="Q8">
-        <v>9.36</v>
+        <v>1</v>
       </c>
       <c r="R8">
-        <f t="shared" ref="P6:R24" si="0">AA8</f>
-        <v>70.201212631578954</v>
+        <f t="shared" ref="R8:R24" si="0">AA8</f>
+        <v>6.5604478724514799</v>
       </c>
       <c r="S8" t="s">
         <v>70</v>
@@ -1104,15 +1092,15 @@
         <v>9237</v>
       </c>
       <c r="Y8">
-        <v>14865.515127033575</v>
+        <v>1544.841468711073</v>
       </c>
       <c r="Z8">
         <f>((($U$4/$Y$22)*Y8)*$T$1)/$U$1</f>
-        <v>12.601212631578948</v>
+        <v>1.1604478724514795</v>
       </c>
       <c r="AA8">
         <f>Z8+$U$2</f>
-        <v>70.201212631578954</v>
+        <v>6.5604478724514799</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.35">
@@ -1141,35 +1129,35 @@
         <v>90</v>
       </c>
       <c r="I9">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J9">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K9">
         <v>68.015751583500688</v>
       </c>
       <c r="L9">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M9">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N9">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O9">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P9">
         <v>69.650954303405584</v>
       </c>
       <c r="Q9">
-        <v>9.36</v>
+        <v>1</v>
       </c>
       <c r="R9">
         <f t="shared" si="0"/>
-        <v>69.737381052631576</v>
+        <v>6.9190068562697657</v>
       </c>
       <c r="S9" t="s">
         <v>70</v>
@@ -1184,15 +1172,15 @@
         <v>8897</v>
       </c>
       <c r="Y9">
-        <v>14318.337997750106</v>
+        <v>2022.171644698406</v>
       </c>
       <c r="Z9">
         <f t="shared" ref="Z9:Z24" si="1">((($U$4/$Y$22)*Y9)*$T$1)/$U$1</f>
-        <v>12.13738105263158</v>
+        <v>1.5190068562697654</v>
       </c>
       <c r="AA9">
         <f t="shared" ref="AA9:AA24" si="2">Z9+$U$2</f>
-        <v>69.737381052631576</v>
+        <v>6.9190068562697657</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.35">
@@ -1221,35 +1209,35 @@
         <v>90</v>
       </c>
       <c r="I10">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J10">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K10">
         <v>68.015751583500688</v>
       </c>
       <c r="L10">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M10">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N10">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O10">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P10">
         <v>71.764597894736838</v>
       </c>
       <c r="Q10">
-        <v>9.36</v>
+        <v>1</v>
       </c>
       <c r="R10">
         <f t="shared" si="0"/>
-        <v>66.790686315789472</v>
+        <v>13.544366046832366</v>
       </c>
       <c r="S10" t="s">
         <v>70</v>
@@ -1268,11 +1256,11 @@
       </c>
       <c r="Z10">
         <f t="shared" si="1"/>
-        <v>9.190686315789474</v>
+        <v>8.1443660468323653</v>
       </c>
       <c r="AA10">
         <f t="shared" si="2"/>
-        <v>66.790686315789472</v>
+        <v>13.544366046832366</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.35">
@@ -1301,35 +1289,35 @@
         <v>90</v>
       </c>
       <c r="I11">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J11">
-        <v>37.799999999999997</v>
+        <v>25.072445424753251</v>
       </c>
       <c r="K11">
         <v>68.015751583500688</v>
       </c>
       <c r="L11">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M11">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N11">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O11">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P11">
         <v>71.764597894736838</v>
       </c>
       <c r="Q11">
-        <v>9.36</v>
+        <v>1</v>
       </c>
       <c r="R11">
         <f t="shared" si="0"/>
-        <v>67.711528421052634</v>
+        <v>14.360374222817502</v>
       </c>
       <c r="S11" t="s">
         <v>70</v>
@@ -1348,11 +1336,11 @@
       </c>
       <c r="Z11">
         <f t="shared" si="1"/>
-        <v>10.111528421052633</v>
+        <v>8.9603742228175012</v>
       </c>
       <c r="AA11">
         <f t="shared" si="2"/>
-        <v>67.711528421052634</v>
+        <v>14.360374222817502</v>
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.35">
@@ -1381,35 +1369,35 @@
         <v>90</v>
       </c>
       <c r="I12">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J12">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K12">
         <v>68.015751583500688</v>
       </c>
       <c r="L12">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M12">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N12">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O12">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P12">
         <v>69.737381052631576</v>
       </c>
       <c r="Q12">
-        <v>9.36</v>
+        <v>1</v>
       </c>
       <c r="R12">
         <f t="shared" si="0"/>
-        <v>67.541002105263161</v>
+        <v>14.209261597635066</v>
       </c>
       <c r="S12" t="s">
         <v>70</v>
@@ -1428,11 +1416,11 @@
       </c>
       <c r="Z12">
         <f t="shared" si="1"/>
-        <v>9.9410021052631592</v>
+        <v>8.8092615976350661</v>
       </c>
       <c r="AA12">
         <f t="shared" si="2"/>
-        <v>67.541002105263161</v>
+        <v>14.209261597635066</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.35">
@@ -1461,35 +1449,35 @@
         <v>90</v>
       </c>
       <c r="I13">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J13">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K13">
         <v>68.015751583500688</v>
       </c>
       <c r="L13">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M13">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N13">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O13">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P13">
         <v>70.56</v>
       </c>
       <c r="Q13">
-        <v>9.36</v>
+        <v>1</v>
       </c>
       <c r="R13">
         <f t="shared" si="0"/>
-        <v>71.475385263157904</v>
+        <v>8.1871969308975281</v>
       </c>
       <c r="S13" t="s">
         <v>70</v>
@@ -1504,15 +1492,15 @@
         <v>10171</v>
       </c>
       <c r="Y13">
-        <v>16368.642888065227</v>
+        <v>3710.444477974399</v>
       </c>
       <c r="Z13">
         <f t="shared" si="1"/>
-        <v>13.875385263157895</v>
+        <v>2.7871969308975273</v>
       </c>
       <c r="AA13">
         <f t="shared" si="2"/>
-        <v>71.475385263157904</v>
+        <v>8.1871969308975281</v>
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.35">
@@ -1541,35 +1529,35 @@
         <v>90</v>
       </c>
       <c r="I14">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J14">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K14">
         <v>68.015751583500688</v>
       </c>
       <c r="L14">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M14">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N14">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O14">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P14">
         <v>66.790686315789472</v>
       </c>
       <c r="Q14">
-        <v>9.36</v>
+        <v>1</v>
       </c>
       <c r="R14">
         <f t="shared" si="0"/>
-        <v>70.291250526315793</v>
+        <v>6.4181490433991044</v>
       </c>
       <c r="S14" t="s">
         <v>70</v>
@@ -1584,15 +1572,15 @@
         <v>9303</v>
       </c>
       <c r="Y14">
-        <v>14971.731863894485</v>
+        <v>1355.4067364083271</v>
       </c>
       <c r="Z14">
         <f t="shared" si="1"/>
-        <v>12.691250526315789</v>
+        <v>1.0181490433991043</v>
       </c>
       <c r="AA14">
         <f t="shared" si="2"/>
-        <v>70.291250526315793</v>
+        <v>6.4181490433991044</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.35">
@@ -1621,35 +1609,35 @@
         <v>90</v>
       </c>
       <c r="I15">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J15">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K15">
         <v>68.015751583500688</v>
       </c>
       <c r="L15">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M15">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N15">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O15">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P15">
         <v>69.650954303405584</v>
       </c>
       <c r="Q15">
-        <v>9.36</v>
+        <v>1</v>
       </c>
       <c r="R15">
         <f t="shared" si="0"/>
-        <v>71.214821052631578</v>
+        <v>6.0724198318715077</v>
       </c>
       <c r="S15" t="s">
         <v>70</v>
@@ -1664,15 +1652,15 @@
         <v>9980</v>
       </c>
       <c r="Y15">
-        <v>16061.258088967748</v>
+        <v>895.15614214051311</v>
       </c>
       <c r="Z15">
         <f t="shared" si="1"/>
-        <v>13.61482105263158</v>
+        <v>0.67241983187150756</v>
       </c>
       <c r="AA15">
         <f t="shared" si="2"/>
-        <v>71.214821052631578</v>
+        <v>6.0724198318715077</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.35">
@@ -1701,35 +1689,35 @@
         <v>90</v>
       </c>
       <c r="I16">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J16">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K16">
         <v>68.015751583500688</v>
       </c>
       <c r="L16">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M16">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N16">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O16">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P16">
         <v>69.929734736842107</v>
       </c>
       <c r="Q16">
-        <v>9.36</v>
+        <v>1</v>
       </c>
       <c r="R16">
         <f t="shared" si="0"/>
-        <v>68.821995789473689</v>
+        <v>15.344419638005499</v>
       </c>
       <c r="S16" t="s">
         <v>70</v>
@@ -1748,11 +1736,11 @@
       </c>
       <c r="Z16">
         <f t="shared" si="1"/>
-        <v>11.221995789473684</v>
+        <v>9.944419638005499</v>
       </c>
       <c r="AA16">
         <f t="shared" si="2"/>
-        <v>68.821995789473689</v>
+        <v>15.344419638005499</v>
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.35">
@@ -1781,35 +1769,35 @@
         <v>90</v>
       </c>
       <c r="I17">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J17">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K17">
         <v>67.958745558473652</v>
       </c>
       <c r="L17">
-        <v>72.72</v>
+        <v>67.958745558473652</v>
       </c>
       <c r="M17">
-        <v>72.72</v>
+        <v>67.958745558473652</v>
       </c>
       <c r="N17">
-        <v>72.72</v>
+        <v>67.958745558473652</v>
       </c>
       <c r="O17">
-        <v>72.72</v>
+        <v>67.958745558473652</v>
       </c>
       <c r="P17">
         <v>71.475385263157904</v>
       </c>
       <c r="Q17">
-        <v>9.36</v>
+        <v>1</v>
       </c>
       <c r="R17">
         <f t="shared" si="0"/>
-        <v>67.991191578947365</v>
+        <v>14.608198928116689</v>
       </c>
       <c r="S17" t="s">
         <v>70</v>
@@ -1828,11 +1816,11 @@
       </c>
       <c r="Z17">
         <f t="shared" si="1"/>
-        <v>10.391191578947371</v>
+        <v>9.2081989281166887</v>
       </c>
       <c r="AA17">
         <f t="shared" si="2"/>
-        <v>67.991191578947365</v>
+        <v>14.608198928116689</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.35">
@@ -1861,35 +1849,35 @@
         <v>90</v>
       </c>
       <c r="I18">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J18">
-        <v>37.799999999999997</v>
+        <v>28.599772152949953</v>
       </c>
       <c r="K18">
         <v>68.015751583500688</v>
       </c>
       <c r="L18">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M18">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N18">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O18">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P18">
         <v>71.682745263157898</v>
       </c>
       <c r="Q18">
-        <v>9.36</v>
+        <v>1</v>
       </c>
       <c r="R18">
         <f t="shared" si="0"/>
-        <v>66.640623157894737</v>
+        <v>8.9049813556623505</v>
       </c>
       <c r="S18" t="s">
         <v>70</v>
@@ -1904,15 +1892,15 @@
         <v>6627</v>
       </c>
       <c r="Y18">
-        <v>10665.125987533995</v>
+        <v>4665.9920482664747</v>
       </c>
       <c r="Z18">
         <f t="shared" si="1"/>
-        <v>9.0406231578947374</v>
+        <v>3.5049813556623493</v>
       </c>
       <c r="AA18">
         <f t="shared" si="2"/>
-        <v>66.640623157894737</v>
+        <v>8.9049813556623505</v>
       </c>
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.35">
@@ -1941,35 +1929,35 @@
         <v>90</v>
       </c>
       <c r="I19">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J19">
-        <v>37.799999999999997</v>
+        <v>29.604968491332414</v>
       </c>
       <c r="K19">
         <v>68.015751583500688</v>
       </c>
       <c r="L19">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M19">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N19">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O19">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P19">
         <v>69.650954303405584</v>
       </c>
       <c r="Q19">
-        <v>9.36</v>
+        <v>1</v>
       </c>
       <c r="R19">
         <f t="shared" si="0"/>
-        <v>69.947469473684208</v>
+        <v>6.4475155923877008</v>
       </c>
       <c r="S19" t="s">
         <v>70</v>
@@ -1984,15 +1972,15 @@
         <v>9051</v>
       </c>
       <c r="Y19">
-        <v>14566.17705042556</v>
+        <v>1394.5008342540841</v>
       </c>
       <c r="Z19">
         <f t="shared" si="1"/>
-        <v>12.347469473684212</v>
+        <v>1.0475155923877004</v>
       </c>
       <c r="AA19">
         <f t="shared" si="2"/>
-        <v>69.947469473684208</v>
+        <v>6.4475155923877008</v>
       </c>
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.35">
@@ -2021,35 +2009,35 @@
         <v>90</v>
       </c>
       <c r="I20">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J20">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K20">
         <v>68.015751583500688</v>
       </c>
       <c r="L20">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M20">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N20">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O20">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P20">
         <v>69.650954303405584</v>
       </c>
       <c r="Q20">
-        <v>9.36</v>
+        <v>1</v>
       </c>
       <c r="R20">
         <f t="shared" si="0"/>
-        <v>71.764597894736838</v>
+        <v>17.952019098153549</v>
       </c>
       <c r="S20" t="s">
         <v>70</v>
@@ -2068,11 +2056,11 @@
       </c>
       <c r="Z20">
         <f t="shared" si="1"/>
-        <v>14.164597894736842</v>
+        <v>12.552019098153547</v>
       </c>
       <c r="AA20">
         <f t="shared" si="2"/>
-        <v>71.764597894736838</v>
+        <v>17.952019098153549</v>
       </c>
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.35">
@@ -2101,35 +2089,35 @@
         <v>90</v>
       </c>
       <c r="I21">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J21">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K21">
         <v>68.015751583500688</v>
       </c>
       <c r="L21">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M21">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N21">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O21">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P21">
         <v>69.650954303405584</v>
       </c>
       <c r="Q21">
-        <v>9.36</v>
+        <v>1</v>
       </c>
       <c r="R21">
         <f t="shared" si="0"/>
-        <v>71.764597894736838</v>
+        <v>7.6233472479453335</v>
       </c>
       <c r="S21" t="s">
         <v>70</v>
@@ -2144,15 +2132,15 @@
         <v>10383</v>
       </c>
       <c r="Y21">
-        <v>16709.823921618448</v>
+        <v>2959.8219011032761</v>
       </c>
       <c r="Z21">
         <f t="shared" si="1"/>
-        <v>14.164597894736842</v>
+        <v>2.2233472479453331</v>
       </c>
       <c r="AA21">
         <f t="shared" si="2"/>
-        <v>71.764597894736838</v>
+        <v>7.6233472479453335</v>
       </c>
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.35">
@@ -2181,35 +2169,35 @@
         <v>90</v>
       </c>
       <c r="I22">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J22">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K22">
         <v>68.015751583500688</v>
       </c>
       <c r="L22">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M22">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N22">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O22">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P22">
         <v>70.291250526315793</v>
       </c>
       <c r="Q22">
-        <v>9.36</v>
+        <v>1</v>
       </c>
       <c r="R22">
         <f t="shared" si="0"/>
-        <v>70.56</v>
+        <v>6.48</v>
       </c>
       <c r="S22" t="s">
         <v>70</v>
@@ -2224,15 +2212,15 @@
         <v>9500</v>
       </c>
       <c r="Y22">
-        <v>15288.772729979319</v>
+        <v>1437.745568599609</v>
       </c>
       <c r="Z22">
-        <f t="shared" si="1"/>
-        <v>12.96</v>
+        <f>((($U$4/$Y$22)*Y22)*$T$1)/$U$1</f>
+        <v>1.08</v>
       </c>
       <c r="AA22">
         <f t="shared" si="2"/>
-        <v>70.56</v>
+        <v>6.48</v>
       </c>
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.35">
@@ -2261,35 +2249,35 @@
         <v>90</v>
       </c>
       <c r="I23">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J23">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K23">
         <v>68.015751583500688</v>
       </c>
       <c r="L23">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M23">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N23">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O23">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P23">
         <v>69.650954303405584</v>
       </c>
       <c r="Q23">
-        <v>9.36</v>
+        <v>1</v>
       </c>
       <c r="R23">
         <f t="shared" si="0"/>
-        <v>69.929734736842107</v>
+        <v>8.3414841829733888</v>
       </c>
       <c r="S23" t="s">
         <v>70</v>
@@ -2304,15 +2292,15 @@
         <v>9038</v>
       </c>
       <c r="Y23">
-        <v>14545.255571952957</v>
+        <v>3915.8387492368802</v>
       </c>
       <c r="Z23">
         <f t="shared" si="1"/>
-        <v>12.329734736842108</v>
+        <v>2.941484182973388</v>
       </c>
       <c r="AA23">
         <f t="shared" si="2"/>
-        <v>69.929734736842107</v>
+        <v>8.3414841829733888</v>
       </c>
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.35">
@@ -2341,35 +2329,35 @@
         <v>90</v>
       </c>
       <c r="I24">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J24">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K24">
         <v>68.015751583500688</v>
       </c>
       <c r="L24">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M24">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N24">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O24">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P24">
         <v>69.650954303405584</v>
       </c>
       <c r="Q24">
-        <v>9.36</v>
+        <v>1</v>
       </c>
       <c r="R24">
         <f t="shared" si="0"/>
-        <v>71.682745263157898</v>
+        <v>5.4</v>
       </c>
       <c r="S24" t="s">
         <v>70</v>
@@ -2384,15 +2372,15 @@
         <v>10323</v>
       </c>
       <c r="Y24">
-        <v>16613.263251744895</v>
+        <v>0</v>
       </c>
       <c r="Z24">
         <f t="shared" si="1"/>
-        <v>14.082745263157895</v>
+        <v>0</v>
       </c>
       <c r="AA24">
         <f t="shared" si="2"/>
-        <v>71.682745263157898</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.35">
@@ -2421,35 +2409,35 @@
         <v>90</v>
       </c>
       <c r="I25">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J25">
-        <v>37.799999999999997</v>
+        <v>33.046222524758605</v>
       </c>
       <c r="K25">
         <v>68.015751583500688</v>
       </c>
       <c r="L25">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M25">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N25">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O25">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P25">
         <v>71.214821052631578</v>
       </c>
       <c r="Q25">
-        <v>9.36</v>
+        <v>1</v>
       </c>
       <c r="R25">
         <f>AVERAGE(R8:R24)</f>
-        <v>69.650954303405584</v>
+        <v>9.8454816732599308</v>
       </c>
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.35">
@@ -2478,31 +2466,35 @@
         <v>90</v>
       </c>
       <c r="I26">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J26">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K26">
         <v>68.015751583500688</v>
       </c>
       <c r="L26">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M26">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N26">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O26">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P26">
         <v>68.821995789473689</v>
       </c>
       <c r="Q26">
-        <v>9.36</v>
+        <v>1</v>
+      </c>
+      <c r="Y26">
+        <f>7.8/Y22</f>
+        <v>5.4251601746179235E-3</v>
       </c>
     </row>
     <row r="27" spans="1:27" x14ac:dyDescent="0.35">
@@ -2531,34 +2523,37 @@
         <v>90</v>
       </c>
       <c r="I27">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J27">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K27">
         <v>68.015751583500688</v>
       </c>
       <c r="L27">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M27">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N27">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O27">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P27">
         <v>69.650954303405584</v>
       </c>
       <c r="Q27">
-        <v>9.36</v>
+        <v>1</v>
       </c>
       <c r="U27">
-        <v>964.8646999038657</v>
+        <v>3681.0367786032052</v>
+      </c>
+      <c r="Y27">
+        <v>1000</v>
       </c>
     </row>
     <row r="28" spans="1:27" x14ac:dyDescent="0.35">
@@ -2587,34 +2582,38 @@
         <v>90</v>
       </c>
       <c r="I28">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J28">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K28">
         <v>68.015751583500688</v>
       </c>
       <c r="L28">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M28">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N28">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O28">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P28">
         <v>69.650954303405584</v>
       </c>
       <c r="Q28">
-        <v>9.36</v>
+        <v>1</v>
       </c>
       <c r="U28">
-        <v>532.10982214783257</v>
+        <v>599.30727457358682</v>
+      </c>
+      <c r="Y28">
+        <f>Y27*Y26</f>
+        <v>5.4251601746179237</v>
       </c>
     </row>
     <row r="29" spans="1:27" x14ac:dyDescent="0.35">
@@ -2643,31 +2642,31 @@
         <v>90</v>
       </c>
       <c r="I29">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J29">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K29">
         <v>68.015751583500688</v>
       </c>
       <c r="L29">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M29">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N29">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O29">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P29">
         <v>69.650954303405584</v>
       </c>
       <c r="Q29">
-        <v>9.36</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:27" x14ac:dyDescent="0.35">
@@ -2696,31 +2695,31 @@
         <v>90</v>
       </c>
       <c r="I30">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J30">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K30">
         <v>68.015751583500688</v>
       </c>
       <c r="L30">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M30">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N30">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O30">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P30">
         <v>69.650954303405584</v>
       </c>
       <c r="Q30">
-        <v>9.36</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:27" x14ac:dyDescent="0.35">
@@ -2749,39 +2748,39 @@
         <v>90</v>
       </c>
       <c r="I31">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J31">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K31">
         <v>68.015751583500688</v>
       </c>
       <c r="L31">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M31">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N31">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O31">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P31">
         <v>69.650954303405584</v>
       </c>
       <c r="Q31">
-        <v>9.36</v>
+        <v>1</v>
       </c>
       <c r="S31">
-        <f>(K32+K17)/2</f>
-        <v>68.015751583500688</v>
+        <f>(Q36+Q22+Q13+Q12+Q9+Q4)/6</f>
+        <v>1</v>
       </c>
       <c r="U31">
         <f>SUM(U27:U29)</f>
-        <v>1496.9745220516984</v>
+        <v>4280.3440531767919</v>
       </c>
     </row>
     <row r="32" spans="1:27" x14ac:dyDescent="0.35">
@@ -2810,31 +2809,31 @@
         <v>90</v>
       </c>
       <c r="I32">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J32">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K32">
         <v>68.072757608527724</v>
       </c>
       <c r="L32">
-        <v>72.72</v>
+        <v>68.072757608527724</v>
       </c>
       <c r="M32">
-        <v>72.72</v>
+        <v>68.072757608527724</v>
       </c>
       <c r="N32">
-        <v>72.72</v>
+        <v>68.072757608527724</v>
       </c>
       <c r="O32">
-        <v>72.72</v>
+        <v>68.072757608527724</v>
       </c>
       <c r="P32">
         <v>67.991191578947365</v>
       </c>
       <c r="Q32">
-        <v>9.36</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.35">
@@ -2863,31 +2862,31 @@
         <v>90</v>
       </c>
       <c r="I33">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J33">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K33">
         <v>68.015751583500688</v>
       </c>
       <c r="L33">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M33">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N33">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O33">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P33">
         <v>69.650954303405584</v>
       </c>
       <c r="Q33">
-        <v>9.36</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.35">
@@ -2916,31 +2915,31 @@
         <v>90</v>
       </c>
       <c r="I34">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J34">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K34">
         <v>68.015751583500688</v>
       </c>
       <c r="L34">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M34">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N34">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O34">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P34">
         <v>69.650954303405584</v>
       </c>
       <c r="Q34">
-        <v>9.36</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.35">
@@ -2969,31 +2968,31 @@
         <v>90</v>
       </c>
       <c r="I35">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J35">
-        <v>37.799999999999997</v>
+        <v>35.374900727604761</v>
       </c>
       <c r="K35">
         <v>68.015751583500688</v>
       </c>
       <c r="L35">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M35">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N35">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O35">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P35">
         <v>66.640623157894737</v>
       </c>
       <c r="Q35">
-        <v>9.36</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.35">
@@ -3022,31 +3021,31 @@
         <v>90</v>
       </c>
       <c r="I36">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J36">
-        <v>37.799999999999997</v>
+        <v>30.423920107841273</v>
       </c>
       <c r="K36">
         <v>68.015751583500688</v>
       </c>
       <c r="L36">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M36">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N36">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O36">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P36">
         <v>69.947469473684208</v>
       </c>
       <c r="Q36">
-        <v>9.36</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.35">
@@ -3075,31 +3074,31 @@
         <v>90</v>
       </c>
       <c r="I37">
-        <v>37.799999999999997</v>
+        <v>19.276703276025685</v>
       </c>
       <c r="J37">
-        <v>37.799999999999997</v>
+        <v>30.845211325648673</v>
       </c>
       <c r="K37">
         <v>68.015751583500688</v>
       </c>
       <c r="L37">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="M37">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="N37">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="O37">
-        <v>72.72</v>
+        <v>68.015751583500688</v>
       </c>
       <c r="P37">
         <v>69.650954303405584</v>
       </c>
       <c r="Q37">
-        <v>9.36</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update LNG import emissions from NO
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
+++ b/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD679743-7103-470C-84DC-12B613816F5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3F39453-DFD2-43C1-BC1A-E59EFFC80406}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BAA9D55F-0FEB-4558-AFDF-92239B956412}"/>
   </bookViews>
@@ -737,7 +737,7 @@
         <v>69.650954303405584</v>
       </c>
       <c r="Q2">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
       <c r="S2">
         <f>U5-U4</f>
@@ -802,7 +802,7 @@
         <v>69.650954303405584</v>
       </c>
       <c r="Q3">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.35">
@@ -855,7 +855,7 @@
         <v>70.201212631578954</v>
       </c>
       <c r="Q4">
-        <v>1</v>
+        <v>6.5604478724514799</v>
       </c>
       <c r="U4">
         <v>0.3</v>
@@ -911,7 +911,7 @@
         <v>69.650954303405584</v>
       </c>
       <c r="Q5">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
       <c r="U5">
         <v>1.8</v>
@@ -967,7 +967,7 @@
         <v>69.650954303405584</v>
       </c>
       <c r="Q6">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.35">
@@ -1020,7 +1020,7 @@
         <v>67.541002105263161</v>
       </c>
       <c r="Q7">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.35">
@@ -1073,7 +1073,7 @@
         <v>69.650954303405584</v>
       </c>
       <c r="Q8">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
       <c r="R8">
         <f t="shared" ref="R8:R24" si="0">AA8</f>
@@ -1153,7 +1153,7 @@
         <v>69.650954303405584</v>
       </c>
       <c r="Q9">
-        <v>1</v>
+        <v>6.0724198318715077</v>
       </c>
       <c r="R9">
         <f t="shared" si="0"/>
@@ -1233,7 +1233,7 @@
         <v>71.764597894736838</v>
       </c>
       <c r="Q10">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
       <c r="R10">
         <f t="shared" si="0"/>
@@ -1313,7 +1313,7 @@
         <v>71.764597894736838</v>
       </c>
       <c r="Q11">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
       <c r="R11">
         <f t="shared" si="0"/>
@@ -1393,7 +1393,7 @@
         <v>69.737381052631576</v>
       </c>
       <c r="Q12">
-        <v>1</v>
+        <v>6.9190068562697657</v>
       </c>
       <c r="R12">
         <f t="shared" si="0"/>
@@ -1473,7 +1473,7 @@
         <v>70.56</v>
       </c>
       <c r="Q13">
-        <v>1</v>
+        <v>6.48</v>
       </c>
       <c r="R13">
         <f t="shared" si="0"/>
@@ -1553,7 +1553,7 @@
         <v>66.790686315789472</v>
       </c>
       <c r="Q14">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
       <c r="R14">
         <f t="shared" si="0"/>
@@ -1633,7 +1633,7 @@
         <v>69.650954303405584</v>
       </c>
       <c r="Q15">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
       <c r="R15">
         <f t="shared" si="0"/>
@@ -1713,7 +1713,7 @@
         <v>69.929734736842107</v>
       </c>
       <c r="Q16">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
       <c r="R16">
         <f t="shared" si="0"/>
@@ -1793,7 +1793,7 @@
         <v>71.475385263157904</v>
       </c>
       <c r="Q17">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
       <c r="R17">
         <f t="shared" si="0"/>
@@ -1873,7 +1873,7 @@
         <v>71.682745263157898</v>
       </c>
       <c r="Q18">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
       <c r="R18">
         <f t="shared" si="0"/>
@@ -1953,7 +1953,7 @@
         <v>69.650954303405584</v>
       </c>
       <c r="Q19">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
       <c r="R19">
         <f t="shared" si="0"/>
@@ -2033,7 +2033,7 @@
         <v>69.650954303405584</v>
       </c>
       <c r="Q20">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
       <c r="R20">
         <f t="shared" si="0"/>
@@ -2113,7 +2113,7 @@
         <v>69.650954303405584</v>
       </c>
       <c r="Q21">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
       <c r="R21">
         <f t="shared" si="0"/>
@@ -2193,7 +2193,7 @@
         <v>70.291250526315793</v>
       </c>
       <c r="Q22">
-        <v>1</v>
+        <v>6.4181490433991044</v>
       </c>
       <c r="R22">
         <f t="shared" si="0"/>
@@ -2273,7 +2273,7 @@
         <v>69.650954303405584</v>
       </c>
       <c r="Q23">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
       <c r="R23">
         <f t="shared" si="0"/>
@@ -2353,7 +2353,7 @@
         <v>69.650954303405584</v>
       </c>
       <c r="Q24">
-        <v>1</v>
+        <v>5.4</v>
       </c>
       <c r="R24">
         <f t="shared" si="0"/>
@@ -2433,7 +2433,7 @@
         <v>71.214821052631578</v>
       </c>
       <c r="Q25">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
       <c r="R25">
         <f>AVERAGE(R8:R24)</f>
@@ -2490,7 +2490,7 @@
         <v>68.821995789473689</v>
       </c>
       <c r="Q26">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
       <c r="Y26">
         <f>7.8/Y22</f>
@@ -2547,7 +2547,7 @@
         <v>69.650954303405584</v>
       </c>
       <c r="Q27">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
       <c r="U27">
         <v>3681.0367786032052</v>
@@ -2606,7 +2606,7 @@
         <v>69.650954303405584</v>
       </c>
       <c r="Q28">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
       <c r="U28">
         <v>599.30727457358682</v>
@@ -2666,7 +2666,7 @@
         <v>69.650954303405584</v>
       </c>
       <c r="Q29">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
     </row>
     <row r="30" spans="1:27" x14ac:dyDescent="0.35">
@@ -2719,7 +2719,7 @@
         <v>69.650954303405584</v>
       </c>
       <c r="Q30">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
     </row>
     <row r="31" spans="1:27" x14ac:dyDescent="0.35">
@@ -2772,11 +2772,11 @@
         <v>69.650954303405584</v>
       </c>
       <c r="Q31">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
       <c r="S31">
         <f>(Q36+Q22+Q13+Q12+Q9+Q4)/6</f>
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
       <c r="U31">
         <f>SUM(U27:U29)</f>
@@ -2833,7 +2833,7 @@
         <v>67.991191578947365</v>
       </c>
       <c r="Q32">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.35">
@@ -2886,7 +2886,7 @@
         <v>69.650954303405584</v>
       </c>
       <c r="Q33">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.35">
@@ -2939,7 +2939,7 @@
         <v>69.650954303405584</v>
       </c>
       <c r="Q34">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.35">
@@ -2992,7 +2992,7 @@
         <v>66.640623157894737</v>
       </c>
       <c r="Q35">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.35">
@@ -3045,7 +3045,7 @@
         <v>69.947469473684208</v>
       </c>
       <c r="Q36">
-        <v>1</v>
+        <v>6.4475155923877008</v>
       </c>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.35">
@@ -3098,7 +3098,7 @@
         <v>69.650954303405584</v>
       </c>
       <c r="Q37">
-        <v>1</v>
+        <v>6.4829231993965921</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update emission values for DE and NL
so far, DE is a default value for the rest of the European countries.
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
+++ b/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3F39453-DFD2-43C1-BC1A-E59EFFC80406}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C646ED86-FA2B-456B-9BCE-952F78A9F4E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BAA9D55F-0FEB-4558-AFDF-92239B956412}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{BAA9D55F-0FEB-4558-AFDF-92239B956412}"/>
   </bookViews>
   <sheets>
     <sheet name="Emission_Factors_Import" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="71">
   <si>
     <t>AL</t>
   </si>
@@ -740,16 +740,15 @@
         <v>6.4829231993965921</v>
       </c>
       <c r="S2">
-        <f>U5-U4</f>
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="T2">
         <f>S2*T1</f>
-        <v>5400000</v>
+        <v>6120000</v>
       </c>
       <c r="U2">
         <f>T2/U1</f>
-        <v>5.4</v>
+        <v>6.12</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.35">
@@ -1077,7 +1076,7 @@
       </c>
       <c r="R8">
         <f t="shared" ref="R8:R24" si="0">AA8</f>
-        <v>6.5604478724514799</v>
+        <v>7.2804478724514796</v>
       </c>
       <c r="S8" t="s">
         <v>70</v>
@@ -1100,7 +1099,7 @@
       </c>
       <c r="AA8">
         <f>Z8+$U$2</f>
-        <v>6.5604478724514799</v>
+        <v>7.2804478724514796</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.35">
@@ -1157,7 +1156,7 @@
       </c>
       <c r="R9">
         <f t="shared" si="0"/>
-        <v>6.9190068562697657</v>
+        <v>7.6390068562697655</v>
       </c>
       <c r="S9" t="s">
         <v>70</v>
@@ -1180,7 +1179,7 @@
       </c>
       <c r="AA9">
         <f t="shared" ref="AA9:AA24" si="2">Z9+$U$2</f>
-        <v>6.9190068562697657</v>
+        <v>7.6390068562697655</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.35">
@@ -1237,7 +1236,7 @@
       </c>
       <c r="R10">
         <f t="shared" si="0"/>
-        <v>13.544366046832366</v>
+        <v>14.264366046832365</v>
       </c>
       <c r="S10" t="s">
         <v>70</v>
@@ -1260,7 +1259,7 @@
       </c>
       <c r="AA10">
         <f t="shared" si="2"/>
-        <v>13.544366046832366</v>
+        <v>14.264366046832365</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.35">
@@ -1317,7 +1316,7 @@
       </c>
       <c r="R11">
         <f t="shared" si="0"/>
-        <v>14.360374222817502</v>
+        <v>15.0803742228175</v>
       </c>
       <c r="S11" t="s">
         <v>70</v>
@@ -1340,7 +1339,7 @@
       </c>
       <c r="AA11">
         <f t="shared" si="2"/>
-        <v>14.360374222817502</v>
+        <v>15.0803742228175</v>
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.35">
@@ -1397,7 +1396,7 @@
       </c>
       <c r="R12">
         <f t="shared" si="0"/>
-        <v>14.209261597635066</v>
+        <v>14.929261597635065</v>
       </c>
       <c r="S12" t="s">
         <v>70</v>
@@ -1420,7 +1419,7 @@
       </c>
       <c r="AA12">
         <f t="shared" si="2"/>
-        <v>14.209261597635066</v>
+        <v>14.929261597635065</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.35">
@@ -1477,7 +1476,7 @@
       </c>
       <c r="R13">
         <f t="shared" si="0"/>
-        <v>8.1871969308975281</v>
+        <v>8.907196930897527</v>
       </c>
       <c r="S13" t="s">
         <v>70</v>
@@ -1500,7 +1499,7 @@
       </c>
       <c r="AA13">
         <f t="shared" si="2"/>
-        <v>8.1871969308975281</v>
+        <v>8.907196930897527</v>
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.35">
@@ -1557,7 +1556,7 @@
       </c>
       <c r="R14">
         <f t="shared" si="0"/>
-        <v>6.4181490433991044</v>
+        <v>7.1381490433991042</v>
       </c>
       <c r="S14" t="s">
         <v>70</v>
@@ -1580,7 +1579,7 @@
       </c>
       <c r="AA14">
         <f t="shared" si="2"/>
-        <v>6.4181490433991044</v>
+        <v>7.1381490433991042</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.35">
@@ -1637,7 +1636,7 @@
       </c>
       <c r="R15">
         <f t="shared" si="0"/>
-        <v>6.0724198318715077</v>
+        <v>6.7924198318715074</v>
       </c>
       <c r="S15" t="s">
         <v>70</v>
@@ -1660,7 +1659,7 @@
       </c>
       <c r="AA15">
         <f t="shared" si="2"/>
-        <v>6.0724198318715077</v>
+        <v>6.7924198318715074</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.35">
@@ -1717,7 +1716,7 @@
       </c>
       <c r="R16">
         <f t="shared" si="0"/>
-        <v>15.344419638005499</v>
+        <v>16.0644196380055</v>
       </c>
       <c r="S16" t="s">
         <v>70</v>
@@ -1740,7 +1739,7 @@
       </c>
       <c r="AA16">
         <f t="shared" si="2"/>
-        <v>15.344419638005499</v>
+        <v>16.0644196380055</v>
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.35">
@@ -1797,7 +1796,7 @@
       </c>
       <c r="R17">
         <f t="shared" si="0"/>
-        <v>14.608198928116689</v>
+        <v>15.328198928116688</v>
       </c>
       <c r="S17" t="s">
         <v>70</v>
@@ -1820,7 +1819,7 @@
       </c>
       <c r="AA17">
         <f t="shared" si="2"/>
-        <v>14.608198928116689</v>
+        <v>15.328198928116688</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.35">
@@ -1877,7 +1876,7 @@
       </c>
       <c r="R18">
         <f t="shared" si="0"/>
-        <v>8.9049813556623505</v>
+        <v>9.6249813556623494</v>
       </c>
       <c r="S18" t="s">
         <v>70</v>
@@ -1900,7 +1899,7 @@
       </c>
       <c r="AA18">
         <f t="shared" si="2"/>
-        <v>8.9049813556623505</v>
+        <v>9.6249813556623494</v>
       </c>
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.35">
@@ -1957,7 +1956,7 @@
       </c>
       <c r="R19">
         <f t="shared" si="0"/>
-        <v>6.4475155923877008</v>
+        <v>7.1675155923877005</v>
       </c>
       <c r="S19" t="s">
         <v>70</v>
@@ -1980,7 +1979,7 @@
       </c>
       <c r="AA19">
         <f t="shared" si="2"/>
-        <v>6.4475155923877008</v>
+        <v>7.1675155923877005</v>
       </c>
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.35">
@@ -2037,7 +2036,7 @@
       </c>
       <c r="R20">
         <f t="shared" si="0"/>
-        <v>17.952019098153549</v>
+        <v>18.672019098153548</v>
       </c>
       <c r="S20" t="s">
         <v>70</v>
@@ -2060,7 +2059,7 @@
       </c>
       <c r="AA20">
         <f t="shared" si="2"/>
-        <v>17.952019098153549</v>
+        <v>18.672019098153548</v>
       </c>
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.35">
@@ -2117,7 +2116,7 @@
       </c>
       <c r="R21">
         <f t="shared" si="0"/>
-        <v>7.6233472479453335</v>
+        <v>8.3433472479453332</v>
       </c>
       <c r="S21" t="s">
         <v>70</v>
@@ -2140,7 +2139,7 @@
       </c>
       <c r="AA21">
         <f t="shared" si="2"/>
-        <v>7.6233472479453335</v>
+        <v>8.3433472479453332</v>
       </c>
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.35">
@@ -2197,7 +2196,7 @@
       </c>
       <c r="R22">
         <f t="shared" si="0"/>
-        <v>6.48</v>
+        <v>7.2</v>
       </c>
       <c r="S22" t="s">
         <v>70</v>
@@ -2220,7 +2219,7 @@
       </c>
       <c r="AA22">
         <f t="shared" si="2"/>
-        <v>6.48</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.35">
@@ -2277,7 +2276,7 @@
       </c>
       <c r="R23">
         <f t="shared" si="0"/>
-        <v>8.3414841829733888</v>
+        <v>9.0614841829733876</v>
       </c>
       <c r="S23" t="s">
         <v>70</v>
@@ -2300,7 +2299,7 @@
       </c>
       <c r="AA23">
         <f t="shared" si="2"/>
-        <v>8.3414841829733888</v>
+        <v>9.0614841829733876</v>
       </c>
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.35">
@@ -2357,7 +2356,7 @@
       </c>
       <c r="R24">
         <f t="shared" si="0"/>
-        <v>5.4</v>
+        <v>6.12</v>
       </c>
       <c r="S24" t="s">
         <v>70</v>
@@ -2380,7 +2379,7 @@
       </c>
       <c r="AA24">
         <f t="shared" si="2"/>
-        <v>5.4</v>
+        <v>6.12</v>
       </c>
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.35">
@@ -2437,7 +2436,7 @@
       </c>
       <c r="R25">
         <f>AVERAGE(R8:R24)</f>
-        <v>9.8454816732599308</v>
+        <v>10.56548167325993</v>
       </c>
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.35">
@@ -3108,7 +3107,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7AF71E7E-91D4-4876-B8A6-B29CBB1455A1}">
-  <dimension ref="A1:B37"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -3124,7 +3123,7 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -3132,7 +3131,7 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -3140,7 +3139,7 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -3148,7 +3147,7 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
@@ -3156,7 +3155,7 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -3164,7 +3163,7 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -3172,7 +3171,7 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
@@ -3180,7 +3179,7 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
@@ -3188,7 +3187,7 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
@@ -3196,7 +3195,7 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
@@ -3204,7 +3203,7 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
@@ -3212,7 +3211,7 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
@@ -3220,7 +3219,7 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
@@ -3228,7 +3227,7 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
@@ -3236,7 +3235,7 @@
         <v>14</v>
       </c>
       <c r="B16">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
@@ -3244,7 +3243,7 @@
         <v>15</v>
       </c>
       <c r="B17">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
@@ -3252,7 +3251,7 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
@@ -3260,7 +3259,7 @@
         <v>17</v>
       </c>
       <c r="B19">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -3268,7 +3267,7 @@
         <v>18</v>
       </c>
       <c r="B20">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
@@ -3276,7 +3275,7 @@
         <v>19</v>
       </c>
       <c r="B21">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
@@ -3284,7 +3283,7 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>8.64</v>
+        <v>6.12</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
@@ -3292,119 +3291,111 @@
         <v>21</v>
       </c>
       <c r="B23">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B24">
-        <v>7.9200000000000008</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B25">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B26">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B27">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B28">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B29">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B30">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B31">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B32">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B33">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B34">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B35">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B36">
-        <v>23.04</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
-        <v>35</v>
-      </c>
-      <c r="B37">
-        <v>23.04</v>
+        <v>20.52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update LNG import emissions from AU
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
+++ b/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C646ED86-FA2B-456B-9BCE-952F78A9F4E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0D8BA01-C399-450D-B662-D914989CD574}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{BAA9D55F-0FEB-4558-AFDF-92239B956412}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BAA9D55F-0FEB-4558-AFDF-92239B956412}"/>
   </bookViews>
   <sheets>
     <sheet name="Emission_Factors_Import" sheetId="1" r:id="rId1"/>
@@ -249,7 +249,7 @@
     <t>LV_LNG</t>
   </si>
   <si>
-    <t>IM_LNG</t>
+    <t>AU_LNG</t>
   </si>
 </sst>
 </file>
@@ -710,7 +710,7 @@
         <v>74.52</v>
       </c>
       <c r="H2">
-        <v>90</v>
+        <v>67.144178688061956</v>
       </c>
       <c r="I2">
         <v>19.276703276025685</v>
@@ -740,15 +740,16 @@
         <v>6.4829231993965921</v>
       </c>
       <c r="S2">
-        <v>1.7</v>
+        <f>U5-U4</f>
+        <v>15.020000000000001</v>
       </c>
       <c r="T2">
         <f>S2*T1</f>
-        <v>6120000</v>
+        <v>54072000.000000007</v>
       </c>
       <c r="U2">
         <f>T2/U1</f>
-        <v>6.12</v>
+        <v>54.07200000000001</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.35">
@@ -774,7 +775,7 @@
         <v>74.52</v>
       </c>
       <c r="H3">
-        <v>90</v>
+        <v>67.144178688061956</v>
       </c>
       <c r="I3">
         <v>19.276703276025685</v>
@@ -827,7 +828,7 @@
         <v>74.52</v>
       </c>
       <c r="H4">
-        <v>90</v>
+        <v>67.820594928032904</v>
       </c>
       <c r="I4">
         <v>19.276703276025685</v>
@@ -857,7 +858,7 @@
         <v>6.5604478724514799</v>
       </c>
       <c r="U4">
-        <v>0.3</v>
+        <v>3.92</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.35">
@@ -883,7 +884,7 @@
         <v>74.52</v>
       </c>
       <c r="H5">
-        <v>90</v>
+        <v>67.144178688061956</v>
       </c>
       <c r="I5">
         <v>19.276703276025685</v>
@@ -913,7 +914,8 @@
         <v>6.4829231993965921</v>
       </c>
       <c r="U5">
-        <v>1.8</v>
+        <f>11+0.58+7.26+0.1</f>
+        <v>18.940000000000001</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.35">
@@ -939,7 +941,7 @@
         <v>74.52</v>
       </c>
       <c r="H6">
-        <v>90</v>
+        <v>67.144178688061956</v>
       </c>
       <c r="I6">
         <v>19.276703276025685</v>
@@ -967,6 +969,14 @@
       </c>
       <c r="Q6">
         <v>6.4829231993965921</v>
+      </c>
+      <c r="S6">
+        <f>3.7/17000</f>
+        <v>2.1764705882352942E-4</v>
+      </c>
+      <c r="T6">
+        <f>S6*18000</f>
+        <v>3.9176470588235297</v>
       </c>
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.35">
@@ -992,7 +1002,7 @@
         <v>74.52</v>
       </c>
       <c r="H7">
-        <v>90</v>
+        <v>65.126146675805359</v>
       </c>
       <c r="I7">
         <v>19.276703276025685</v>
@@ -1045,7 +1055,7 @@
         <v>74.52</v>
       </c>
       <c r="H8">
-        <v>90</v>
+        <v>67.144178688061956</v>
       </c>
       <c r="I8">
         <v>19.276703276025685</v>
@@ -1076,7 +1086,7 @@
       </c>
       <c r="R8">
         <f t="shared" ref="R8:R24" si="0">AA8</f>
-        <v>7.2804478724514796</v>
+        <v>67.820594928032904</v>
       </c>
       <c r="S8" t="s">
         <v>70</v>
@@ -1088,18 +1098,18 @@
         <v>0</v>
       </c>
       <c r="X8">
-        <v>9237</v>
+        <v>9950</v>
       </c>
       <c r="Y8">
-        <v>1544.841468711073</v>
+        <v>16012.977754030971</v>
       </c>
       <c r="Z8">
         <f>((($U$4/$Y$22)*Y8)*$T$1)/$U$1</f>
-        <v>1.1604478724514795</v>
+        <v>13.748594928032899</v>
       </c>
       <c r="AA8">
         <f>Z8+$U$2</f>
-        <v>7.2804478724514796</v>
+        <v>67.820594928032904</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.35">
@@ -1125,7 +1135,7 @@
         <v>74.52</v>
       </c>
       <c r="H9">
-        <v>90</v>
+        <v>67.144178688061956</v>
       </c>
       <c r="I9">
         <v>19.276703276025685</v>
@@ -1156,7 +1166,7 @@
       </c>
       <c r="R9">
         <f t="shared" si="0"/>
-        <v>7.6390068562697655</v>
+        <v>65.477115832762181</v>
       </c>
       <c r="S9" t="s">
         <v>70</v>
@@ -1168,18 +1178,18 @@
         <v>0</v>
       </c>
       <c r="X9">
-        <v>8897</v>
+        <v>8254</v>
       </c>
       <c r="Y9">
-        <v>2022.171644698406</v>
+        <v>13283.52948560519</v>
       </c>
       <c r="Z9">
         <f t="shared" ref="Z9:Z24" si="1">((($U$4/$Y$22)*Y9)*$T$1)/$U$1</f>
-        <v>1.5190068562697654</v>
+        <v>11.405115832762167</v>
       </c>
       <c r="AA9">
         <f t="shared" ref="AA9:AA24" si="2">Z9+$U$2</f>
-        <v>7.6390068562697655</v>
+        <v>65.477115832762181</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.35">
@@ -1205,7 +1215,7 @@
         <v>74.52</v>
       </c>
       <c r="H10">
-        <v>90</v>
+        <v>69.404101439342028</v>
       </c>
       <c r="I10">
         <v>19.276703276025685</v>
@@ -1236,7 +1246,7 @@
       </c>
       <c r="R10">
         <f t="shared" si="0"/>
-        <v>14.264366046832365</v>
+        <v>64.215561343385886</v>
       </c>
       <c r="S10" t="s">
         <v>70</v>
@@ -1248,18 +1258,18 @@
         <v>0</v>
       </c>
       <c r="X10">
-        <v>6737</v>
+        <v>7341</v>
       </c>
       <c r="Y10">
-        <v>10842.153882302176</v>
+        <v>11814.197959029283</v>
       </c>
       <c r="Z10">
         <f t="shared" si="1"/>
-        <v>8.1443660468323653</v>
+        <v>10.143561343385882</v>
       </c>
       <c r="AA10">
         <f t="shared" si="2"/>
-        <v>14.264366046832365</v>
+        <v>64.215561343385886</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.35">
@@ -1285,7 +1295,7 @@
         <v>74.52</v>
       </c>
       <c r="H11">
-        <v>90</v>
+        <v>69.404101439342028</v>
       </c>
       <c r="I11">
         <v>19.276703276025685</v>
@@ -1316,7 +1326,7 @@
       </c>
       <c r="R11">
         <f t="shared" si="0"/>
-        <v>15.0803742228175</v>
+        <v>65.298867717614812</v>
       </c>
       <c r="S11" t="s">
         <v>70</v>
@@ -1328,18 +1338,18 @@
         <v>0</v>
       </c>
       <c r="X11">
-        <v>7412</v>
+        <v>8125</v>
       </c>
       <c r="Y11">
-        <v>11928.461418379655</v>
+        <v>13075.924045377049</v>
       </c>
       <c r="Z11">
         <f t="shared" si="1"/>
-        <v>8.9603742228175012</v>
+        <v>11.226867717614804</v>
       </c>
       <c r="AA11">
         <f t="shared" si="2"/>
-        <v>15.0803742228175</v>
+        <v>65.298867717614812</v>
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.35">
@@ -1365,7 +1375,7 @@
         <v>74.52</v>
       </c>
       <c r="H12">
-        <v>90</v>
+        <v>65.477115832762181</v>
       </c>
       <c r="I12">
         <v>19.276703276025685</v>
@@ -1396,7 +1406,7 @@
       </c>
       <c r="R12">
         <f t="shared" si="0"/>
-        <v>14.929261597635065</v>
+        <v>65.126146675805359</v>
       </c>
       <c r="S12" t="s">
         <v>70</v>
@@ -1408,18 +1418,18 @@
         <v>0</v>
       </c>
       <c r="X12">
-        <v>7287</v>
+        <v>8000</v>
       </c>
       <c r="Y12">
-        <v>11727.293356143084</v>
+        <v>12874.75598314048</v>
       </c>
       <c r="Z12">
         <f t="shared" si="1"/>
-        <v>8.8092615976350661</v>
+        <v>11.054146675805345</v>
       </c>
       <c r="AA12">
         <f t="shared" si="2"/>
-        <v>14.929261597635065</v>
+        <v>65.126146675805359</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.35">
@@ -1445,7 +1455,7 @@
         <v>74.52</v>
       </c>
       <c r="H13">
-        <v>90</v>
+        <v>68.184000000000012</v>
       </c>
       <c r="I13">
         <v>19.276703276025685</v>
@@ -1476,7 +1486,7 @@
       </c>
       <c r="R13">
         <f t="shared" si="0"/>
-        <v>8.907196930897527</v>
+        <v>69.11116655243319</v>
       </c>
       <c r="S13" t="s">
         <v>70</v>
@@ -1488,18 +1498,18 @@
         <v>0</v>
       </c>
       <c r="X13">
-        <v>10171</v>
+        <v>10884</v>
       </c>
       <c r="Y13">
-        <v>3710.444477974399</v>
+        <v>17516.105515062623</v>
       </c>
       <c r="Z13">
         <f t="shared" si="1"/>
-        <v>2.7871969308975273</v>
+        <v>15.039166552433175</v>
       </c>
       <c r="AA13">
         <f t="shared" si="2"/>
-        <v>8.907196930897527</v>
+        <v>69.11116655243319</v>
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.35">
@@ -1525,7 +1535,7 @@
         <v>74.52</v>
       </c>
       <c r="H14">
-        <v>90</v>
+        <v>64.215561343385886</v>
       </c>
       <c r="I14">
         <v>19.276703276025685</v>
@@ -1556,7 +1566,7 @@
       </c>
       <c r="R14">
         <f t="shared" si="0"/>
-        <v>7.1381490433991042</v>
+        <v>67.911791638108298</v>
       </c>
       <c r="S14" t="s">
         <v>70</v>
@@ -1568,18 +1578,18 @@
         <v>0</v>
       </c>
       <c r="X14">
-        <v>9303</v>
+        <v>10016</v>
       </c>
       <c r="Y14">
-        <v>1355.4067364083271</v>
+        <v>16119.194490891881</v>
       </c>
       <c r="Z14">
         <f t="shared" si="1"/>
-        <v>1.0181490433991043</v>
+        <v>13.839791638108295</v>
       </c>
       <c r="AA14">
         <f t="shared" si="2"/>
-        <v>7.1381490433991042</v>
+        <v>67.911791638108298</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.35">
@@ -1605,7 +1615,7 @@
         <v>74.52</v>
       </c>
       <c r="H15">
-        <v>90</v>
+        <v>67.144178688061956</v>
       </c>
       <c r="I15">
         <v>19.276703276025685</v>
@@ -1636,7 +1646,7 @@
       </c>
       <c r="R15">
         <f t="shared" si="0"/>
-        <v>6.7924198318715074</v>
+        <v>68.847248800548329</v>
       </c>
       <c r="S15" t="s">
         <v>70</v>
@@ -1648,18 +1658,18 @@
         <v>0</v>
       </c>
       <c r="X15">
-        <v>9980</v>
+        <v>10693</v>
       </c>
       <c r="Y15">
-        <v>895.15614214051311</v>
+        <v>17208.720715965144</v>
       </c>
       <c r="Z15">
         <f t="shared" si="1"/>
-        <v>0.67241983187150756</v>
+        <v>14.77524880054832</v>
       </c>
       <c r="AA15">
         <f t="shared" si="2"/>
-        <v>6.7924198318715074</v>
+        <v>68.847248800548329</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.35">
@@ -1685,7 +1695,7 @@
         <v>74.52</v>
       </c>
       <c r="H16">
-        <v>90</v>
+        <v>67.545623029472253</v>
       </c>
       <c r="I16">
         <v>19.276703276025685</v>
@@ -1716,7 +1726,7 @@
       </c>
       <c r="R16">
         <f t="shared" si="0"/>
-        <v>16.0644196380055</v>
+        <v>66.423627141878015</v>
       </c>
       <c r="S16" t="s">
         <v>70</v>
@@ -1728,18 +1738,18 @@
         <v>0</v>
       </c>
       <c r="X16">
-        <v>8226</v>
+        <v>8939</v>
       </c>
       <c r="Y16">
-        <v>13238.467839664198</v>
+        <v>14385.930466661594</v>
       </c>
       <c r="Z16">
         <f t="shared" si="1"/>
-        <v>9.944419638005499</v>
+        <v>12.351627141878</v>
       </c>
       <c r="AA16">
         <f t="shared" si="2"/>
-        <v>16.0644196380055</v>
+        <v>66.423627141878015</v>
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.35">
@@ -1765,7 +1775,7 @@
         <v>74.52</v>
       </c>
       <c r="H17">
-        <v>90</v>
+        <v>65.298867717614812</v>
       </c>
       <c r="I17">
         <v>19.276703276025685</v>
@@ -1796,7 +1806,7 @@
       </c>
       <c r="R17">
         <f t="shared" si="0"/>
-        <v>15.328198928116688</v>
+        <v>65.582130226182329</v>
       </c>
       <c r="S17" t="s">
         <v>70</v>
@@ -1808,18 +1818,18 @@
         <v>0</v>
       </c>
       <c r="X17">
-        <v>7617</v>
+        <v>8330</v>
       </c>
       <c r="Y17">
-        <v>12258.377040447629</v>
+        <v>13405.839667445025</v>
       </c>
       <c r="Z17">
         <f t="shared" si="1"/>
-        <v>9.2081989281166887</v>
+        <v>11.510130226182318</v>
       </c>
       <c r="AA17">
         <f t="shared" si="2"/>
-        <v>15.328198928116688</v>
+        <v>65.582130226182329</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.35">
@@ -1845,7 +1855,7 @@
         <v>74.52</v>
       </c>
       <c r="H18">
-        <v>90</v>
+        <v>69.321195339273487</v>
       </c>
       <c r="I18">
         <v>19.276703276025685</v>
@@ -1876,7 +1886,7 @@
       </c>
       <c r="R18">
         <f t="shared" si="0"/>
-        <v>9.6249813556623494</v>
+        <v>64.214179575051418</v>
       </c>
       <c r="S18" t="s">
         <v>70</v>
@@ -1888,18 +1898,18 @@
         <v>0</v>
       </c>
       <c r="X18">
-        <v>6627</v>
+        <v>7340</v>
       </c>
       <c r="Y18">
-        <v>4665.9920482664747</v>
+        <v>11812.588614531391</v>
       </c>
       <c r="Z18">
         <f t="shared" si="1"/>
-        <v>3.5049813556623493</v>
+        <v>10.142179575051406</v>
       </c>
       <c r="AA18">
         <f t="shared" si="2"/>
-        <v>9.6249813556623494</v>
+        <v>64.214179575051418</v>
       </c>
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.35">
@@ -1925,7 +1935,7 @@
         <v>74.52</v>
       </c>
       <c r="H19">
-        <v>90</v>
+        <v>69.11116655243319</v>
       </c>
       <c r="I19">
         <v>19.276703276025685</v>
@@ -1956,7 +1966,7 @@
       </c>
       <c r="R19">
         <f t="shared" si="0"/>
-        <v>7.1675155923877005</v>
+        <v>67.563586017820441</v>
       </c>
       <c r="S19" t="s">
         <v>70</v>
@@ -1968,18 +1978,18 @@
         <v>0</v>
       </c>
       <c r="X19">
-        <v>9051</v>
+        <v>9764</v>
       </c>
       <c r="Y19">
-        <v>1394.5008342540841</v>
+        <v>15713.639677422956</v>
       </c>
       <c r="Z19">
         <f t="shared" si="1"/>
-        <v>1.0475155923877004</v>
+        <v>13.491586017820426</v>
       </c>
       <c r="AA19">
         <f t="shared" si="2"/>
-        <v>7.1675155923877005</v>
+        <v>67.563586017820441</v>
       </c>
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.35">
@@ -2005,7 +2015,7 @@
         <v>74.52</v>
       </c>
       <c r="H20">
-        <v>90</v>
+        <v>67.144178688061956</v>
       </c>
       <c r="I20">
         <v>19.276703276025685</v>
@@ -2036,7 +2046,7 @@
       </c>
       <c r="R20">
         <f t="shared" si="0"/>
-        <v>18.672019098153548</v>
+        <v>69.404101439342028</v>
       </c>
       <c r="S20" t="s">
         <v>70</v>
@@ -2048,18 +2058,18 @@
         <v>0</v>
       </c>
       <c r="X20">
-        <v>10383</v>
+        <v>11096</v>
       </c>
       <c r="Y20">
-        <v>16709.823921618448</v>
+        <v>17857.286548615844</v>
       </c>
       <c r="Z20">
         <f t="shared" si="1"/>
-        <v>12.552019098153547</v>
+        <v>15.332101439342017</v>
       </c>
       <c r="AA20">
         <f t="shared" si="2"/>
-        <v>18.672019098153548</v>
+        <v>69.404101439342028</v>
       </c>
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.35">
@@ -2085,7 +2095,7 @@
         <v>74.52</v>
       </c>
       <c r="H21">
-        <v>90</v>
+        <v>67.144178688061956</v>
       </c>
       <c r="I21">
         <v>19.276703276025685</v>
@@ -2116,7 +2126,7 @@
       </c>
       <c r="R21">
         <f t="shared" si="0"/>
-        <v>8.3433472479453332</v>
+        <v>69.404101439342028</v>
       </c>
       <c r="S21" t="s">
         <v>70</v>
@@ -2128,18 +2138,18 @@
         <v>0</v>
       </c>
       <c r="X21">
-        <v>10383</v>
+        <v>11096</v>
       </c>
       <c r="Y21">
-        <v>2959.8219011032761</v>
+        <v>17857.286548615844</v>
       </c>
       <c r="Z21">
         <f t="shared" si="1"/>
-        <v>2.2233472479453331</v>
+        <v>15.332101439342017</v>
       </c>
       <c r="AA21">
         <f t="shared" si="2"/>
-        <v>8.3433472479453332</v>
+        <v>69.404101439342028</v>
       </c>
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.35">
@@ -2165,7 +2175,7 @@
         <v>74.52</v>
       </c>
       <c r="H22">
-        <v>90</v>
+        <v>67.911791638108298</v>
       </c>
       <c r="I22">
         <v>19.276703276025685</v>
@@ -2196,7 +2206,7 @@
       </c>
       <c r="R22">
         <f t="shared" si="0"/>
-        <v>7.2</v>
+        <v>68.184000000000012</v>
       </c>
       <c r="S22" t="s">
         <v>70</v>
@@ -2208,18 +2218,18 @@
         <v>0</v>
       </c>
       <c r="X22">
-        <v>9500</v>
+        <v>10213</v>
       </c>
       <c r="Y22">
-        <v>1437.745568599609</v>
+        <v>16436.235356976715</v>
       </c>
       <c r="Z22">
         <f>((($U$4/$Y$22)*Y22)*$T$1)/$U$1</f>
-        <v>1.08</v>
+        <v>14.112</v>
       </c>
       <c r="AA22">
         <f t="shared" si="2"/>
-        <v>7.2</v>
+        <v>68.184000000000012</v>
       </c>
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.35">
@@ -2245,7 +2255,7 @@
         <v>74.52</v>
       </c>
       <c r="H23">
-        <v>90</v>
+        <v>67.144178688061956</v>
       </c>
       <c r="I23">
         <v>19.276703276025685</v>
@@ -2276,7 +2286,7 @@
       </c>
       <c r="R23">
         <f t="shared" si="0"/>
-        <v>9.0614841829733876</v>
+        <v>67.545623029472253</v>
       </c>
       <c r="S23" t="s">
         <v>70</v>
@@ -2288,18 +2298,18 @@
         <v>0</v>
       </c>
       <c r="X23">
-        <v>9038</v>
+        <v>9751</v>
       </c>
       <c r="Y23">
-        <v>3915.8387492368802</v>
+        <v>15692.718198950352</v>
       </c>
       <c r="Z23">
         <f t="shared" si="1"/>
-        <v>2.941484182973388</v>
+        <v>13.473623029472241</v>
       </c>
       <c r="AA23">
         <f t="shared" si="2"/>
-        <v>9.0614841829733876</v>
+        <v>67.545623029472253</v>
       </c>
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.35">
@@ -2325,7 +2335,7 @@
         <v>74.52</v>
       </c>
       <c r="H24">
-        <v>90</v>
+        <v>67.144178688061956</v>
       </c>
       <c r="I24">
         <v>19.276703276025685</v>
@@ -2356,7 +2366,7 @@
       </c>
       <c r="R24">
         <f t="shared" si="0"/>
-        <v>6.12</v>
+        <v>69.321195339273487</v>
       </c>
       <c r="S24" t="s">
         <v>70</v>
@@ -2368,18 +2378,18 @@
         <v>0</v>
       </c>
       <c r="X24">
-        <v>10323</v>
+        <v>11036</v>
       </c>
       <c r="Y24">
-        <v>0</v>
+        <v>17760.725878742291</v>
       </c>
       <c r="Z24">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>15.249195339273475</v>
       </c>
       <c r="AA24">
         <f t="shared" si="2"/>
-        <v>6.12</v>
+        <v>69.321195339273487</v>
       </c>
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.35">
@@ -2405,7 +2415,7 @@
         <v>74.52</v>
       </c>
       <c r="H25">
-        <v>90</v>
+        <v>68.847248800548329</v>
       </c>
       <c r="I25">
         <v>19.276703276025685</v>
@@ -2436,7 +2446,7 @@
       </c>
       <c r="R25">
         <f>AVERAGE(R8:R24)</f>
-        <v>10.56548167325993</v>
+        <v>67.144178688061956</v>
       </c>
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.35">
@@ -2462,7 +2472,7 @@
         <v>74.52</v>
       </c>
       <c r="H26">
-        <v>90</v>
+        <v>66.423627141878015</v>
       </c>
       <c r="I26">
         <v>19.276703276025685</v>
@@ -2493,7 +2503,7 @@
       </c>
       <c r="Y26">
         <f>7.8/Y22</f>
-        <v>5.4251601746179235E-3</v>
+        <v>4.7456122588857436E-4</v>
       </c>
     </row>
     <row r="27" spans="1:27" x14ac:dyDescent="0.35">
@@ -2519,7 +2529,7 @@
         <v>74.52</v>
       </c>
       <c r="H27">
-        <v>90</v>
+        <v>67.144178688061956</v>
       </c>
       <c r="I27">
         <v>19.276703276025685</v>
@@ -2578,7 +2588,7 @@
         <v>74.52</v>
       </c>
       <c r="H28">
-        <v>90</v>
+        <v>67.144178688061956</v>
       </c>
       <c r="I28">
         <v>19.276703276025685</v>
@@ -2612,7 +2622,7 @@
       </c>
       <c r="Y28">
         <f>Y27*Y26</f>
-        <v>5.4251601746179237</v>
+        <v>0.47456122588857436</v>
       </c>
     </row>
     <row r="29" spans="1:27" x14ac:dyDescent="0.35">
@@ -2638,7 +2648,7 @@
         <v>74.52</v>
       </c>
       <c r="H29">
-        <v>90</v>
+        <v>67.144178688061956</v>
       </c>
       <c r="I29">
         <v>19.276703276025685</v>
@@ -2691,7 +2701,7 @@
         <v>74.52</v>
       </c>
       <c r="H30">
-        <v>90</v>
+        <v>67.144178688061956</v>
       </c>
       <c r="I30">
         <v>19.276703276025685</v>
@@ -2744,7 +2754,7 @@
         <v>74.52</v>
       </c>
       <c r="H31">
-        <v>90</v>
+        <v>67.144178688061956</v>
       </c>
       <c r="I31">
         <v>19.276703276025685</v>
@@ -2805,7 +2815,7 @@
         <v>74.52</v>
       </c>
       <c r="H32">
-        <v>90</v>
+        <v>65.582130226182329</v>
       </c>
       <c r="I32">
         <v>19.276703276025685</v>
@@ -2858,7 +2868,7 @@
         <v>74.52</v>
       </c>
       <c r="H33">
-        <v>90</v>
+        <v>67.144178688061956</v>
       </c>
       <c r="I33">
         <v>19.276703276025685</v>
@@ -2911,7 +2921,7 @@
         <v>74.52</v>
       </c>
       <c r="H34">
-        <v>90</v>
+        <v>67.144178688061956</v>
       </c>
       <c r="I34">
         <v>19.276703276025685</v>
@@ -2964,7 +2974,7 @@
         <v>74.52</v>
       </c>
       <c r="H35">
-        <v>90</v>
+        <v>64.214179575051418</v>
       </c>
       <c r="I35">
         <v>19.276703276025685</v>
@@ -3017,7 +3027,7 @@
         <v>74.52</v>
       </c>
       <c r="H36">
-        <v>90</v>
+        <v>67.563586017820441</v>
       </c>
       <c r="I36">
         <v>19.276703276025685</v>
@@ -3070,7 +3080,7 @@
         <v>74.52</v>
       </c>
       <c r="H37">
-        <v>90</v>
+        <v>67.144178688061956</v>
       </c>
       <c r="I37">
         <v>19.276703276025685</v>

</xml_diff>

<commit_message>
fix bug in Australian emission factor calculation
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
+++ b/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0D8BA01-C399-450D-B662-D914989CD574}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C5CBCE0-5DFC-41CA-BBBC-B24BB823D1DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BAA9D55F-0FEB-4558-AFDF-92239B956412}"/>
   </bookViews>
@@ -710,7 +710,7 @@
         <v>74.52</v>
       </c>
       <c r="H2">
-        <v>67.144178688061956</v>
+        <v>81.256178688061908</v>
       </c>
       <c r="I2">
         <v>19.276703276025685</v>
@@ -741,15 +741,15 @@
       </c>
       <c r="S2">
         <f>U5-U4</f>
-        <v>15.020000000000001</v>
+        <v>18.939999999999998</v>
       </c>
       <c r="T2">
         <f>S2*T1</f>
-        <v>54072000.000000007</v>
+        <v>68183999.999999985</v>
       </c>
       <c r="U2">
         <f>T2/U1</f>
-        <v>54.07200000000001</v>
+        <v>68.183999999999983</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.35">
@@ -775,7 +775,7 @@
         <v>74.52</v>
       </c>
       <c r="H3">
-        <v>67.144178688061956</v>
+        <v>81.256178688061908</v>
       </c>
       <c r="I3">
         <v>19.276703276025685</v>
@@ -828,7 +828,7 @@
         <v>74.52</v>
       </c>
       <c r="H4">
-        <v>67.820594928032904</v>
+        <v>81.932594928032884</v>
       </c>
       <c r="I4">
         <v>19.276703276025685</v>
@@ -884,7 +884,7 @@
         <v>74.52</v>
       </c>
       <c r="H5">
-        <v>67.144178688061956</v>
+        <v>81.256178688061908</v>
       </c>
       <c r="I5">
         <v>19.276703276025685</v>
@@ -914,8 +914,8 @@
         <v>6.4829231993965921</v>
       </c>
       <c r="U5">
-        <f>11+0.58+7.26+0.1</f>
-        <v>18.940000000000001</v>
+        <f>11+0.58+7.26+0.1+3.92</f>
+        <v>22.86</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.35">
@@ -941,7 +941,7 @@
         <v>74.52</v>
       </c>
       <c r="H6">
-        <v>67.144178688061956</v>
+        <v>81.256178688061908</v>
       </c>
       <c r="I6">
         <v>19.276703276025685</v>
@@ -1002,7 +1002,7 @@
         <v>74.52</v>
       </c>
       <c r="H7">
-        <v>65.126146675805359</v>
+        <v>79.238146675805325</v>
       </c>
       <c r="I7">
         <v>19.276703276025685</v>
@@ -1055,7 +1055,7 @@
         <v>74.52</v>
       </c>
       <c r="H8">
-        <v>67.144178688061956</v>
+        <v>81.256178688061908</v>
       </c>
       <c r="I8">
         <v>19.276703276025685</v>
@@ -1086,7 +1086,7 @@
       </c>
       <c r="R8">
         <f t="shared" ref="R8:R24" si="0">AA8</f>
-        <v>67.820594928032904</v>
+        <v>81.932594928032884</v>
       </c>
       <c r="S8" t="s">
         <v>70</v>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="AA8">
         <f>Z8+$U$2</f>
-        <v>67.820594928032904</v>
+        <v>81.932594928032884</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.35">
@@ -1135,7 +1135,7 @@
         <v>74.52</v>
       </c>
       <c r="H9">
-        <v>67.144178688061956</v>
+        <v>81.256178688061908</v>
       </c>
       <c r="I9">
         <v>19.276703276025685</v>
@@ -1166,7 +1166,7 @@
       </c>
       <c r="R9">
         <f t="shared" si="0"/>
-        <v>65.477115832762181</v>
+        <v>79.589115832762147</v>
       </c>
       <c r="S9" t="s">
         <v>70</v>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="AA9">
         <f t="shared" ref="AA9:AA24" si="2">Z9+$U$2</f>
-        <v>65.477115832762181</v>
+        <v>79.589115832762147</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.35">
@@ -1215,7 +1215,7 @@
         <v>74.52</v>
       </c>
       <c r="H10">
-        <v>69.404101439342028</v>
+        <v>83.516101439341995</v>
       </c>
       <c r="I10">
         <v>19.276703276025685</v>
@@ -1246,7 +1246,7 @@
       </c>
       <c r="R10">
         <f t="shared" si="0"/>
-        <v>64.215561343385886</v>
+        <v>78.327561343385867</v>
       </c>
       <c r="S10" t="s">
         <v>70</v>
@@ -1269,7 +1269,7 @@
       </c>
       <c r="AA10">
         <f t="shared" si="2"/>
-        <v>64.215561343385886</v>
+        <v>78.327561343385867</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.35">
@@ -1295,7 +1295,7 @@
         <v>74.52</v>
       </c>
       <c r="H11">
-        <v>69.404101439342028</v>
+        <v>83.516101439341995</v>
       </c>
       <c r="I11">
         <v>19.276703276025685</v>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="R11">
         <f t="shared" si="0"/>
-        <v>65.298867717614812</v>
+        <v>79.410867717614792</v>
       </c>
       <c r="S11" t="s">
         <v>70</v>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="AA11">
         <f t="shared" si="2"/>
-        <v>65.298867717614812</v>
+        <v>79.410867717614792</v>
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.35">
@@ -1375,7 +1375,7 @@
         <v>74.52</v>
       </c>
       <c r="H12">
-        <v>65.477115832762181</v>
+        <v>79.589115832762147</v>
       </c>
       <c r="I12">
         <v>19.276703276025685</v>
@@ -1406,7 +1406,7 @@
       </c>
       <c r="R12">
         <f t="shared" si="0"/>
-        <v>65.126146675805359</v>
+        <v>79.238146675805325</v>
       </c>
       <c r="S12" t="s">
         <v>70</v>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="AA12">
         <f t="shared" si="2"/>
-        <v>65.126146675805359</v>
+        <v>79.238146675805325</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.35">
@@ -1455,7 +1455,7 @@
         <v>74.52</v>
       </c>
       <c r="H13">
-        <v>68.184000000000012</v>
+        <v>82.295999999999978</v>
       </c>
       <c r="I13">
         <v>19.276703276025685</v>
@@ -1486,7 +1486,7 @@
       </c>
       <c r="R13">
         <f t="shared" si="0"/>
-        <v>69.11116655243319</v>
+        <v>83.223166552433156</v>
       </c>
       <c r="S13" t="s">
         <v>70</v>
@@ -1509,7 +1509,7 @@
       </c>
       <c r="AA13">
         <f t="shared" si="2"/>
-        <v>69.11116655243319</v>
+        <v>83.223166552433156</v>
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.35">
@@ -1535,7 +1535,7 @@
         <v>74.52</v>
       </c>
       <c r="H14">
-        <v>64.215561343385886</v>
+        <v>78.327561343385867</v>
       </c>
       <c r="I14">
         <v>19.276703276025685</v>
@@ -1566,7 +1566,7 @@
       </c>
       <c r="R14">
         <f t="shared" si="0"/>
-        <v>67.911791638108298</v>
+        <v>82.023791638108278</v>
       </c>
       <c r="S14" t="s">
         <v>70</v>
@@ -1589,7 +1589,7 @@
       </c>
       <c r="AA14">
         <f t="shared" si="2"/>
-        <v>67.911791638108298</v>
+        <v>82.023791638108278</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.35">
@@ -1615,7 +1615,7 @@
         <v>74.52</v>
       </c>
       <c r="H15">
-        <v>67.144178688061956</v>
+        <v>81.256178688061908</v>
       </c>
       <c r="I15">
         <v>19.276703276025685</v>
@@ -1646,7 +1646,7 @@
       </c>
       <c r="R15">
         <f t="shared" si="0"/>
-        <v>68.847248800548329</v>
+        <v>82.959248800548309</v>
       </c>
       <c r="S15" t="s">
         <v>70</v>
@@ -1669,7 +1669,7 @@
       </c>
       <c r="AA15">
         <f t="shared" si="2"/>
-        <v>68.847248800548329</v>
+        <v>82.959248800548309</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.35">
@@ -1695,7 +1695,7 @@
         <v>74.52</v>
       </c>
       <c r="H16">
-        <v>67.545623029472253</v>
+        <v>81.657623029472219</v>
       </c>
       <c r="I16">
         <v>19.276703276025685</v>
@@ -1726,7 +1726,7 @@
       </c>
       <c r="R16">
         <f t="shared" si="0"/>
-        <v>66.423627141878015</v>
+        <v>80.535627141877981</v>
       </c>
       <c r="S16" t="s">
         <v>70</v>
@@ -1749,7 +1749,7 @@
       </c>
       <c r="AA16">
         <f t="shared" si="2"/>
-        <v>66.423627141878015</v>
+        <v>80.535627141877981</v>
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.35">
@@ -1775,7 +1775,7 @@
         <v>74.52</v>
       </c>
       <c r="H17">
-        <v>65.298867717614812</v>
+        <v>79.410867717614792</v>
       </c>
       <c r="I17">
         <v>19.276703276025685</v>
@@ -1806,7 +1806,7 @@
       </c>
       <c r="R17">
         <f t="shared" si="0"/>
-        <v>65.582130226182329</v>
+        <v>79.694130226182295</v>
       </c>
       <c r="S17" t="s">
         <v>70</v>
@@ -1829,7 +1829,7 @@
       </c>
       <c r="AA17">
         <f t="shared" si="2"/>
-        <v>65.582130226182329</v>
+        <v>79.694130226182295</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.35">
@@ -1855,7 +1855,7 @@
         <v>74.52</v>
       </c>
       <c r="H18">
-        <v>69.321195339273487</v>
+        <v>83.433195339273453</v>
       </c>
       <c r="I18">
         <v>19.276703276025685</v>
@@ -1886,7 +1886,7 @@
       </c>
       <c r="R18">
         <f t="shared" si="0"/>
-        <v>64.214179575051418</v>
+        <v>78.326179575051384</v>
       </c>
       <c r="S18" t="s">
         <v>70</v>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="AA18">
         <f t="shared" si="2"/>
-        <v>64.214179575051418</v>
+        <v>78.326179575051384</v>
       </c>
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.35">
@@ -1935,7 +1935,7 @@
         <v>74.52</v>
       </c>
       <c r="H19">
-        <v>69.11116655243319</v>
+        <v>83.223166552433156</v>
       </c>
       <c r="I19">
         <v>19.276703276025685</v>
@@ -1966,7 +1966,7 @@
       </c>
       <c r="R19">
         <f t="shared" si="0"/>
-        <v>67.563586017820441</v>
+        <v>81.675586017820407</v>
       </c>
       <c r="S19" t="s">
         <v>70</v>
@@ -1989,7 +1989,7 @@
       </c>
       <c r="AA19">
         <f t="shared" si="2"/>
-        <v>67.563586017820441</v>
+        <v>81.675586017820407</v>
       </c>
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.35">
@@ -2015,7 +2015,7 @@
         <v>74.52</v>
       </c>
       <c r="H20">
-        <v>67.144178688061956</v>
+        <v>81.256178688061908</v>
       </c>
       <c r="I20">
         <v>19.276703276025685</v>
@@ -2046,7 +2046,7 @@
       </c>
       <c r="R20">
         <f t="shared" si="0"/>
-        <v>69.404101439342028</v>
+        <v>83.516101439341995</v>
       </c>
       <c r="S20" t="s">
         <v>70</v>
@@ -2069,7 +2069,7 @@
       </c>
       <c r="AA20">
         <f t="shared" si="2"/>
-        <v>69.404101439342028</v>
+        <v>83.516101439341995</v>
       </c>
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.35">
@@ -2095,7 +2095,7 @@
         <v>74.52</v>
       </c>
       <c r="H21">
-        <v>67.144178688061956</v>
+        <v>81.256178688061908</v>
       </c>
       <c r="I21">
         <v>19.276703276025685</v>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="R21">
         <f t="shared" si="0"/>
-        <v>69.404101439342028</v>
+        <v>83.516101439341995</v>
       </c>
       <c r="S21" t="s">
         <v>70</v>
@@ -2149,7 +2149,7 @@
       </c>
       <c r="AA21">
         <f t="shared" si="2"/>
-        <v>69.404101439342028</v>
+        <v>83.516101439341995</v>
       </c>
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.35">
@@ -2175,7 +2175,7 @@
         <v>74.52</v>
       </c>
       <c r="H22">
-        <v>67.911791638108298</v>
+        <v>82.023791638108278</v>
       </c>
       <c r="I22">
         <v>19.276703276025685</v>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="R22">
         <f t="shared" si="0"/>
-        <v>68.184000000000012</v>
+        <v>82.295999999999978</v>
       </c>
       <c r="S22" t="s">
         <v>70</v>
@@ -2229,7 +2229,7 @@
       </c>
       <c r="AA22">
         <f t="shared" si="2"/>
-        <v>68.184000000000012</v>
+        <v>82.295999999999978</v>
       </c>
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.35">
@@ -2255,7 +2255,7 @@
         <v>74.52</v>
       </c>
       <c r="H23">
-        <v>67.144178688061956</v>
+        <v>81.256178688061908</v>
       </c>
       <c r="I23">
         <v>19.276703276025685</v>
@@ -2286,7 +2286,7 @@
       </c>
       <c r="R23">
         <f t="shared" si="0"/>
-        <v>67.545623029472253</v>
+        <v>81.657623029472219</v>
       </c>
       <c r="S23" t="s">
         <v>70</v>
@@ -2309,7 +2309,7 @@
       </c>
       <c r="AA23">
         <f t="shared" si="2"/>
-        <v>67.545623029472253</v>
+        <v>81.657623029472219</v>
       </c>
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.35">
@@ -2335,7 +2335,7 @@
         <v>74.52</v>
       </c>
       <c r="H24">
-        <v>67.144178688061956</v>
+        <v>81.256178688061908</v>
       </c>
       <c r="I24">
         <v>19.276703276025685</v>
@@ -2366,7 +2366,7 @@
       </c>
       <c r="R24">
         <f t="shared" si="0"/>
-        <v>69.321195339273487</v>
+        <v>83.433195339273453</v>
       </c>
       <c r="S24" t="s">
         <v>70</v>
@@ -2389,7 +2389,7 @@
       </c>
       <c r="AA24">
         <f t="shared" si="2"/>
-        <v>69.321195339273487</v>
+        <v>83.433195339273453</v>
       </c>
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.35">
@@ -2415,7 +2415,7 @@
         <v>74.52</v>
       </c>
       <c r="H25">
-        <v>68.847248800548329</v>
+        <v>82.959248800548309</v>
       </c>
       <c r="I25">
         <v>19.276703276025685</v>
@@ -2446,7 +2446,7 @@
       </c>
       <c r="R25">
         <f>AVERAGE(R8:R24)</f>
-        <v>67.144178688061956</v>
+        <v>81.256178688061908</v>
       </c>
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.35">
@@ -2472,7 +2472,7 @@
         <v>74.52</v>
       </c>
       <c r="H26">
-        <v>66.423627141878015</v>
+        <v>80.535627141877981</v>
       </c>
       <c r="I26">
         <v>19.276703276025685</v>
@@ -2529,7 +2529,7 @@
         <v>74.52</v>
       </c>
       <c r="H27">
-        <v>67.144178688061956</v>
+        <v>81.256178688061908</v>
       </c>
       <c r="I27">
         <v>19.276703276025685</v>
@@ -2588,7 +2588,7 @@
         <v>74.52</v>
       </c>
       <c r="H28">
-        <v>67.144178688061956</v>
+        <v>81.256178688061908</v>
       </c>
       <c r="I28">
         <v>19.276703276025685</v>
@@ -2648,7 +2648,7 @@
         <v>74.52</v>
       </c>
       <c r="H29">
-        <v>67.144178688061956</v>
+        <v>81.256178688061908</v>
       </c>
       <c r="I29">
         <v>19.276703276025685</v>
@@ -2701,7 +2701,7 @@
         <v>74.52</v>
       </c>
       <c r="H30">
-        <v>67.144178688061956</v>
+        <v>81.256178688061908</v>
       </c>
       <c r="I30">
         <v>19.276703276025685</v>
@@ -2754,7 +2754,7 @@
         <v>74.52</v>
       </c>
       <c r="H31">
-        <v>67.144178688061956</v>
+        <v>81.256178688061908</v>
       </c>
       <c r="I31">
         <v>19.276703276025685</v>
@@ -2815,7 +2815,7 @@
         <v>74.52</v>
       </c>
       <c r="H32">
-        <v>65.582130226182329</v>
+        <v>79.694130226182295</v>
       </c>
       <c r="I32">
         <v>19.276703276025685</v>
@@ -2868,7 +2868,7 @@
         <v>74.52</v>
       </c>
       <c r="H33">
-        <v>67.144178688061956</v>
+        <v>81.256178688061908</v>
       </c>
       <c r="I33">
         <v>19.276703276025685</v>
@@ -2921,7 +2921,7 @@
         <v>74.52</v>
       </c>
       <c r="H34">
-        <v>67.144178688061956</v>
+        <v>81.256178688061908</v>
       </c>
       <c r="I34">
         <v>19.276703276025685</v>
@@ -2974,7 +2974,7 @@
         <v>74.52</v>
       </c>
       <c r="H35">
-        <v>64.214179575051418</v>
+        <v>78.326179575051384</v>
       </c>
       <c r="I35">
         <v>19.276703276025685</v>
@@ -3027,7 +3027,7 @@
         <v>74.52</v>
       </c>
       <c r="H36">
-        <v>67.563586017820441</v>
+        <v>81.675586017820407</v>
       </c>
       <c r="I36">
         <v>19.276703276025685</v>
@@ -3080,7 +3080,7 @@
         <v>74.52</v>
       </c>
       <c r="H37">
-        <v>67.144178688061956</v>
+        <v>81.256178688061908</v>
       </c>
       <c r="I37">
         <v>19.276703276025685</v>

</xml_diff>

<commit_message>
update LNG import emissions from AF
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
+++ b/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C5CBCE0-5DFC-41CA-BBBC-B24BB823D1DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{224764F7-D697-4C79-A3DA-16661990EC1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BAA9D55F-0FEB-4558-AFDF-92239B956412}"/>
   </bookViews>
@@ -249,7 +249,7 @@
     <t>LV_LNG</t>
   </si>
   <si>
-    <t>AU_LNG</t>
+    <t>AF_LNG</t>
   </si>
 </sst>
 </file>
@@ -707,7 +707,7 @@
         <v>62.637176470588244</v>
       </c>
       <c r="G2">
-        <v>74.52</v>
+        <v>74.521832446706739</v>
       </c>
       <c r="H2">
         <v>81.256178688061908</v>
@@ -741,15 +741,15 @@
       </c>
       <c r="S2">
         <f>U5-U4</f>
-        <v>18.939999999999998</v>
+        <v>18.8</v>
       </c>
       <c r="T2">
         <f>S2*T1</f>
-        <v>68183999.999999985</v>
+        <v>67680000</v>
       </c>
       <c r="U2">
         <f>T2/U1</f>
-        <v>68.183999999999983</v>
+        <v>67.680000000000007</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.35">
@@ -772,7 +772,7 @@
         <v>62.637176470588244</v>
       </c>
       <c r="G3">
-        <v>74.52</v>
+        <v>74.521832446706739</v>
       </c>
       <c r="H3">
         <v>81.256178688061908</v>
@@ -825,7 +825,7 @@
         <v>63.343596330275233</v>
       </c>
       <c r="G4">
-        <v>74.52</v>
+        <v>74.129863370201704</v>
       </c>
       <c r="H4">
         <v>81.932594928032884</v>
@@ -858,7 +858,7 @@
         <v>6.5604478724514799</v>
       </c>
       <c r="U4">
-        <v>3.92</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.35">
@@ -881,7 +881,7 @@
         <v>62.637176470588244</v>
       </c>
       <c r="G5">
-        <v>74.52</v>
+        <v>74.521832446706739</v>
       </c>
       <c r="H5">
         <v>81.256178688061908</v>
@@ -914,8 +914,7 @@
         <v>6.4829231993965921</v>
       </c>
       <c r="U5">
-        <f>11+0.58+7.26+0.1+3.92</f>
-        <v>22.86</v>
+        <v>20.7</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.35">
@@ -938,7 +937,7 @@
         <v>62.637176470588244</v>
       </c>
       <c r="G6">
-        <v>74.52</v>
+        <v>74.521832446706739</v>
       </c>
       <c r="H6">
         <v>81.256178688061908</v>
@@ -969,14 +968,6 @@
       </c>
       <c r="Q6">
         <v>6.4829231993965921</v>
-      </c>
-      <c r="S6">
-        <f>3.7/17000</f>
-        <v>2.1764705882352942E-4</v>
-      </c>
-      <c r="T6">
-        <f>S6*18000</f>
-        <v>3.9176470588235297</v>
       </c>
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.35">
@@ -999,7 +990,7 @@
         <v>60.552770642201835</v>
       </c>
       <c r="G7">
-        <v>74.52</v>
+        <v>75.021392322706575</v>
       </c>
       <c r="H7">
         <v>79.238146675805325</v>
@@ -1052,7 +1043,7 @@
         <v>62.637176470588244</v>
       </c>
       <c r="G8">
-        <v>74.52</v>
+        <v>74.521832446706739</v>
       </c>
       <c r="H8">
         <v>81.256178688061908</v>
@@ -1086,7 +1077,7 @@
       </c>
       <c r="R8">
         <f t="shared" ref="R8:R24" si="0">AA8</f>
-        <v>81.932594928032884</v>
+        <v>74.129863370201704</v>
       </c>
       <c r="S8" t="s">
         <v>70</v>
@@ -1098,18 +1089,18 @@
         <v>0</v>
       </c>
       <c r="X8">
-        <v>9950</v>
+        <v>4348</v>
       </c>
       <c r="Y8">
-        <v>16012.977754030971</v>
+        <v>6997.4298768368508</v>
       </c>
       <c r="Z8">
         <f>((($U$4/$Y$22)*Y8)*$T$1)/$U$1</f>
-        <v>13.748594928032899</v>
+        <v>6.4498633702016912</v>
       </c>
       <c r="AA8">
         <f>Z8+$U$2</f>
-        <v>81.932594928032884</v>
+        <v>74.129863370201704</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.35">
@@ -1132,7 +1123,7 @@
         <v>62.637176470588244</v>
       </c>
       <c r="G9">
-        <v>74.52</v>
+        <v>74.521832446706739</v>
       </c>
       <c r="H9">
         <v>81.256178688061908</v>
@@ -1166,7 +1157,7 @@
       </c>
       <c r="R9">
         <f t="shared" si="0"/>
-        <v>79.589115832762147</v>
+        <v>73.583968770331822</v>
       </c>
       <c r="S9" t="s">
         <v>70</v>
@@ -1178,18 +1169,18 @@
         <v>0</v>
       </c>
       <c r="X9">
-        <v>8254</v>
+        <v>3980</v>
       </c>
       <c r="Y9">
-        <v>13283.52948560519</v>
+        <v>6405.1911016123886</v>
       </c>
       <c r="Z9">
         <f t="shared" ref="Z9:Z24" si="1">((($U$4/$Y$22)*Y9)*$T$1)/$U$1</f>
-        <v>11.405115832762167</v>
+        <v>5.903968770331816</v>
       </c>
       <c r="AA9">
         <f t="shared" ref="AA9:AA24" si="2">Z9+$U$2</f>
-        <v>79.589115832762147</v>
+        <v>73.583968770331822</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.35">
@@ -1212,7 +1203,7 @@
         <v>64.983743119266052</v>
       </c>
       <c r="G10">
-        <v>74.52</v>
+        <v>75.829850357839959</v>
       </c>
       <c r="H10">
         <v>83.516101439341995</v>
@@ -1246,7 +1237,7 @@
       </c>
       <c r="R10">
         <f t="shared" si="0"/>
-        <v>78.327561343385867</v>
+        <v>74.835966167859468</v>
       </c>
       <c r="S10" t="s">
         <v>70</v>
@@ -1258,18 +1249,18 @@
         <v>0</v>
       </c>
       <c r="X10">
-        <v>7341</v>
+        <v>4824</v>
       </c>
       <c r="Y10">
-        <v>11814.197959029283</v>
+        <v>7763.4778578337091</v>
       </c>
       <c r="Z10">
         <f t="shared" si="1"/>
-        <v>10.143561343385882</v>
+        <v>7.155966167859467</v>
       </c>
       <c r="AA10">
         <f t="shared" si="2"/>
-        <v>78.327561343385867</v>
+        <v>74.835966167859468</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.35">
@@ -1292,7 +1283,7 @@
         <v>64.983743119266052</v>
       </c>
       <c r="G11">
-        <v>74.52</v>
+        <v>75.829850357839959</v>
       </c>
       <c r="H11">
         <v>83.516101439341995</v>
@@ -1326,7 +1317,7 @@
       </c>
       <c r="R11">
         <f t="shared" si="0"/>
-        <v>79.410867717614792</v>
+        <v>73.868783344176975</v>
       </c>
       <c r="S11" t="s">
         <v>70</v>
@@ -1338,18 +1329,18 @@
         <v>0</v>
       </c>
       <c r="X11">
-        <v>8125</v>
+        <v>4172</v>
       </c>
       <c r="Y11">
-        <v>13075.924045377049</v>
+        <v>6714.1852452077601</v>
       </c>
       <c r="Z11">
         <f t="shared" si="1"/>
-        <v>11.226867717614804</v>
+        <v>6.1887833441769677</v>
       </c>
       <c r="AA11">
         <f t="shared" si="2"/>
-        <v>79.410867717614792</v>
+        <v>73.868783344176975</v>
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.35">
@@ -1372,7 +1363,7 @@
         <v>60.916293577981648</v>
       </c>
       <c r="G12">
-        <v>74.52</v>
+        <v>73.583968770331822</v>
       </c>
       <c r="H12">
         <v>79.589115832762147</v>
@@ -1406,7 +1397,7 @@
       </c>
       <c r="R12">
         <f t="shared" si="0"/>
-        <v>79.238146675805325</v>
+        <v>75.021392322706575</v>
       </c>
       <c r="S12" t="s">
         <v>70</v>
@@ -1418,18 +1409,18 @@
         <v>0</v>
       </c>
       <c r="X12">
-        <v>8000</v>
+        <v>4949</v>
       </c>
       <c r="Y12">
-        <v>12874.75598314048</v>
+        <v>7964.6459200702793</v>
       </c>
       <c r="Z12">
         <f t="shared" si="1"/>
-        <v>11.054146675805345</v>
+        <v>7.3413923227065707</v>
       </c>
       <c r="AA12">
         <f t="shared" si="2"/>
-        <v>79.238146675805325</v>
+        <v>75.021392322706575</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.35">
@@ -1486,7 +1477,7 @@
       </c>
       <c r="R13">
         <f t="shared" si="0"/>
-        <v>83.223166552433156</v>
+        <v>75.51536759921926</v>
       </c>
       <c r="S13" t="s">
         <v>70</v>
@@ -1498,18 +1489,18 @@
         <v>0</v>
       </c>
       <c r="X13">
-        <v>10884</v>
+        <v>5282</v>
       </c>
       <c r="Y13">
-        <v>17516.105515062623</v>
+        <v>8500.5576378685018</v>
       </c>
       <c r="Z13">
         <f t="shared" si="1"/>
-        <v>15.039166552433175</v>
+        <v>7.835367599219258</v>
       </c>
       <c r="AA13">
         <f t="shared" si="2"/>
-        <v>83.223166552433156</v>
+        <v>75.51536759921926</v>
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.35">
@@ -1532,7 +1523,7 @@
         <v>59.609614678899085</v>
       </c>
       <c r="G14">
-        <v>74.52</v>
+        <v>74.835966167859468</v>
       </c>
       <c r="H14">
         <v>78.327561343385867</v>
@@ -1566,7 +1557,7 @@
       </c>
       <c r="R14">
         <f t="shared" si="0"/>
-        <v>82.023791638108278</v>
+        <v>74.227768379960963</v>
       </c>
       <c r="S14" t="s">
         <v>70</v>
@@ -1578,18 +1569,18 @@
         <v>0</v>
       </c>
       <c r="X14">
-        <v>10016</v>
+        <v>4414</v>
       </c>
       <c r="Y14">
-        <v>16119.194490891881</v>
+        <v>7103.6466136977597</v>
       </c>
       <c r="Z14">
         <f t="shared" si="1"/>
-        <v>13.839791638108295</v>
+        <v>6.5477683799609636</v>
       </c>
       <c r="AA14">
         <f t="shared" si="2"/>
-        <v>82.023791638108278</v>
+        <v>74.227768379960963</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.35">
@@ -1612,7 +1603,7 @@
         <v>62.637176470588244</v>
       </c>
       <c r="G15">
-        <v>74.52</v>
+        <v>74.521832446706739</v>
       </c>
       <c r="H15">
         <v>81.256178688061908</v>
@@ -1646,7 +1637,7 @@
       </c>
       <c r="R15">
         <f t="shared" si="0"/>
-        <v>82.959248800548309</v>
+        <v>75.232036434612894</v>
       </c>
       <c r="S15" t="s">
         <v>70</v>
@@ -1658,18 +1649,18 @@
         <v>0</v>
       </c>
       <c r="X15">
-        <v>10693</v>
+        <v>5091</v>
       </c>
       <c r="Y15">
-        <v>17208.720715965144</v>
+        <v>8193.1728387710227</v>
       </c>
       <c r="Z15">
         <f t="shared" si="1"/>
-        <v>14.77524880054832</v>
+        <v>7.5520364346128828</v>
       </c>
       <c r="AA15">
         <f t="shared" si="2"/>
-        <v>82.959248800548309</v>
+        <v>75.232036434612894</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.35">
@@ -1692,7 +1683,7 @@
         <v>63.05878899082569</v>
       </c>
       <c r="G16">
-        <v>74.52</v>
+        <v>73.834664931685111</v>
       </c>
       <c r="H16">
         <v>81.657623029472219</v>
@@ -1726,7 +1717,7 @@
       </c>
       <c r="R16">
         <f t="shared" si="0"/>
-        <v>80.535627141877981</v>
+        <v>72.70727391021471</v>
       </c>
       <c r="S16" t="s">
         <v>70</v>
@@ -1738,18 +1729,18 @@
         <v>0</v>
       </c>
       <c r="X16">
-        <v>8939</v>
+        <v>3389</v>
       </c>
       <c r="Y16">
-        <v>14385.930466661594</v>
+        <v>5454.0685033578857</v>
       </c>
       <c r="Z16">
         <f t="shared" si="1"/>
-        <v>12.351627141878</v>
+        <v>5.0272739102147046</v>
       </c>
       <c r="AA16">
         <f t="shared" si="2"/>
-        <v>80.535627141877981</v>
+        <v>72.70727391021471</v>
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.35">
@@ -1772,7 +1763,7 @@
         <v>60.62862385321101</v>
       </c>
       <c r="G17">
-        <v>74.52</v>
+        <v>73.868783344176975</v>
       </c>
       <c r="H17">
         <v>79.410867717614792</v>
@@ -1806,7 +1797,7 @@
       </c>
       <c r="R17">
         <f t="shared" si="0"/>
-        <v>79.694130226182295</v>
+        <v>72.662771633051406</v>
       </c>
       <c r="S17" t="s">
         <v>70</v>
@@ -1818,18 +1809,18 @@
         <v>0</v>
       </c>
       <c r="X17">
-        <v>8330</v>
+        <v>3359</v>
       </c>
       <c r="Y17">
-        <v>13405.839667445025</v>
+        <v>5405.7881684211088</v>
       </c>
       <c r="Z17">
         <f t="shared" si="1"/>
-        <v>11.510130226182318</v>
+        <v>4.9827716330513985</v>
       </c>
       <c r="AA17">
         <f t="shared" si="2"/>
-        <v>79.694130226182295</v>
+        <v>72.662771633051406</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.35">
@@ -1852,7 +1843,7 @@
         <v>64.897871559633032</v>
       </c>
       <c r="G18">
-        <v>74.52</v>
+        <v>75.740845803513338</v>
       </c>
       <c r="H18">
         <v>83.433195339273453</v>
@@ -1886,7 +1877,7 @@
       </c>
       <c r="R18">
         <f t="shared" si="0"/>
-        <v>78.326179575051384</v>
+        <v>75.258737800910865</v>
       </c>
       <c r="S18" t="s">
         <v>70</v>
@@ -1898,18 +1889,18 @@
         <v>0</v>
       </c>
       <c r="X18">
-        <v>7340</v>
+        <v>5109</v>
       </c>
       <c r="Y18">
-        <v>11812.588614531391</v>
+        <v>8222.1410397330892</v>
       </c>
       <c r="Z18">
         <f t="shared" si="1"/>
-        <v>10.142179575051406</v>
+        <v>7.578737800910865</v>
       </c>
       <c r="AA18">
         <f t="shared" si="2"/>
-        <v>78.326179575051384</v>
+        <v>75.258737800910865</v>
       </c>
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.35">
@@ -1932,7 +1923,7 @@
         <v>64.680330275229352</v>
       </c>
       <c r="G19">
-        <v>74.52</v>
+        <v>75.51536759921926</v>
       </c>
       <c r="H19">
         <v>83.223166552433156</v>
@@ -1966,7 +1957,7 @@
       </c>
       <c r="R19">
         <f t="shared" si="0"/>
-        <v>81.675586017820407</v>
+        <v>74.072010409889401</v>
       </c>
       <c r="S19" t="s">
         <v>70</v>
@@ -1978,18 +1969,18 @@
         <v>0</v>
       </c>
       <c r="X19">
-        <v>9764</v>
+        <v>4309</v>
       </c>
       <c r="Y19">
-        <v>15713.639677422956</v>
+        <v>6934.6654414190407</v>
       </c>
       <c r="Z19">
         <f t="shared" si="1"/>
-        <v>13.491586017820426</v>
+        <v>6.3920104098893944</v>
       </c>
       <c r="AA19">
         <f t="shared" si="2"/>
-        <v>81.675586017820407</v>
+        <v>74.072010409889401</v>
       </c>
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.35">
@@ -2012,7 +2003,7 @@
         <v>62.637176470588244</v>
       </c>
       <c r="G20">
-        <v>74.52</v>
+        <v>74.521832446706739</v>
       </c>
       <c r="H20">
         <v>81.256178688061908</v>
@@ -2046,7 +2037,7 @@
       </c>
       <c r="R20">
         <f t="shared" si="0"/>
-        <v>83.516101439341995</v>
+        <v>75.829850357839959</v>
       </c>
       <c r="S20" t="s">
         <v>70</v>
@@ -2058,18 +2049,18 @@
         <v>0</v>
       </c>
       <c r="X20">
-        <v>11096</v>
+        <v>5494</v>
       </c>
       <c r="Y20">
-        <v>17857.286548615844</v>
+        <v>8841.7386714217246</v>
       </c>
       <c r="Z20">
         <f t="shared" si="1"/>
-        <v>15.332101439342017</v>
+        <v>8.1498503578399468</v>
       </c>
       <c r="AA20">
         <f t="shared" si="2"/>
-        <v>83.516101439341995</v>
+        <v>75.829850357839959</v>
       </c>
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.35">
@@ -2092,7 +2083,7 @@
         <v>62.637176470588244</v>
       </c>
       <c r="G21">
-        <v>74.52</v>
+        <v>74.521832446706739</v>
       </c>
       <c r="H21">
         <v>81.256178688061908</v>
@@ -2126,7 +2117,7 @@
       </c>
       <c r="R21">
         <f t="shared" si="0"/>
-        <v>83.516101439341995</v>
+        <v>75.829850357839959</v>
       </c>
       <c r="S21" t="s">
         <v>70</v>
@@ -2138,18 +2129,18 @@
         <v>0</v>
       </c>
       <c r="X21">
-        <v>11096</v>
+        <v>5494</v>
       </c>
       <c r="Y21">
-        <v>17857.286548615844</v>
+        <v>8841.7386714217246</v>
       </c>
       <c r="Z21">
         <f t="shared" si="1"/>
-        <v>15.332101439342017</v>
+        <v>8.1498503578399468</v>
       </c>
       <c r="AA21">
         <f t="shared" si="2"/>
-        <v>83.516101439341995</v>
+        <v>75.829850357839959</v>
       </c>
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.35">
@@ -2172,7 +2163,7 @@
         <v>63.442348623853213</v>
       </c>
       <c r="G22">
-        <v>74.52</v>
+        <v>74.227768379960963</v>
       </c>
       <c r="H22">
         <v>82.023791638108278</v>
@@ -2206,7 +2197,7 @@
       </c>
       <c r="R22">
         <f t="shared" si="0"/>
-        <v>82.295999999999978</v>
+        <v>74.52000000000001</v>
       </c>
       <c r="S22" t="s">
         <v>70</v>
@@ -2218,18 +2209,18 @@
         <v>0</v>
       </c>
       <c r="X22">
-        <v>10213</v>
+        <v>4611</v>
       </c>
       <c r="Y22">
-        <v>16436.235356976715</v>
+        <v>7420.687479782594</v>
       </c>
       <c r="Z22">
         <f>((($U$4/$Y$22)*Y22)*$T$1)/$U$1</f>
-        <v>14.112</v>
+        <v>6.84</v>
       </c>
       <c r="AA22">
         <f t="shared" si="2"/>
-        <v>82.295999999999978</v>
+        <v>74.52000000000001</v>
       </c>
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.35">
@@ -2252,7 +2243,7 @@
         <v>62.637176470588244</v>
       </c>
       <c r="G23">
-        <v>74.52</v>
+        <v>74.521832446706739</v>
       </c>
       <c r="H23">
         <v>81.256178688061908</v>
@@ -2286,7 +2277,7 @@
       </c>
       <c r="R23">
         <f t="shared" si="0"/>
-        <v>81.657623029472219</v>
+        <v>73.834664931685111</v>
       </c>
       <c r="S23" t="s">
         <v>70</v>
@@ -2298,18 +2289,18 @@
         <v>0</v>
       </c>
       <c r="X23">
-        <v>9751</v>
+        <v>4149</v>
       </c>
       <c r="Y23">
-        <v>15692.718198950352</v>
+        <v>6677.1703217562308</v>
       </c>
       <c r="Z23">
         <f t="shared" si="1"/>
-        <v>13.473623029472241</v>
+        <v>6.1546649316851001</v>
       </c>
       <c r="AA23">
         <f t="shared" si="2"/>
-        <v>81.657623029472219</v>
+        <v>73.834664931685111</v>
       </c>
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.35">
@@ -2332,7 +2323,7 @@
         <v>62.637176470588244</v>
       </c>
       <c r="G24">
-        <v>74.52</v>
+        <v>74.521832446706739</v>
       </c>
       <c r="H24">
         <v>81.256178688061908</v>
@@ -2366,7 +2357,7 @@
       </c>
       <c r="R24">
         <f t="shared" si="0"/>
-        <v>83.433195339273453</v>
+        <v>75.740845803513338</v>
       </c>
       <c r="S24" t="s">
         <v>70</v>
@@ -2378,18 +2369,18 @@
         <v>0</v>
       </c>
       <c r="X24">
-        <v>11036</v>
+        <v>5434</v>
       </c>
       <c r="Y24">
-        <v>17760.725878742291</v>
+        <v>8745.1780015481709</v>
       </c>
       <c r="Z24">
         <f t="shared" si="1"/>
-        <v>15.249195339273475</v>
+        <v>8.0608458035133381</v>
       </c>
       <c r="AA24">
         <f t="shared" si="2"/>
-        <v>83.433195339273453</v>
+        <v>75.740845803513338</v>
       </c>
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.35">
@@ -2412,7 +2403,7 @@
         <v>64.406972477064215</v>
       </c>
       <c r="G25">
-        <v>74.52</v>
+        <v>75.232036434612894</v>
       </c>
       <c r="H25">
         <v>82.959248800548309</v>
@@ -2446,7 +2437,7 @@
       </c>
       <c r="R25">
         <f>AVERAGE(R8:R24)</f>
-        <v>81.256178688061908</v>
+        <v>74.521832446706739</v>
       </c>
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.35">
@@ -2469,7 +2460,7 @@
         <v>61.896660550458719</v>
       </c>
       <c r="G26">
-        <v>74.52</v>
+        <v>72.70727391021471</v>
       </c>
       <c r="H26">
         <v>80.535627141877981</v>
@@ -2503,7 +2494,7 @@
       </c>
       <c r="Y26">
         <f>7.8/Y22</f>
-        <v>4.7456122588857436E-4</v>
+        <v>1.0511155497722859E-3</v>
       </c>
     </row>
     <row r="27" spans="1:27" x14ac:dyDescent="0.35">
@@ -2526,7 +2517,7 @@
         <v>62.637176470588244</v>
       </c>
       <c r="G27">
-        <v>74.52</v>
+        <v>74.521832446706739</v>
       </c>
       <c r="H27">
         <v>81.256178688061908</v>
@@ -2585,7 +2576,7 @@
         <v>62.637176470588244</v>
       </c>
       <c r="G28">
-        <v>74.52</v>
+        <v>74.521832446706739</v>
       </c>
       <c r="H28">
         <v>81.256178688061908</v>
@@ -2622,7 +2613,7 @@
       </c>
       <c r="Y28">
         <f>Y27*Y26</f>
-        <v>0.47456122588857436</v>
+        <v>1.0511155497722859</v>
       </c>
     </row>
     <row r="29" spans="1:27" x14ac:dyDescent="0.35">
@@ -2645,7 +2636,7 @@
         <v>62.637176470588244</v>
       </c>
       <c r="G29">
-        <v>74.52</v>
+        <v>74.521832446706739</v>
       </c>
       <c r="H29">
         <v>81.256178688061908</v>
@@ -2698,7 +2689,7 @@
         <v>62.637176470588244</v>
       </c>
       <c r="G30">
-        <v>74.52</v>
+        <v>74.521832446706739</v>
       </c>
       <c r="H30">
         <v>81.256178688061908</v>
@@ -2751,7 +2742,7 @@
         <v>62.637176470588244</v>
       </c>
       <c r="G31">
-        <v>74.52</v>
+        <v>74.521832446706739</v>
       </c>
       <c r="H31">
         <v>81.256178688061908</v>
@@ -2812,7 +2803,7 @@
         <v>61.025064220183488</v>
       </c>
       <c r="G32">
-        <v>74.52</v>
+        <v>72.662771633051406</v>
       </c>
       <c r="H32">
         <v>79.694130226182295</v>
@@ -2865,7 +2856,7 @@
         <v>62.637176470588244</v>
       </c>
       <c r="G33">
-        <v>74.52</v>
+        <v>74.521832446706739</v>
       </c>
       <c r="H33">
         <v>81.256178688061908</v>
@@ -2918,7 +2909,7 @@
         <v>62.637176470588244</v>
       </c>
       <c r="G34">
-        <v>74.52</v>
+        <v>74.521832446706739</v>
       </c>
       <c r="H34">
         <v>81.256178688061908</v>
@@ -2971,7 +2962,7 @@
         <v>59.608183486238531</v>
       </c>
       <c r="G35">
-        <v>74.52</v>
+        <v>75.258737800910865</v>
       </c>
       <c r="H35">
         <v>78.326179575051384</v>
@@ -3024,7 +3015,7 @@
         <v>63.077394495412847</v>
       </c>
       <c r="G36">
-        <v>74.52</v>
+        <v>74.072010409889401</v>
       </c>
       <c r="H36">
         <v>81.675586017820407</v>
@@ -3077,7 +3068,7 @@
         <v>62.637176470588244</v>
       </c>
       <c r="G37">
-        <v>74.52</v>
+        <v>74.521832446706739</v>
       </c>
       <c r="H37">
         <v>81.256178688061908</v>

</xml_diff>

<commit_message>
fix bug in Russian emission factor calculation
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
+++ b/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{224764F7-D697-4C79-A3DA-16661990EC1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77D248AE-8677-4F4D-9910-32E4280B226B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BAA9D55F-0FEB-4558-AFDF-92239B956412}"/>
   </bookViews>
@@ -716,7 +716,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J2">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K2">
         <v>68.015751583500688</v>
@@ -740,16 +740,15 @@
         <v>6.4829231993965921</v>
       </c>
       <c r="S2">
-        <f>U5-U4</f>
-        <v>18.8</v>
+        <v>2</v>
       </c>
       <c r="T2">
         <f>S2*T1</f>
-        <v>67680000</v>
+        <v>7200000</v>
       </c>
       <c r="U2">
         <f>T2/U1</f>
-        <v>67.680000000000007</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.35">
@@ -781,7 +780,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J3">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K3">
         <v>68.015751583500688</v>
@@ -834,7 +833,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J4">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K4">
         <v>68.015751583500688</v>
@@ -858,7 +857,7 @@
         <v>6.5604478724514799</v>
       </c>
       <c r="U4">
-        <v>1.9</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.35">
@@ -890,7 +889,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J5">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K5">
         <v>68.015751583500688</v>
@@ -914,7 +913,7 @@
         <v>6.4829231993965921</v>
       </c>
       <c r="U5">
-        <v>20.7</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.35">
@@ -946,7 +945,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J6">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K6">
         <v>68.015751583500688</v>
@@ -999,7 +998,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J7">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K7">
         <v>68.015751583500688</v>
@@ -1052,7 +1051,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J8">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K8">
         <v>68.015751583500688</v>
@@ -1077,7 +1076,7 @@
       </c>
       <c r="R8">
         <f t="shared" ref="R8:R24" si="0">AA8</f>
-        <v>74.129863370201704</v>
+        <v>33.678386467143788</v>
       </c>
       <c r="S8" t="s">
         <v>70</v>
@@ -1096,11 +1095,11 @@
       </c>
       <c r="Z8">
         <f>((($U$4/$Y$22)*Y8)*$T$1)/$U$1</f>
-        <v>6.4498633702016912</v>
+        <v>26.478386467143785</v>
       </c>
       <c r="AA8">
         <f>Z8+$U$2</f>
-        <v>74.129863370201704</v>
+        <v>33.678386467143788</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.35">
@@ -1132,7 +1131,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J9">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K9">
         <v>68.015751583500688</v>
@@ -1157,7 +1156,7 @@
       </c>
       <c r="R9">
         <f t="shared" si="0"/>
-        <v>73.583968770331822</v>
+        <v>31.437345478204293</v>
       </c>
       <c r="S9" t="s">
         <v>70</v>
@@ -1176,11 +1175,11 @@
       </c>
       <c r="Z9">
         <f t="shared" ref="Z9:Z24" si="1">((($U$4/$Y$22)*Y9)*$T$1)/$U$1</f>
-        <v>5.903968770331816</v>
+        <v>24.237345478204293</v>
       </c>
       <c r="AA9">
         <f t="shared" ref="AA9:AA24" si="2">Z9+$U$2</f>
-        <v>73.583968770331822</v>
+        <v>31.437345478204293</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.35">
@@ -1212,7 +1211,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J10">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K10">
         <v>68.015751583500688</v>
@@ -1237,7 +1236,7 @@
       </c>
       <c r="R10">
         <f t="shared" si="0"/>
-        <v>74.835966167859468</v>
+        <v>36.577124268054654</v>
       </c>
       <c r="S10" t="s">
         <v>70</v>
@@ -1256,11 +1255,11 @@
       </c>
       <c r="Z10">
         <f t="shared" si="1"/>
-        <v>7.155966167859467</v>
+        <v>29.377124268054654</v>
       </c>
       <c r="AA10">
         <f t="shared" si="2"/>
-        <v>74.835966167859468</v>
+        <v>36.577124268054654</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.35">
@@ -1317,7 +1316,7 @@
       </c>
       <c r="R11">
         <f t="shared" si="0"/>
-        <v>73.868783344176975</v>
+        <v>32.606584255042293</v>
       </c>
       <c r="S11" t="s">
         <v>70</v>
@@ -1336,11 +1335,11 @@
       </c>
       <c r="Z11">
         <f t="shared" si="1"/>
-        <v>6.1887833441769677</v>
+        <v>25.40658425504229</v>
       </c>
       <c r="AA11">
         <f t="shared" si="2"/>
-        <v>73.868783344176975</v>
+        <v>32.606584255042293</v>
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.35">
@@ -1372,7 +1371,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J12">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K12">
         <v>68.015751583500688</v>
@@ -1397,7 +1396,7 @@
       </c>
       <c r="R12">
         <f t="shared" si="0"/>
-        <v>75.021392322706575</v>
+        <v>37.338347430058562</v>
       </c>
       <c r="S12" t="s">
         <v>70</v>
@@ -1416,11 +1415,11 @@
       </c>
       <c r="Z12">
         <f t="shared" si="1"/>
-        <v>7.3413923227065707</v>
+        <v>30.138347430058559</v>
       </c>
       <c r="AA12">
         <f t="shared" si="2"/>
-        <v>75.021392322706575</v>
+        <v>37.338347430058562</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.35">
@@ -1452,7 +1451,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J13">
-        <v>30.423920107841273</v>
+        <v>35.28</v>
       </c>
       <c r="K13">
         <v>68.015751583500688</v>
@@ -1477,7 +1476,7 @@
       </c>
       <c r="R13">
         <f t="shared" si="0"/>
-        <v>75.51536759921926</v>
+        <v>39.366245933636961</v>
       </c>
       <c r="S13" t="s">
         <v>70</v>
@@ -1496,11 +1495,11 @@
       </c>
       <c r="Z13">
         <f t="shared" si="1"/>
-        <v>7.835367599219258</v>
+        <v>32.166245933636958</v>
       </c>
       <c r="AA13">
         <f t="shared" si="2"/>
-        <v>75.51536759921926</v>
+        <v>39.366245933636961</v>
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.35">
@@ -1532,7 +1531,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J14">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K14">
         <v>68.015751583500688</v>
@@ -1557,7 +1556,7 @@
       </c>
       <c r="R14">
         <f t="shared" si="0"/>
-        <v>74.227768379960963</v>
+        <v>34.080312296681846</v>
       </c>
       <c r="S14" t="s">
         <v>70</v>
@@ -1576,11 +1575,11 @@
       </c>
       <c r="Z14">
         <f t="shared" si="1"/>
-        <v>6.5477683799609636</v>
+        <v>26.880312296681847</v>
       </c>
       <c r="AA14">
         <f t="shared" si="2"/>
-        <v>74.227768379960963</v>
+        <v>34.080312296681846</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.35">
@@ -1612,7 +1611,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J15">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K15">
         <v>68.015751583500688</v>
@@ -1637,7 +1636,7 @@
       </c>
       <c r="R15">
         <f t="shared" si="0"/>
-        <v>75.232036434612894</v>
+        <v>38.203096942094987</v>
       </c>
       <c r="S15" t="s">
         <v>70</v>
@@ -1656,11 +1655,11 @@
       </c>
       <c r="Z15">
         <f t="shared" si="1"/>
-        <v>7.5520364346128828</v>
+        <v>31.003096942094988</v>
       </c>
       <c r="AA15">
         <f t="shared" si="2"/>
-        <v>75.232036434612894</v>
+        <v>38.203096942094987</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.35">
@@ -1692,7 +1691,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J16">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K16">
         <v>68.015751583500688</v>
@@ -1717,7 +1716,7 @@
       </c>
       <c r="R16">
         <f t="shared" si="0"/>
-        <v>72.70727391021471</v>
+        <v>27.838282368249835</v>
       </c>
       <c r="S16" t="s">
         <v>70</v>
@@ -1736,11 +1735,11 @@
       </c>
       <c r="Z16">
         <f t="shared" si="1"/>
-        <v>5.0272739102147046</v>
+        <v>20.638282368249836</v>
       </c>
       <c r="AA16">
         <f t="shared" si="2"/>
-        <v>72.70727391021471</v>
+        <v>27.838282368249835</v>
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.35">
@@ -1772,7 +1771,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J17">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K17">
         <v>67.958745558473652</v>
@@ -1797,7 +1796,7 @@
       </c>
       <c r="R17">
         <f t="shared" si="0"/>
-        <v>72.662771633051406</v>
+        <v>27.655588809368901</v>
       </c>
       <c r="S17" t="s">
         <v>70</v>
@@ -1816,11 +1815,11 @@
       </c>
       <c r="Z17">
         <f t="shared" si="1"/>
-        <v>4.9827716330513985</v>
+        <v>20.455588809368901</v>
       </c>
       <c r="AA17">
         <f t="shared" si="2"/>
-        <v>72.662771633051406</v>
+        <v>27.655588809368901</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.35">
@@ -1877,7 +1876,7 @@
       </c>
       <c r="R18">
         <f t="shared" si="0"/>
-        <v>75.258737800910865</v>
+        <v>38.312713077423552</v>
       </c>
       <c r="S18" t="s">
         <v>70</v>
@@ -1896,11 +1895,11 @@
       </c>
       <c r="Z18">
         <f t="shared" si="1"/>
-        <v>7.578737800910865</v>
+        <v>31.11271307742355</v>
       </c>
       <c r="AA18">
         <f t="shared" si="2"/>
-        <v>75.258737800910865</v>
+        <v>38.312713077423552</v>
       </c>
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.35">
@@ -1957,7 +1956,7 @@
       </c>
       <c r="R19">
         <f t="shared" si="0"/>
-        <v>74.072010409889401</v>
+        <v>33.440884840598571</v>
       </c>
       <c r="S19" t="s">
         <v>70</v>
@@ -1976,11 +1975,11 @@
       </c>
       <c r="Z19">
         <f t="shared" si="1"/>
-        <v>6.3920104098893944</v>
+        <v>26.240884840598568</v>
       </c>
       <c r="AA19">
         <f t="shared" si="2"/>
-        <v>74.072010409889401</v>
+        <v>33.440884840598571</v>
       </c>
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.35">
@@ -2012,7 +2011,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J20">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K20">
         <v>68.015751583500688</v>
@@ -2037,7 +2036,7 @@
       </c>
       <c r="R20">
         <f t="shared" si="0"/>
-        <v>75.829850357839959</v>
+        <v>40.657280416395579</v>
       </c>
       <c r="S20" t="s">
         <v>70</v>
@@ -2056,11 +2055,11 @@
       </c>
       <c r="Z20">
         <f t="shared" si="1"/>
-        <v>8.1498503578399468</v>
+        <v>33.457280416395577</v>
       </c>
       <c r="AA20">
         <f t="shared" si="2"/>
-        <v>75.829850357839959</v>
+        <v>40.657280416395579</v>
       </c>
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.35">
@@ -2092,7 +2091,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J21">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K21">
         <v>68.015751583500688</v>
@@ -2117,7 +2116,7 @@
       </c>
       <c r="R21">
         <f t="shared" si="0"/>
-        <v>75.829850357839959</v>
+        <v>40.657280416395579</v>
       </c>
       <c r="S21" t="s">
         <v>70</v>
@@ -2136,11 +2135,11 @@
       </c>
       <c r="Z21">
         <f t="shared" si="1"/>
-        <v>8.1498503578399468</v>
+        <v>33.457280416395577</v>
       </c>
       <c r="AA21">
         <f t="shared" si="2"/>
-        <v>75.829850357839959</v>
+        <v>40.657280416395579</v>
       </c>
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.35">
@@ -2172,7 +2171,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J22">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K22">
         <v>68.015751583500688</v>
@@ -2197,7 +2196,7 @@
       </c>
       <c r="R22">
         <f t="shared" si="0"/>
-        <v>74.52000000000001</v>
+        <v>35.28</v>
       </c>
       <c r="S22" t="s">
         <v>70</v>
@@ -2216,11 +2215,11 @@
       </c>
       <c r="Z22">
         <f>((($U$4/$Y$22)*Y22)*$T$1)/$U$1</f>
-        <v>6.84</v>
+        <v>28.08</v>
       </c>
       <c r="AA22">
         <f t="shared" si="2"/>
-        <v>74.52000000000001</v>
+        <v>35.28</v>
       </c>
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.35">
@@ -2252,7 +2251,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J23">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K23">
         <v>68.015751583500688</v>
@@ -2277,7 +2276,7 @@
       </c>
       <c r="R23">
         <f t="shared" si="0"/>
-        <v>73.834664931685111</v>
+        <v>32.466519193233573</v>
       </c>
       <c r="S23" t="s">
         <v>70</v>
@@ -2296,11 +2295,11 @@
       </c>
       <c r="Z23">
         <f t="shared" si="1"/>
-        <v>6.1546649316851001</v>
+        <v>25.26651919323357</v>
       </c>
       <c r="AA23">
         <f t="shared" si="2"/>
-        <v>73.834664931685111</v>
+        <v>32.466519193233573</v>
       </c>
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.35">
@@ -2332,7 +2331,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J24">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K24">
         <v>68.015751583500688</v>
@@ -2357,7 +2356,7 @@
       </c>
       <c r="R24">
         <f t="shared" si="0"/>
-        <v>75.740845803513338</v>
+        <v>40.291893298633703</v>
       </c>
       <c r="S24" t="s">
         <v>70</v>
@@ -2376,11 +2375,11 @@
       </c>
       <c r="Z24">
         <f t="shared" si="1"/>
-        <v>8.0608458035133381</v>
+        <v>33.0918932986337</v>
       </c>
       <c r="AA24">
         <f t="shared" si="2"/>
-        <v>75.740845803513338</v>
+        <v>40.291893298633703</v>
       </c>
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.35">
@@ -2437,7 +2436,7 @@
       </c>
       <c r="R25">
         <f>AVERAGE(R8:R24)</f>
-        <v>74.521832446706739</v>
+        <v>35.287522675953916</v>
       </c>
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.35">
@@ -2469,7 +2468,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J26">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K26">
         <v>68.015751583500688</v>
@@ -2526,7 +2525,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J27">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K27">
         <v>68.015751583500688</v>
@@ -2585,7 +2584,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J28">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K28">
         <v>68.015751583500688</v>
@@ -2645,7 +2644,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J29">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K29">
         <v>68.015751583500688</v>
@@ -2698,7 +2697,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J30">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K30">
         <v>68.015751583500688</v>
@@ -2751,7 +2750,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J31">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K31">
         <v>68.015751583500688</v>
@@ -2812,7 +2811,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J32">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K32">
         <v>68.072757608527724</v>
@@ -2865,7 +2864,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J33">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K33">
         <v>68.015751583500688</v>
@@ -2918,7 +2917,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J34">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K34">
         <v>68.015751583500688</v>
@@ -3024,7 +3023,7 @@
         <v>19.276703276025685</v>
       </c>
       <c r="J36">
-        <v>30.423920107841273</v>
+        <v>31.117645806721097</v>
       </c>
       <c r="K36">
         <v>68.015751583500688</v>

</xml_diff>

<commit_message>
update emission values for DK and UK
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
+++ b/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77D248AE-8677-4F4D-9910-32E4280B226B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E37ED7FE-2F3B-4F69-94F5-DF5CB84DEA35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BAA9D55F-0FEB-4558-AFDF-92239B956412}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{BAA9D55F-0FEB-4558-AFDF-92239B956412}"/>
   </bookViews>
   <sheets>
     <sheet name="Emission_Factors_Import" sheetId="1" r:id="rId1"/>
@@ -249,7 +249,7 @@
     <t>LV_LNG</t>
   </si>
   <si>
-    <t>AF_LNG</t>
+    <t>TT_LNG</t>
   </si>
 </sst>
 </file>
@@ -740,15 +740,16 @@
         <v>6.4829231993965921</v>
       </c>
       <c r="S2">
-        <v>2</v>
+        <f>U5-U4</f>
+        <v>16.3</v>
       </c>
       <c r="T2">
         <f>S2*T1</f>
-        <v>7200000</v>
+        <v>58680000</v>
       </c>
       <c r="U2">
         <f>T2/U1</f>
-        <v>7.2</v>
+        <v>58.68</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.35">
@@ -856,8 +857,12 @@
       <c r="Q4">
         <v>6.5604478724514799</v>
       </c>
+      <c r="S4">
+        <f>(2.1/9500)*7900</f>
+        <v>1.7463157894736843</v>
+      </c>
       <c r="U4">
-        <v>7.8</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.35">
@@ -913,7 +918,8 @@
         <v>6.4829231993965921</v>
       </c>
       <c r="U5">
-        <v>7.8</v>
+        <f>16.3+1.75</f>
+        <v>18.05</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.35">
@@ -1076,7 +1082,7 @@
       </c>
       <c r="R8">
         <f t="shared" ref="R8:R24" si="0">AA8</f>
-        <v>33.678386467143788</v>
+        <v>64.58995762711865</v>
       </c>
       <c r="S8" t="s">
         <v>70</v>
@@ -1088,18 +1094,18 @@
         <v>0</v>
       </c>
       <c r="X8">
-        <v>4348</v>
+        <v>3985</v>
       </c>
       <c r="Y8">
-        <v>6997.4298768368508</v>
+        <v>6413.2378241018514</v>
       </c>
       <c r="Z8">
         <f>((($U$4/$Y$22)*Y8)*$T$1)/$U$1</f>
-        <v>26.478386467143785</v>
+        <v>5.9099576271186454</v>
       </c>
       <c r="AA8">
         <f>Z8+$U$2</f>
-        <v>33.678386467143788</v>
+        <v>64.58995762711865</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.35">
@@ -1156,7 +1162,7 @@
       </c>
       <c r="R9">
         <f t="shared" si="0"/>
-        <v>31.437345478204293</v>
+        <v>64.541016949152549</v>
       </c>
       <c r="S9" t="s">
         <v>70</v>
@@ -1168,18 +1174,18 @@
         <v>0</v>
       </c>
       <c r="X9">
-        <v>3980</v>
+        <v>3952</v>
       </c>
       <c r="Y9">
-        <v>6405.1911016123886</v>
+        <v>6360.1294556713965</v>
       </c>
       <c r="Z9">
         <f t="shared" ref="Z9:Z24" si="1">((($U$4/$Y$22)*Y9)*$T$1)/$U$1</f>
-        <v>24.237345478204293</v>
+        <v>5.8610169491525426</v>
       </c>
       <c r="AA9">
         <f t="shared" ref="AA9:AA24" si="2">Z9+$U$2</f>
-        <v>31.437345478204293</v>
+        <v>64.541016949152549</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.35">
@@ -1236,7 +1242,7 @@
       </c>
       <c r="R10">
         <f t="shared" si="0"/>
-        <v>36.577124268054654</v>
+        <v>65.943983050847464</v>
       </c>
       <c r="S10" t="s">
         <v>70</v>
@@ -1248,18 +1254,18 @@
         <v>0</v>
       </c>
       <c r="X10">
-        <v>4824</v>
+        <v>4898</v>
       </c>
       <c r="Y10">
-        <v>7763.4778578337091</v>
+        <v>7882.5693506777588</v>
       </c>
       <c r="Z10">
         <f t="shared" si="1"/>
-        <v>29.377124268054654</v>
+        <v>7.2639830508474574</v>
       </c>
       <c r="AA10">
         <f t="shared" si="2"/>
-        <v>36.577124268054654</v>
+        <v>65.943983050847464</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.35">
@@ -1316,7 +1322,7 @@
       </c>
       <c r="R11">
         <f t="shared" si="0"/>
-        <v>32.606584255042293</v>
+        <v>66.206483050847453</v>
       </c>
       <c r="S11" t="s">
         <v>70</v>
@@ -1328,18 +1334,18 @@
         <v>0</v>
       </c>
       <c r="X11">
-        <v>4172</v>
+        <v>5075</v>
       </c>
       <c r="Y11">
-        <v>6714.1852452077601</v>
+        <v>8167.4233268047419</v>
       </c>
       <c r="Z11">
         <f t="shared" si="1"/>
-        <v>25.40658425504229</v>
+        <v>7.5264830508474594</v>
       </c>
       <c r="AA11">
         <f t="shared" si="2"/>
-        <v>32.606584255042293</v>
+        <v>66.206483050847453</v>
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.35">
@@ -1396,7 +1402,7 @@
       </c>
       <c r="R12">
         <f t="shared" si="0"/>
-        <v>37.338347430058562</v>
+        <v>66.129364406779658</v>
       </c>
       <c r="S12" t="s">
         <v>70</v>
@@ -1408,18 +1414,18 @@
         <v>0</v>
       </c>
       <c r="X12">
-        <v>4949</v>
+        <v>5023</v>
       </c>
       <c r="Y12">
-        <v>7964.6459200702793</v>
+        <v>8083.7374129143291</v>
       </c>
       <c r="Z12">
         <f t="shared" si="1"/>
-        <v>30.138347430058559</v>
+        <v>7.4493644067796625</v>
       </c>
       <c r="AA12">
         <f t="shared" si="2"/>
-        <v>37.338347430058562</v>
+        <v>66.129364406779658</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.35">
@@ -1476,7 +1482,7 @@
       </c>
       <c r="R13">
         <f t="shared" si="0"/>
-        <v>39.366245933636961</v>
+        <v>65.832754237288128</v>
       </c>
       <c r="S13" t="s">
         <v>70</v>
@@ -1488,18 +1494,18 @@
         <v>0</v>
       </c>
       <c r="X13">
-        <v>5282</v>
+        <v>4823</v>
       </c>
       <c r="Y13">
-        <v>8500.5576378685018</v>
+        <v>7761.8685133358167</v>
       </c>
       <c r="Z13">
         <f t="shared" si="1"/>
-        <v>32.166245933636958</v>
+        <v>7.1527542372881356</v>
       </c>
       <c r="AA13">
         <f t="shared" si="2"/>
-        <v>39.366245933636961</v>
+        <v>65.832754237288128</v>
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.35">
@@ -1556,7 +1562,7 @@
       </c>
       <c r="R14">
         <f t="shared" si="0"/>
-        <v>34.080312296681846</v>
+        <v>64.687838983050852</v>
       </c>
       <c r="S14" t="s">
         <v>70</v>
@@ -1568,18 +1574,18 @@
         <v>0</v>
       </c>
       <c r="X14">
-        <v>4414</v>
+        <v>4051</v>
       </c>
       <c r="Y14">
-        <v>7103.6466136977597</v>
+        <v>6519.4545609627603</v>
       </c>
       <c r="Z14">
         <f t="shared" si="1"/>
-        <v>26.880312296681847</v>
+        <v>6.0078389830508483</v>
       </c>
       <c r="AA14">
         <f t="shared" si="2"/>
-        <v>34.080312296681846</v>
+        <v>64.687838983050852</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.35">
@@ -1636,7 +1642,7 @@
       </c>
       <c r="R15">
         <f t="shared" si="0"/>
-        <v>38.203096942094987</v>
+        <v>65.549491525423733</v>
       </c>
       <c r="S15" t="s">
         <v>70</v>
@@ -1648,18 +1654,18 @@
         <v>0</v>
       </c>
       <c r="X15">
-        <v>5091</v>
+        <v>4632</v>
       </c>
       <c r="Y15">
-        <v>8193.1728387710227</v>
+        <v>7454.4837142383376</v>
       </c>
       <c r="Z15">
         <f t="shared" si="1"/>
-        <v>31.003096942094988</v>
+        <v>6.8694915254237285</v>
       </c>
       <c r="AA15">
         <f t="shared" si="2"/>
-        <v>38.203096942094987</v>
+        <v>65.549491525423733</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.35">
@@ -1716,7 +1722,7 @@
       </c>
       <c r="R16">
         <f t="shared" si="0"/>
-        <v>27.838282368249835</v>
+        <v>63.572584745762711</v>
       </c>
       <c r="S16" t="s">
         <v>70</v>
@@ -1728,18 +1734,18 @@
         <v>0</v>
       </c>
       <c r="X16">
-        <v>3389</v>
+        <v>3299</v>
       </c>
       <c r="Y16">
-        <v>5454.0685033578857</v>
+        <v>5309.2274985475551</v>
       </c>
       <c r="Z16">
         <f t="shared" si="1"/>
-        <v>20.638282368249836</v>
+        <v>4.8925847457627123</v>
       </c>
       <c r="AA16">
         <f t="shared" si="2"/>
-        <v>27.838282368249835</v>
+        <v>63.572584745762711</v>
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.35">
@@ -1796,7 +1802,7 @@
       </c>
       <c r="R17">
         <f t="shared" si="0"/>
-        <v>27.655588809368901</v>
+        <v>64.085720338983052</v>
       </c>
       <c r="S17" t="s">
         <v>70</v>
@@ -1808,18 +1814,18 @@
         <v>0</v>
       </c>
       <c r="X17">
-        <v>3359</v>
+        <v>3645</v>
       </c>
       <c r="Y17">
-        <v>5405.7881684211088</v>
+        <v>5866.0606948183813</v>
       </c>
       <c r="Z17">
         <f t="shared" si="1"/>
-        <v>20.455588809368901</v>
+        <v>5.405720338983051</v>
       </c>
       <c r="AA17">
         <f t="shared" si="2"/>
-        <v>27.655588809368901</v>
+        <v>64.085720338983052</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.35">
@@ -1876,7 +1882,7 @@
       </c>
       <c r="R18">
         <f t="shared" si="0"/>
-        <v>38.312713077423552</v>
+        <v>66.172372881355926</v>
       </c>
       <c r="S18" t="s">
         <v>70</v>
@@ -1888,18 +1894,18 @@
         <v>0</v>
       </c>
       <c r="X18">
-        <v>5109</v>
+        <v>5052</v>
       </c>
       <c r="Y18">
-        <v>8222.1410397330892</v>
+        <v>8130.4084033532126</v>
       </c>
       <c r="Z18">
         <f t="shared" si="1"/>
-        <v>31.11271307742355</v>
+        <v>7.4923728813559318</v>
       </c>
       <c r="AA18">
         <f t="shared" si="2"/>
-        <v>38.312713077423552</v>
+        <v>66.172372881355926</v>
       </c>
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.35">
@@ -1956,7 +1962,7 @@
       </c>
       <c r="R19">
         <f t="shared" si="0"/>
-        <v>33.440884840598571</v>
+        <v>64.573644067796607</v>
       </c>
       <c r="S19" t="s">
         <v>70</v>
@@ -1968,18 +1974,18 @@
         <v>0</v>
       </c>
       <c r="X19">
-        <v>4309</v>
+        <v>3974</v>
       </c>
       <c r="Y19">
-        <v>6934.6654414190407</v>
+        <v>6395.5350346250334</v>
       </c>
       <c r="Z19">
         <f t="shared" si="1"/>
-        <v>26.240884840598568</v>
+        <v>5.8936440677966111</v>
       </c>
       <c r="AA19">
         <f t="shared" si="2"/>
-        <v>33.440884840598571</v>
+        <v>64.573644067796607</v>
       </c>
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.35">
@@ -2036,7 +2042,7 @@
       </c>
       <c r="R20">
         <f t="shared" si="0"/>
-        <v>40.657280416395579</v>
+        <v>66.147161016949156</v>
       </c>
       <c r="S20" t="s">
         <v>70</v>
@@ -2048,18 +2054,18 @@
         <v>0</v>
       </c>
       <c r="X20">
-        <v>5494</v>
+        <v>5035</v>
       </c>
       <c r="Y20">
-        <v>8841.7386714217246</v>
+        <v>8103.0495468890394</v>
       </c>
       <c r="Z20">
         <f t="shared" si="1"/>
-        <v>33.457280416395577</v>
+        <v>7.4671610169491531</v>
       </c>
       <c r="AA20">
         <f t="shared" si="2"/>
-        <v>40.657280416395579</v>
+        <v>66.147161016949156</v>
       </c>
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.35">
@@ -2116,7 +2122,7 @@
       </c>
       <c r="R21">
         <f t="shared" si="0"/>
-        <v>40.657280416395579</v>
+        <v>66.147161016949156</v>
       </c>
       <c r="S21" t="s">
         <v>70</v>
@@ -2128,18 +2134,18 @@
         <v>0</v>
       </c>
       <c r="X21">
-        <v>5494</v>
+        <v>5035</v>
       </c>
       <c r="Y21">
-        <v>8841.7386714217246</v>
+        <v>8103.0495468890394</v>
       </c>
       <c r="Z21">
         <f t="shared" si="1"/>
-        <v>33.457280416395577</v>
+        <v>7.4671610169491531</v>
       </c>
       <c r="AA21">
         <f t="shared" si="2"/>
-        <v>40.657280416395579</v>
+        <v>66.147161016949156</v>
       </c>
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.35">
@@ -2196,7 +2202,7 @@
       </c>
       <c r="R22">
         <f t="shared" si="0"/>
-        <v>35.28</v>
+        <v>64.98</v>
       </c>
       <c r="S22" t="s">
         <v>70</v>
@@ -2208,18 +2214,18 @@
         <v>0</v>
       </c>
       <c r="X22">
-        <v>4611</v>
+        <v>4248</v>
       </c>
       <c r="Y22">
-        <v>7420.687479782594</v>
+        <v>6836.4954270475946</v>
       </c>
       <c r="Z22">
         <f>((($U$4/$Y$22)*Y22)*$T$1)/$U$1</f>
-        <v>28.08</v>
+        <v>6.3000000000000007</v>
       </c>
       <c r="AA22">
         <f t="shared" si="2"/>
-        <v>35.28</v>
+        <v>64.98</v>
       </c>
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.35">
@@ -2276,7 +2282,7 @@
       </c>
       <c r="R23">
         <f t="shared" si="0"/>
-        <v>32.466519193233573</v>
+        <v>64.017499999999998</v>
       </c>
       <c r="S23" t="s">
         <v>70</v>
@@ -2288,18 +2294,18 @@
         <v>0</v>
       </c>
       <c r="X23">
-        <v>4149</v>
+        <v>3599</v>
       </c>
       <c r="Y23">
-        <v>6677.1703217562308</v>
+        <v>5792.0308479153236</v>
       </c>
       <c r="Z23">
         <f t="shared" si="1"/>
-        <v>25.26651919323357</v>
+        <v>5.3375000000000012</v>
       </c>
       <c r="AA23">
         <f t="shared" si="2"/>
-        <v>32.466519193233573</v>
+        <v>64.017499999999998</v>
       </c>
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.35">
@@ -2356,7 +2362,7 @@
       </c>
       <c r="R24">
         <f t="shared" si="0"/>
-        <v>40.291893298633703</v>
+        <v>66.058177966101695</v>
       </c>
       <c r="S24" t="s">
         <v>70</v>
@@ -2368,18 +2374,18 @@
         <v>0</v>
       </c>
       <c r="X24">
-        <v>5434</v>
+        <v>4975</v>
       </c>
       <c r="Y24">
-        <v>8745.1780015481709</v>
+        <v>8006.4888770154857</v>
       </c>
       <c r="Z24">
         <f t="shared" si="1"/>
-        <v>33.0918932986337</v>
+        <v>7.3781779661016955</v>
       </c>
       <c r="AA24">
         <f t="shared" si="2"/>
-        <v>40.291893298633703</v>
+        <v>66.058177966101695</v>
       </c>
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.35">
@@ -2436,7 +2442,7 @@
       </c>
       <c r="R25">
         <f>AVERAGE(R8:R24)</f>
-        <v>35.287522675953916</v>
+        <v>65.249130109671</v>
       </c>
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.35">
@@ -2493,7 +2499,7 @@
       </c>
       <c r="Y26">
         <f>7.8/Y22</f>
-        <v>1.0511155497722859E-3</v>
+        <v>1.1409354519774035E-3</v>
       </c>
     </row>
     <row r="27" spans="1:27" x14ac:dyDescent="0.35">
@@ -2612,7 +2618,7 @@
       </c>
       <c r="Y28">
         <f>Y27*Y26</f>
-        <v>1.0511155497722859</v>
+        <v>1.1409354519774035</v>
       </c>
     </row>
     <row r="29" spans="1:27" x14ac:dyDescent="0.35">
@@ -3179,7 +3185,7 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>20.52</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
@@ -3387,7 +3393,7 @@
         <v>34</v>
       </c>
       <c r="B35">
-        <v>20.52</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
update LNG import emissions from TT
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
+++ b/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E37ED7FE-2F3B-4F69-94F5-DF5CB84DEA35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E912C8C-686D-40EA-B2E8-C0B0C4E471D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{BAA9D55F-0FEB-4558-AFDF-92239B956412}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BAA9D55F-0FEB-4558-AFDF-92239B956412}"/>
   </bookViews>
   <sheets>
     <sheet name="Emission_Factors_Import" sheetId="1" r:id="rId1"/>
@@ -698,7 +698,7 @@
         <v>81.639529411764684</v>
       </c>
       <c r="D2">
-        <v>70</v>
+        <v>53.765130109670991</v>
       </c>
       <c r="E2">
         <v>62.773291046064649</v>
@@ -741,15 +741,15 @@
       </c>
       <c r="S2">
         <f>U5-U4</f>
-        <v>16.3</v>
+        <v>13.11</v>
       </c>
       <c r="T2">
         <f>S2*T1</f>
-        <v>58680000</v>
+        <v>47196000</v>
       </c>
       <c r="U2">
         <f>T2/U1</f>
-        <v>58.68</v>
+        <v>47.195999999999998</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.35">
@@ -763,7 +763,7 @@
         <v>81.639529411764684</v>
       </c>
       <c r="D3">
-        <v>70</v>
+        <v>53.765130109670991</v>
       </c>
       <c r="E3">
         <v>62.773291046064649</v>
@@ -816,7 +816,7 @@
         <v>81.028026845637584</v>
       </c>
       <c r="D4">
-        <v>70</v>
+        <v>53.105957627118642</v>
       </c>
       <c r="E4">
         <v>63.33970029352696</v>
@@ -876,7 +876,7 @@
         <v>81.639529411764684</v>
       </c>
       <c r="D5">
-        <v>70</v>
+        <v>53.765130109670991</v>
       </c>
       <c r="E5">
         <v>62.773291046064649</v>
@@ -918,8 +918,7 @@
         <v>6.4829231993965921</v>
       </c>
       <c r="U5">
-        <f>16.3+1.75</f>
-        <v>18.05</v>
+        <v>14.86</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.35">
@@ -933,7 +932,7 @@
         <v>81.639529411764684</v>
       </c>
       <c r="D6">
-        <v>70</v>
+        <v>53.765130109670991</v>
       </c>
       <c r="E6">
         <v>62.773291046064649</v>
@@ -986,7 +985,7 @@
         <v>83.048859060402691</v>
       </c>
       <c r="D7">
-        <v>70</v>
+        <v>54.645364406779663</v>
       </c>
       <c r="E7">
         <v>60.519987640970186</v>
@@ -1039,7 +1038,7 @@
         <v>81.639529411764684</v>
       </c>
       <c r="D8">
-        <v>70</v>
+        <v>53.765130109670991</v>
       </c>
       <c r="E8">
         <v>62.773291046064649</v>
@@ -1082,7 +1081,7 @@
       </c>
       <c r="R8">
         <f t="shared" ref="R8:R24" si="0">AA8</f>
-        <v>64.58995762711865</v>
+        <v>53.105957627118642</v>
       </c>
       <c r="S8" t="s">
         <v>70</v>
@@ -1105,7 +1104,7 @@
       </c>
       <c r="AA8">
         <f>Z8+$U$2</f>
-        <v>64.58995762711865</v>
+        <v>53.105957627118642</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.35">
@@ -1119,7 +1118,7 @@
         <v>81.639529411764684</v>
       </c>
       <c r="D9">
-        <v>70</v>
+        <v>53.765130109670991</v>
       </c>
       <c r="E9">
         <v>62.773291046064649</v>
@@ -1162,7 +1161,7 @@
       </c>
       <c r="R9">
         <f t="shared" si="0"/>
-        <v>64.541016949152549</v>
+        <v>53.057016949152541</v>
       </c>
       <c r="S9" t="s">
         <v>70</v>
@@ -1185,7 +1184,7 @@
       </c>
       <c r="AA9">
         <f t="shared" ref="AA9:AA24" si="2">Z9+$U$2</f>
-        <v>64.541016949152549</v>
+        <v>53.057016949152541</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.35">
@@ -1199,7 +1198,7 @@
         <v>82.274738255033554</v>
       </c>
       <c r="D10">
-        <v>70</v>
+        <v>54.663161016949154</v>
       </c>
       <c r="E10">
         <v>64.996823729337251</v>
@@ -1242,7 +1241,7 @@
       </c>
       <c r="R10">
         <f t="shared" si="0"/>
-        <v>65.943983050847464</v>
+        <v>54.459983050847455</v>
       </c>
       <c r="S10" t="s">
         <v>70</v>
@@ -1265,7 +1264,7 @@
       </c>
       <c r="AA10">
         <f t="shared" si="2"/>
-        <v>65.943983050847464</v>
+        <v>54.459983050847455</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.35">
@@ -1279,7 +1278,7 @@
         <v>82.274738255033554</v>
       </c>
       <c r="D11">
-        <v>70</v>
+        <v>54.663161016949154</v>
       </c>
       <c r="E11">
         <v>64.996823729337251</v>
@@ -1322,7 +1321,7 @@
       </c>
       <c r="R11">
         <f t="shared" si="0"/>
-        <v>66.206483050847453</v>
+        <v>54.722483050847458</v>
       </c>
       <c r="S11" t="s">
         <v>70</v>
@@ -1345,7 +1344,7 @@
       </c>
       <c r="AA11">
         <f t="shared" si="2"/>
-        <v>66.206483050847453</v>
+        <v>54.722483050847458</v>
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.35">
@@ -1359,7 +1358,7 @@
         <v>80.987436241610737</v>
       </c>
       <c r="D12">
-        <v>70</v>
+        <v>53.057016949152541</v>
       </c>
       <c r="E12">
         <v>63.291982079406765</v>
@@ -1402,7 +1401,7 @@
       </c>
       <c r="R12">
         <f t="shared" si="0"/>
-        <v>66.129364406779658</v>
+        <v>54.645364406779663</v>
       </c>
       <c r="S12" t="s">
         <v>70</v>
@@ -1425,7 +1424,7 @@
       </c>
       <c r="AA12">
         <f t="shared" si="2"/>
-        <v>66.129364406779658</v>
+        <v>54.645364406779663</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.35">
@@ -1439,7 +1438,7 @@
         <v>81.36</v>
       </c>
       <c r="D13">
-        <v>70</v>
+        <v>53.495999999999995</v>
       </c>
       <c r="E13">
         <v>63.72</v>
@@ -1482,7 +1481,7 @@
       </c>
       <c r="R13">
         <f t="shared" si="0"/>
-        <v>65.832754237288128</v>
+        <v>54.348754237288134</v>
       </c>
       <c r="S13" t="s">
         <v>70</v>
@@ -1505,7 +1504,7 @@
       </c>
       <c r="AA13">
         <f t="shared" si="2"/>
-        <v>65.832754237288128</v>
+        <v>54.348754237288134</v>
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.35">
@@ -1519,7 +1518,7 @@
         <v>82.867651006711412</v>
       </c>
       <c r="D14">
-        <v>70</v>
+        <v>54.459983050847455</v>
       </c>
       <c r="E14">
         <v>59.567069365054842</v>
@@ -1562,7 +1561,7 @@
       </c>
       <c r="R14">
         <f t="shared" si="0"/>
-        <v>64.687838983050852</v>
+        <v>53.203838983050844</v>
       </c>
       <c r="S14" t="s">
         <v>70</v>
@@ -1585,7 +1584,7 @@
       </c>
       <c r="AA14">
         <f t="shared" si="2"/>
-        <v>64.687838983050852</v>
+        <v>53.203838983050844</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.35">
@@ -1599,7 +1598,7 @@
         <v>81.639529411764684</v>
       </c>
       <c r="D15">
-        <v>70</v>
+        <v>53.765130109670991</v>
       </c>
       <c r="E15">
         <v>62.773291046064649</v>
@@ -1642,7 +1641,7 @@
       </c>
       <c r="R15">
         <f t="shared" si="0"/>
-        <v>65.549491525423733</v>
+        <v>54.065491525423724</v>
       </c>
       <c r="S15" t="s">
         <v>70</v>
@@ -1665,7 +1664,7 @@
       </c>
       <c r="AA15">
         <f t="shared" si="2"/>
-        <v>65.549491525423733</v>
+        <v>54.065491525423724</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.35">
@@ -1679,7 +1678,7 @@
         <v>80.416268456375832</v>
       </c>
       <c r="D16">
-        <v>70</v>
+        <v>52.533499999999997</v>
       </c>
       <c r="E16">
         <v>63.051945002317318</v>
@@ -1722,7 +1721,7 @@
       </c>
       <c r="R16">
         <f t="shared" si="0"/>
-        <v>63.572584745762711</v>
+        <v>52.088584745762709</v>
       </c>
       <c r="S16" t="s">
         <v>70</v>
@@ -1745,7 +1744,7 @@
       </c>
       <c r="AA16">
         <f t="shared" si="2"/>
-        <v>63.572584745762711</v>
+        <v>52.088584745762709</v>
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.35">
@@ -1759,7 +1758,7 @@
         <v>81.963060402684562</v>
       </c>
       <c r="D17">
-        <v>70</v>
+        <v>54.722483050847458</v>
       </c>
       <c r="E17">
         <v>60.700738452031516</v>
@@ -1802,7 +1801,7 @@
       </c>
       <c r="R17">
         <f t="shared" si="0"/>
-        <v>64.085720338983052</v>
+        <v>52.60172033898305</v>
       </c>
       <c r="S17" t="s">
         <v>70</v>
@@ -1825,7 +1824,7 @@
       </c>
       <c r="AA17">
         <f t="shared" si="2"/>
-        <v>64.085720338983052</v>
+        <v>52.60172033898305</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.35">
@@ -1839,7 +1838,7 @@
         <v>82.187758389261745</v>
       </c>
       <c r="D18">
-        <v>70</v>
+        <v>54.574177966101693</v>
       </c>
       <c r="E18">
         <v>64.910063340027804</v>
@@ -1882,7 +1881,7 @@
       </c>
       <c r="R18">
         <f t="shared" si="0"/>
-        <v>66.172372881355926</v>
+        <v>54.688372881355932</v>
       </c>
       <c r="S18" t="s">
         <v>70</v>
@@ -1905,7 +1904,7 @@
       </c>
       <c r="AA18">
         <f t="shared" si="2"/>
-        <v>66.172372881355926</v>
+        <v>54.688372881355932</v>
       </c>
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.35">
@@ -1919,7 +1918,7 @@
         <v>81.967409395973149</v>
       </c>
       <c r="D19">
-        <v>70</v>
+        <v>54.348754237288134</v>
       </c>
       <c r="E19">
         <v>64.690270353777223</v>
@@ -1962,7 +1961,7 @@
       </c>
       <c r="R19">
         <f t="shared" si="0"/>
-        <v>64.573644067796607</v>
+        <v>53.089644067796613</v>
       </c>
       <c r="S19" t="s">
         <v>70</v>
@@ -1985,7 +1984,7 @@
       </c>
       <c r="AA19">
         <f t="shared" si="2"/>
-        <v>64.573644067796607</v>
+        <v>53.089644067796613</v>
       </c>
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.35">
@@ -1999,7 +1998,7 @@
         <v>81.639529411764684</v>
       </c>
       <c r="D20">
-        <v>70</v>
+        <v>53.765130109670991</v>
       </c>
       <c r="E20">
         <v>62.773291046064649</v>
@@ -2042,7 +2041,7 @@
       </c>
       <c r="R20">
         <f t="shared" si="0"/>
-        <v>66.147161016949156</v>
+        <v>54.663161016949154</v>
       </c>
       <c r="S20" t="s">
         <v>70</v>
@@ -2065,7 +2064,7 @@
       </c>
       <c r="AA20">
         <f t="shared" si="2"/>
-        <v>66.147161016949156</v>
+        <v>54.663161016949154</v>
       </c>
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.35">
@@ -2079,7 +2078,7 @@
         <v>81.639529411764684</v>
       </c>
       <c r="D21">
-        <v>70</v>
+        <v>53.765130109670991</v>
       </c>
       <c r="E21">
         <v>62.773291046064649</v>
@@ -2122,7 +2121,7 @@
       </c>
       <c r="R21">
         <f t="shared" si="0"/>
-        <v>66.147161016949156</v>
+        <v>54.663161016949154</v>
       </c>
       <c r="S21" t="s">
         <v>70</v>
@@ -2145,7 +2144,7 @@
       </c>
       <c r="AA21">
         <f t="shared" si="2"/>
-        <v>66.147161016949156</v>
+        <v>54.663161016949154</v>
       </c>
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.35">
@@ -2159,7 +2158,7 @@
         <v>81.123704697986582</v>
       </c>
       <c r="D22">
-        <v>70</v>
+        <v>53.203838983050844</v>
       </c>
       <c r="E22">
         <v>63.435136721767336</v>
@@ -2202,7 +2201,7 @@
       </c>
       <c r="R22">
         <f t="shared" si="0"/>
-        <v>64.98</v>
+        <v>53.495999999999995</v>
       </c>
       <c r="S22" t="s">
         <v>70</v>
@@ -2225,7 +2224,7 @@
       </c>
       <c r="AA22">
         <f t="shared" si="2"/>
-        <v>64.98</v>
+        <v>53.495999999999995</v>
       </c>
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.35">
@@ -2239,7 +2238,7 @@
         <v>81.639529411764684</v>
       </c>
       <c r="D23">
-        <v>70</v>
+        <v>53.765130109670991</v>
       </c>
       <c r="E23">
         <v>62.773291046064649</v>
@@ -2282,7 +2281,7 @@
       </c>
       <c r="R23">
         <f t="shared" si="0"/>
-        <v>64.017499999999998</v>
+        <v>52.533499999999997</v>
       </c>
       <c r="S23" t="s">
         <v>70</v>
@@ -2305,7 +2304,7 @@
       </c>
       <c r="AA23">
         <f t="shared" si="2"/>
-        <v>64.017499999999998</v>
+        <v>52.533499999999997</v>
       </c>
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.35">
@@ -2319,7 +2318,7 @@
         <v>81.639529411764684</v>
       </c>
       <c r="D24">
-        <v>70</v>
+        <v>53.765130109670991</v>
       </c>
       <c r="E24">
         <v>62.773291046064649</v>
@@ -2362,7 +2361,7 @@
       </c>
       <c r="R24">
         <f t="shared" si="0"/>
-        <v>66.058177966101695</v>
+        <v>54.574177966101693</v>
       </c>
       <c r="S24" t="s">
         <v>70</v>
@@ -2385,7 +2384,7 @@
       </c>
       <c r="AA24">
         <f t="shared" si="2"/>
-        <v>66.058177966101695</v>
+        <v>54.574177966101693</v>
       </c>
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.35">
@@ -2399,7 +2398,7 @@
         <v>81.690523489932886</v>
       </c>
       <c r="D25">
-        <v>70</v>
+        <v>54.065491525423724</v>
       </c>
       <c r="E25">
         <v>64.414083114475517</v>
@@ -2442,7 +2441,7 @@
       </c>
       <c r="R25">
         <f>AVERAGE(R8:R24)</f>
-        <v>65.249130109671</v>
+        <v>53.765130109670991</v>
       </c>
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.35">
@@ -2456,7 +2455,7 @@
         <v>80.417718120805375</v>
       </c>
       <c r="D26">
-        <v>70</v>
+        <v>52.088584745762709</v>
       </c>
       <c r="E26">
         <v>61.877787733662906</v>
@@ -2513,7 +2512,7 @@
         <v>81.639529411764684</v>
       </c>
       <c r="D27">
-        <v>70</v>
+        <v>53.765130109670991</v>
       </c>
       <c r="E27">
         <v>62.773291046064649</v>
@@ -2572,7 +2571,7 @@
         <v>81.639529411764684</v>
       </c>
       <c r="D28">
-        <v>70</v>
+        <v>53.765130109670991</v>
       </c>
       <c r="E28">
         <v>62.773291046064649</v>
@@ -2632,7 +2631,7 @@
         <v>81.639529411764684</v>
       </c>
       <c r="D29">
-        <v>70</v>
+        <v>53.765130109670991</v>
       </c>
       <c r="E29">
         <v>62.773291046064649</v>
@@ -2685,7 +2684,7 @@
         <v>81.639529411764684</v>
       </c>
       <c r="D30">
-        <v>70</v>
+        <v>53.765130109670991</v>
       </c>
       <c r="E30">
         <v>62.773291046064649</v>
@@ -2738,7 +2737,7 @@
         <v>81.639529411764684</v>
       </c>
       <c r="D31">
-        <v>70</v>
+        <v>53.765130109670991</v>
       </c>
       <c r="E31">
         <v>62.773291046064649</v>
@@ -2799,7 +2798,7 @@
         <v>80.609073825503359</v>
       </c>
       <c r="D32">
-        <v>70</v>
+        <v>52.60172033898305</v>
       </c>
       <c r="E32">
         <v>60.997169782172101</v>
@@ -2852,7 +2851,7 @@
         <v>81.639529411764684</v>
       </c>
       <c r="D33">
-        <v>70</v>
+        <v>53.765130109670991</v>
       </c>
       <c r="E33">
         <v>62.773291046064649</v>
@@ -2905,7 +2904,7 @@
         <v>81.639529411764684</v>
       </c>
       <c r="D34">
-        <v>70</v>
+        <v>53.765130109670991</v>
       </c>
       <c r="E34">
         <v>62.773291046064649</v>
@@ -2958,7 +2957,7 @@
         <v>83.090899328859052</v>
       </c>
       <c r="D35">
-        <v>70</v>
+        <v>54.688372881355932</v>
       </c>
       <c r="E35">
         <v>59.565623358566349</v>
@@ -3011,7 +3010,7 @@
         <v>80.564134228187925</v>
       </c>
       <c r="D36">
-        <v>70</v>
+        <v>53.089644067796613</v>
       </c>
       <c r="E36">
         <v>63.070743086667697</v>
@@ -3064,7 +3063,7 @@
         <v>81.639529411764684</v>
       </c>
       <c r="D37">
-        <v>70</v>
+        <v>53.765130109670991</v>
       </c>
       <c r="E37">
         <v>62.773291046064649</v>

</xml_diff>

<commit_message>
update LNG import emissions from EG
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
+++ b/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E912C8C-686D-40EA-B2E8-C0B0C4E471D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22487EB8-98FF-4D5D-8D07-9788B057CA7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BAA9D55F-0FEB-4558-AFDF-92239B956412}"/>
   </bookViews>
@@ -249,7 +249,7 @@
     <t>LV_LNG</t>
   </si>
   <si>
-    <t>TT_LNG</t>
+    <t>EG_LNG</t>
   </si>
 </sst>
 </file>
@@ -731,7 +731,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O2">
-        <v>68.015751583500688</v>
+        <v>72.142818929885323</v>
       </c>
       <c r="P2">
         <v>69.650954303405584</v>
@@ -741,15 +741,15 @@
       </c>
       <c r="S2">
         <f>U5-U4</f>
-        <v>13.11</v>
+        <v>19.419148936170213</v>
       </c>
       <c r="T2">
         <f>S2*T1</f>
-        <v>47196000</v>
+        <v>69908936.170212761</v>
       </c>
       <c r="U2">
         <f>T2/U1</f>
-        <v>47.195999999999998</v>
+        <v>69.908936170212755</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.35">
@@ -796,7 +796,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O3">
-        <v>68.015751583500688</v>
+        <v>72.142818929885323</v>
       </c>
       <c r="P3">
         <v>69.650954303405584</v>
@@ -849,7 +849,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O4">
-        <v>68.015751583500688</v>
+        <v>72.570716636937036</v>
       </c>
       <c r="P4">
         <v>70.201212631578954</v>
@@ -862,7 +862,11 @@
         <v>1.7463157894736843</v>
       </c>
       <c r="U4">
-        <v>1.75</v>
+        <v>0.8</v>
+      </c>
+      <c r="X4">
+        <f>(15.4+12.8)/2</f>
+        <v>14.100000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.35">
@@ -909,7 +913,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O5">
-        <v>68.015751583500688</v>
+        <v>72.142818929885323</v>
       </c>
       <c r="P5">
         <v>69.650954303405584</v>
@@ -918,7 +922,15 @@
         <v>6.4829231993965921</v>
       </c>
       <c r="U5">
-        <v>14.86</v>
+        <f>27.3-19.2+V5</f>
+        <v>20.219148936170214</v>
+      </c>
+      <c r="V5">
+        <f>19.2*(X5/X4)</f>
+        <v>12.119148936170211</v>
+      </c>
+      <c r="X5">
+        <v>8.9</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.35">
@@ -965,7 +977,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O6">
-        <v>68.015751583500688</v>
+        <v>72.142818929885323</v>
       </c>
       <c r="P6">
         <v>69.650954303405584</v>
@@ -1018,7 +1030,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O7">
-        <v>68.015751583500688</v>
+        <v>70.952739108847155</v>
       </c>
       <c r="P7">
         <v>67.541002105263161</v>
@@ -1071,7 +1083,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O8">
-        <v>68.015751583500688</v>
+        <v>72.142818929885323</v>
       </c>
       <c r="P8">
         <v>69.650954303405584</v>
@@ -1081,7 +1093,7 @@
       </c>
       <c r="R8">
         <f t="shared" ref="R8:R24" si="0">AA8</f>
-        <v>53.105957627118642</v>
+        <v>72.570716636937036</v>
       </c>
       <c r="S8" t="s">
         <v>70</v>
@@ -1093,18 +1105,18 @@
         <v>0</v>
       </c>
       <c r="X8">
-        <v>3985</v>
+        <v>3208</v>
       </c>
       <c r="Y8">
-        <v>6413.2378241018514</v>
+        <v>5162.7771492393322</v>
       </c>
       <c r="Z8">
         <f>((($U$4/$Y$22)*Y8)*$T$1)/$U$1</f>
-        <v>5.9099576271186454</v>
+        <v>2.661780466724287</v>
       </c>
       <c r="AA8">
         <f>Z8+$U$2</f>
-        <v>53.105957627118642</v>
+        <v>72.570716636937036</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.35">
@@ -1151,7 +1163,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O9">
-        <v>68.015751583500688</v>
+        <v>72.142818929885323</v>
       </c>
       <c r="P9">
         <v>69.650954303405584</v>
@@ -1161,7 +1173,7 @@
       </c>
       <c r="R9">
         <f t="shared" si="0"/>
-        <v>53.057016949152541</v>
+        <v>71.074709722503158</v>
       </c>
       <c r="S9" t="s">
         <v>70</v>
@@ -1173,18 +1185,18 @@
         <v>0</v>
       </c>
       <c r="X9">
-        <v>3952</v>
+        <v>1405</v>
       </c>
       <c r="Y9">
-        <v>6360.1294556713965</v>
+        <v>2261.1290195390466</v>
       </c>
       <c r="Z9">
         <f t="shared" ref="Z9:Z24" si="1">((($U$4/$Y$22)*Y9)*$T$1)/$U$1</f>
-        <v>5.8610169491525426</v>
+        <v>1.1657735522904062</v>
       </c>
       <c r="AA9">
         <f t="shared" ref="AA9:AA24" si="2">Z9+$U$2</f>
-        <v>53.057016949152541</v>
+        <v>71.074709722503158</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.35">
@@ -1231,7 +1243,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O10">
-        <v>68.015751583500688</v>
+        <v>73.521589584214482</v>
       </c>
       <c r="P10">
         <v>71.764597894736838</v>
@@ -1241,7 +1253,7 @@
       </c>
       <c r="R10">
         <f t="shared" si="0"/>
-        <v>54.459983050847455</v>
+        <v>70.338737380238683</v>
       </c>
       <c r="S10" t="s">
         <v>70</v>
@@ -1253,18 +1265,18 @@
         <v>0</v>
       </c>
       <c r="X10">
-        <v>4898</v>
+        <v>518</v>
       </c>
       <c r="Y10">
-        <v>7882.5693506777588</v>
+        <v>833.64044990834611</v>
       </c>
       <c r="Z10">
         <f t="shared" si="1"/>
-        <v>7.2639830508474574</v>
+        <v>0.42980121002592919</v>
       </c>
       <c r="AA10">
         <f t="shared" si="2"/>
-        <v>54.459983050847455</v>
+        <v>70.338737380238683</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.35">
@@ -1311,7 +1323,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O11">
-        <v>68.015751583500688</v>
+        <v>73.521589584214482</v>
       </c>
       <c r="P11">
         <v>71.764597894736838</v>
@@ -1321,7 +1333,7 @@
       </c>
       <c r="R11">
         <f t="shared" si="0"/>
-        <v>54.722483050847458</v>
+        <v>70.936974199599092</v>
       </c>
       <c r="S11" t="s">
         <v>70</v>
@@ -1333,18 +1345,18 @@
         <v>0</v>
       </c>
       <c r="X11">
-        <v>5075</v>
+        <v>1239</v>
       </c>
       <c r="Y11">
-        <v>8167.4233268047419</v>
+        <v>1993.9778328888817</v>
       </c>
       <c r="Z11">
         <f t="shared" si="1"/>
-        <v>7.5264830508474594</v>
+        <v>1.028038029386344</v>
       </c>
       <c r="AA11">
         <f t="shared" si="2"/>
-        <v>54.722483050847458</v>
+        <v>70.936974199599092</v>
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.35">
@@ -1391,7 +1403,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O12">
-        <v>68.015751583500688</v>
+        <v>71.074709722503158</v>
       </c>
       <c r="P12">
         <v>69.737381052631576</v>
@@ -1401,7 +1413,7 @@
       </c>
       <c r="R12">
         <f t="shared" si="0"/>
-        <v>54.645364406779663</v>
+        <v>70.952739108847155</v>
       </c>
       <c r="S12" t="s">
         <v>70</v>
@@ -1413,18 +1425,18 @@
         <v>0</v>
       </c>
       <c r="X12">
-        <v>5023</v>
+        <v>1258</v>
       </c>
       <c r="Y12">
-        <v>8083.7374129143291</v>
+        <v>2024.5553783488403</v>
       </c>
       <c r="Z12">
         <f t="shared" si="1"/>
-        <v>7.4493644067796625</v>
+        <v>1.0438029386343994</v>
       </c>
       <c r="AA12">
         <f t="shared" si="2"/>
-        <v>54.645364406779663</v>
+        <v>70.952739108847155</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.35">
@@ -1471,7 +1483,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O13">
-        <v>68.015751583500688</v>
+        <v>72.78893617021275</v>
       </c>
       <c r="P13">
         <v>70.56</v>
@@ -1481,7 +1493,7 @@
       </c>
       <c r="R13">
         <f t="shared" si="0"/>
-        <v>54.348754237288134</v>
+        <v>73.345686386288818</v>
       </c>
       <c r="S13" t="s">
         <v>70</v>
@@ -1493,18 +1505,18 @@
         <v>0</v>
       </c>
       <c r="X13">
-        <v>4823</v>
+        <v>4142</v>
       </c>
       <c r="Y13">
-        <v>7761.8685133358167</v>
+        <v>6665.9049102709832</v>
       </c>
       <c r="Z13">
         <f t="shared" si="1"/>
-        <v>7.1527542372881356</v>
+        <v>3.4367502160760592</v>
       </c>
       <c r="AA13">
         <f t="shared" si="2"/>
-        <v>54.348754237288134</v>
+        <v>73.345686386288818</v>
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.35">
@@ -1551,7 +1563,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O14">
-        <v>68.015751583500688</v>
+        <v>70.338737380238683</v>
       </c>
       <c r="P14">
         <v>66.790686315789472</v>
@@ -1561,7 +1573,7 @@
       </c>
       <c r="R14">
         <f t="shared" si="0"/>
-        <v>53.203838983050844</v>
+        <v>72.625478953272392</v>
       </c>
       <c r="S14" t="s">
         <v>70</v>
@@ -1573,18 +1585,18 @@
         <v>0</v>
       </c>
       <c r="X14">
-        <v>4051</v>
+        <v>3274</v>
       </c>
       <c r="Y14">
-        <v>6519.4545609627603</v>
+        <v>5268.9938861002411</v>
       </c>
       <c r="Z14">
         <f t="shared" si="1"/>
-        <v>6.0078389830508483</v>
+        <v>2.7165427830596371</v>
       </c>
       <c r="AA14">
         <f t="shared" si="2"/>
-        <v>53.203838983050844</v>
+        <v>72.625478953272392</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.35">
@@ -1631,7 +1643,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O15">
-        <v>68.015751583500688</v>
+        <v>72.142818929885323</v>
       </c>
       <c r="P15">
         <v>69.650954303405584</v>
@@ -1641,7 +1653,7 @@
       </c>
       <c r="R15">
         <f t="shared" si="0"/>
-        <v>54.065491525423724</v>
+        <v>73.091788374188553</v>
       </c>
       <c r="S15" t="s">
         <v>70</v>
@@ -1653,18 +1665,18 @@
         <v>0</v>
       </c>
       <c r="X15">
-        <v>4632</v>
+        <v>3836</v>
       </c>
       <c r="Y15">
-        <v>7454.4837142383376</v>
+        <v>6173.4454939158604</v>
       </c>
       <c r="Z15">
         <f t="shared" si="1"/>
-        <v>6.8694915254237285</v>
+        <v>3.1828522039757998</v>
       </c>
       <c r="AA15">
         <f t="shared" si="2"/>
-        <v>54.065491525423724</v>
+        <v>73.091788374188553</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.35">
@@ -1711,7 +1723,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O16">
-        <v>68.015751583500688</v>
+        <v>72.405599955865299</v>
       </c>
       <c r="P16">
         <v>69.929734736842107</v>
@@ -1721,7 +1733,7 @@
       </c>
       <c r="R16">
         <f t="shared" si="0"/>
-        <v>52.088584745762709</v>
+        <v>71.636438330973348</v>
       </c>
       <c r="S16" t="s">
         <v>70</v>
@@ -1733,18 +1745,18 @@
         <v>0</v>
       </c>
       <c r="X16">
-        <v>3299</v>
+        <v>2082</v>
       </c>
       <c r="Y16">
-        <v>5309.2274985475551</v>
+        <v>3350.6552446123096</v>
       </c>
       <c r="Z16">
         <f t="shared" si="1"/>
-        <v>4.8925847457627123</v>
+        <v>1.7275021607605878</v>
       </c>
       <c r="AA16">
         <f t="shared" si="2"/>
-        <v>52.088584745762709</v>
+        <v>71.636438330973348</v>
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.35">
@@ -1791,7 +1803,7 @@
         <v>67.958745558473652</v>
       </c>
       <c r="O17">
-        <v>67.958745558473652</v>
+        <v>70.936974199599092</v>
       </c>
       <c r="P17">
         <v>71.475385263157904</v>
@@ -1801,7 +1813,7 @@
       </c>
       <c r="R17">
         <f t="shared" si="0"/>
-        <v>52.60172033898305</v>
+        <v>71.316161753618118</v>
       </c>
       <c r="S17" t="s">
         <v>70</v>
@@ -1813,18 +1825,18 @@
         <v>0</v>
       </c>
       <c r="X17">
-        <v>3645</v>
+        <v>1696</v>
       </c>
       <c r="Y17">
-        <v>5866.0606948183813</v>
+        <v>2729.4482684257819</v>
       </c>
       <c r="Z17">
         <f t="shared" si="1"/>
-        <v>5.405720338983051</v>
+        <v>1.4072255834053586</v>
       </c>
       <c r="AA17">
         <f t="shared" si="2"/>
-        <v>52.60172033898305</v>
+        <v>71.316161753618118</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.35">
@@ -1871,7 +1883,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O18">
-        <v>68.015751583500688</v>
+        <v>73.471805660273262</v>
       </c>
       <c r="P18">
         <v>71.682745263157898</v>
@@ -1881,7 +1893,7 @@
       </c>
       <c r="R18">
         <f t="shared" si="0"/>
-        <v>54.688372881355932</v>
+        <v>70.50800272163886</v>
       </c>
       <c r="S18" t="s">
         <v>70</v>
@@ -1893,18 +1905,18 @@
         <v>0</v>
       </c>
       <c r="X18">
-        <v>5052</v>
+        <v>722</v>
       </c>
       <c r="Y18">
-        <v>8130.4084033532126</v>
+        <v>1161.9467274784283</v>
       </c>
       <c r="Z18">
         <f t="shared" si="1"/>
-        <v>7.4923728813559318</v>
+        <v>0.5990665514261021</v>
       </c>
       <c r="AA18">
         <f t="shared" si="2"/>
-        <v>54.688372881355932</v>
+        <v>70.50800272163886</v>
       </c>
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.35">
@@ -1951,7 +1963,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O19">
-        <v>68.015751583500688</v>
+        <v>73.345686386288818</v>
       </c>
       <c r="P19">
         <v>69.650954303405584</v>
@@ -1961,7 +1973,7 @@
       </c>
       <c r="R19">
         <f t="shared" si="0"/>
-        <v>53.089644067796613</v>
+        <v>72.320967285165224</v>
       </c>
       <c r="S19" t="s">
         <v>70</v>
@@ -1973,18 +1985,18 @@
         <v>0</v>
       </c>
       <c r="X19">
-        <v>3974</v>
+        <v>2907</v>
       </c>
       <c r="Y19">
-        <v>6395.5350346250334</v>
+        <v>4678.3644553736722</v>
       </c>
       <c r="Z19">
         <f t="shared" si="1"/>
-        <v>5.8936440677966111</v>
+        <v>2.4120311149524638</v>
       </c>
       <c r="AA19">
         <f t="shared" si="2"/>
-        <v>53.089644067796613</v>
+        <v>72.320967285165224</v>
       </c>
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.35">
@@ -2031,7 +2043,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O20">
-        <v>68.015751583500688</v>
+        <v>72.142818929885323</v>
       </c>
       <c r="P20">
         <v>69.650954303405584</v>
@@ -2041,7 +2053,7 @@
       </c>
       <c r="R20">
         <f t="shared" si="0"/>
-        <v>54.663161016949154</v>
+        <v>73.521589584214482</v>
       </c>
       <c r="S20" t="s">
         <v>70</v>
@@ -2053,18 +2065,18 @@
         <v>0</v>
       </c>
       <c r="X20">
-        <v>5035</v>
+        <v>4354</v>
       </c>
       <c r="Y20">
-        <v>8103.0495468890394</v>
+        <v>7007.085943824206</v>
       </c>
       <c r="Z20">
         <f t="shared" si="1"/>
-        <v>7.4671610169491531</v>
+        <v>3.6126534140017288</v>
       </c>
       <c r="AA20">
         <f t="shared" si="2"/>
-        <v>54.663161016949154</v>
+        <v>73.521589584214482</v>
       </c>
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.35">
@@ -2111,7 +2123,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O21">
-        <v>68.015751583500688</v>
+        <v>72.142818929885323</v>
       </c>
       <c r="P21">
         <v>69.650954303405584</v>
@@ -2121,7 +2133,7 @@
       </c>
       <c r="R21">
         <f t="shared" si="0"/>
-        <v>54.663161016949154</v>
+        <v>73.521589584214482</v>
       </c>
       <c r="S21" t="s">
         <v>70</v>
@@ -2133,18 +2145,18 @@
         <v>0</v>
       </c>
       <c r="X21">
-        <v>5035</v>
+        <v>4354</v>
       </c>
       <c r="Y21">
-        <v>8103.0495468890394</v>
+        <v>7007.085943824206</v>
       </c>
       <c r="Z21">
         <f t="shared" si="1"/>
-        <v>7.4671610169491531</v>
+        <v>3.6126534140017288</v>
       </c>
       <c r="AA21">
         <f t="shared" si="2"/>
-        <v>54.663161016949154</v>
+        <v>73.521589584214482</v>
       </c>
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.35">
@@ -2191,7 +2203,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O22">
-        <v>68.015751583500688</v>
+        <v>72.625478953272392</v>
       </c>
       <c r="P22">
         <v>70.291250526315793</v>
@@ -2201,7 +2213,7 @@
       </c>
       <c r="R22">
         <f t="shared" si="0"/>
-        <v>53.495999999999995</v>
+        <v>72.78893617021275</v>
       </c>
       <c r="S22" t="s">
         <v>70</v>
@@ -2213,18 +2225,18 @@
         <v>0</v>
       </c>
       <c r="X22">
-        <v>4248</v>
+        <v>3471</v>
       </c>
       <c r="Y22">
-        <v>6836.4954270475946</v>
+        <v>5586.0347521850754</v>
       </c>
       <c r="Z22">
         <f>((($U$4/$Y$22)*Y22)*$T$1)/$U$1</f>
-        <v>6.3000000000000007</v>
+        <v>2.88</v>
       </c>
       <c r="AA22">
         <f t="shared" si="2"/>
-        <v>53.495999999999995</v>
+        <v>72.78893617021275</v>
       </c>
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.35">
@@ -2271,7 +2283,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O23">
-        <v>68.015751583500688</v>
+        <v>72.142818929885323</v>
       </c>
       <c r="P23">
         <v>69.650954303405584</v>
@@ -2281,7 +2293,7 @@
       </c>
       <c r="R23">
         <f t="shared" si="0"/>
-        <v>52.533499999999997</v>
+        <v>72.405599955865299</v>
       </c>
       <c r="S23" t="s">
         <v>70</v>
@@ -2293,18 +2305,18 @@
         <v>0</v>
       </c>
       <c r="X23">
-        <v>3599</v>
+        <v>3009</v>
       </c>
       <c r="Y23">
-        <v>5792.0308479153236</v>
+        <v>4842.5175941587131</v>
       </c>
       <c r="Z23">
         <f t="shared" si="1"/>
-        <v>5.3375000000000012</v>
+        <v>2.49666378565255</v>
       </c>
       <c r="AA23">
         <f t="shared" si="2"/>
-        <v>52.533499999999997</v>
+        <v>72.405599955865299</v>
       </c>
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.35">
@@ -2351,7 +2363,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O24">
-        <v>68.015751583500688</v>
+        <v>72.142818929885323</v>
       </c>
       <c r="P24">
         <v>69.650954303405584</v>
@@ -2361,7 +2373,7 @@
       </c>
       <c r="R24">
         <f t="shared" si="0"/>
-        <v>54.574177966101693</v>
+        <v>73.471805660273262</v>
       </c>
       <c r="S24" t="s">
         <v>70</v>
@@ -2373,18 +2385,18 @@
         <v>0</v>
       </c>
       <c r="X24">
-        <v>4975</v>
+        <v>4294</v>
       </c>
       <c r="Y24">
-        <v>8006.4888770154857</v>
+        <v>6910.5252739506523</v>
       </c>
       <c r="Z24">
         <f t="shared" si="1"/>
-        <v>7.3781779661016955</v>
+        <v>3.5628694900605016</v>
       </c>
       <c r="AA24">
         <f t="shared" si="2"/>
-        <v>54.574177966101693</v>
+        <v>73.471805660273262</v>
       </c>
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.35">
@@ -2431,7 +2443,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O25">
-        <v>68.015751583500688</v>
+        <v>73.091788374188553</v>
       </c>
       <c r="P25">
         <v>71.214821052631578</v>
@@ -2441,7 +2453,7 @@
       </c>
       <c r="R25">
         <f>AVERAGE(R8:R24)</f>
-        <v>53.765130109670991</v>
+        <v>72.142818929885323</v>
       </c>
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.35">
@@ -2488,7 +2500,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O26">
-        <v>68.015751583500688</v>
+        <v>71.636438330973348</v>
       </c>
       <c r="P26">
         <v>68.821995789473689</v>
@@ -2498,7 +2510,7 @@
       </c>
       <c r="Y26">
         <f>7.8/Y22</f>
-        <v>1.1409354519774035E-3</v>
+        <v>1.3963393258426995E-3</v>
       </c>
     </row>
     <row r="27" spans="1:27" x14ac:dyDescent="0.35">
@@ -2545,7 +2557,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O27">
-        <v>68.015751583500688</v>
+        <v>72.142818929885323</v>
       </c>
       <c r="P27">
         <v>69.650954303405584</v>
@@ -2604,7 +2616,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O28">
-        <v>68.015751583500688</v>
+        <v>72.142818929885323</v>
       </c>
       <c r="P28">
         <v>69.650954303405584</v>
@@ -2617,7 +2629,7 @@
       </c>
       <c r="Y28">
         <f>Y27*Y26</f>
-        <v>1.1409354519774035</v>
+        <v>1.3963393258426995</v>
       </c>
     </row>
     <row r="29" spans="1:27" x14ac:dyDescent="0.35">
@@ -2664,7 +2676,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O29">
-        <v>68.015751583500688</v>
+        <v>72.142818929885323</v>
       </c>
       <c r="P29">
         <v>69.650954303405584</v>
@@ -2717,7 +2729,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O30">
-        <v>68.015751583500688</v>
+        <v>72.142818929885323</v>
       </c>
       <c r="P30">
         <v>69.650954303405584</v>
@@ -2770,7 +2782,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O31">
-        <v>68.015751583500688</v>
+        <v>72.142818929885323</v>
       </c>
       <c r="P31">
         <v>69.650954303405584</v>
@@ -2831,7 +2843,7 @@
         <v>68.072757608527724</v>
       </c>
       <c r="O32">
-        <v>68.072757608527724</v>
+        <v>71.316161753618118</v>
       </c>
       <c r="P32">
         <v>67.991191578947365</v>
@@ -2884,7 +2896,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O33">
-        <v>68.015751583500688</v>
+        <v>72.142818929885323</v>
       </c>
       <c r="P33">
         <v>69.650954303405584</v>
@@ -2937,7 +2949,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O34">
-        <v>68.015751583500688</v>
+        <v>72.142818929885323</v>
       </c>
       <c r="P34">
         <v>69.650954303405584</v>
@@ -2990,7 +3002,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O35">
-        <v>68.015751583500688</v>
+        <v>70.50800272163886</v>
       </c>
       <c r="P35">
         <v>66.640623157894737</v>
@@ -3043,7 +3055,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O36">
-        <v>68.015751583500688</v>
+        <v>72.320967285165224</v>
       </c>
       <c r="P36">
         <v>69.947469473684208</v>
@@ -3096,7 +3108,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="O37">
-        <v>68.015751583500688</v>
+        <v>72.142818929885323</v>
       </c>
       <c r="P37">
         <v>69.650954303405584</v>

</xml_diff>

<commit_message>
update LNG import emissions from LY
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
+++ b/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22487EB8-98FF-4D5D-8D07-9788B057CA7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD580442-770A-48A5-AFA9-BADEAD102BAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BAA9D55F-0FEB-4558-AFDF-92239B956412}"/>
   </bookViews>
@@ -621,13 +621,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6177B6A9-4CD7-49C9-8407-62B26396811D}">
-  <dimension ref="A1:AA37"/>
+  <dimension ref="A1:AC37"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="26" max="26" width="11.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>52</v>
       </c>
@@ -687,7 +687,7 @@
         <v>1000000</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -722,7 +722,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L2">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M2">
         <v>68.015751583500688</v>
@@ -741,18 +741,18 @@
       </c>
       <c r="S2">
         <f>U5-U4</f>
-        <v>19.419148936170213</v>
+        <v>13.440141843971631</v>
       </c>
       <c r="T2">
         <f>S2*T1</f>
-        <v>69908936.170212761</v>
+        <v>48384510.638297871</v>
       </c>
       <c r="U2">
         <f>T2/U1</f>
-        <v>69.908936170212755</v>
-      </c>
-    </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.35">
+        <v>48.384510638297868</v>
+      </c>
+    </row>
+    <row r="3" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -787,7 +787,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L3">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M3">
         <v>68.015751583500688</v>
@@ -804,8 +804,11 @@
       <c r="Q3">
         <v>6.4829231993965921</v>
       </c>
-    </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AC3">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -840,7 +843,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L4">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M4">
         <v>68.015751583500688</v>
@@ -862,14 +865,21 @@
         <v>1.7463157894736843</v>
       </c>
       <c r="U4">
-        <v>0.8</v>
+        <v>1.54</v>
       </c>
       <c r="X4">
         <f>(15.4+12.8)/2</f>
         <v>14.100000000000001</v>
       </c>
-    </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="AA4">
+        <v>1835.2610026544089</v>
+      </c>
+      <c r="AC4">
+        <f>AC3*(AA4/AA5)</f>
+        <v>1.5430393455280786</v>
+      </c>
+    </row>
+    <row r="5" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -904,7 +914,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L5">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M5">
         <v>68.015751583500688</v>
@@ -922,18 +932,22 @@
         <v>6.4829231993965921</v>
       </c>
       <c r="U5">
-        <f>27.3-19.2+V5</f>
-        <v>20.219148936170214</v>
+        <f>1+V5</f>
+        <v>14.98014184397163</v>
       </c>
       <c r="V5">
         <f>19.2*(X5/X4)</f>
-        <v>12.119148936170211</v>
+        <v>13.98014184397163</v>
       </c>
       <c r="X5">
-        <v>8.9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.35">
+        <f>(8.9+8.3+13.6)/3</f>
+        <v>10.266666666666667</v>
+      </c>
+      <c r="AA5">
+        <v>356.81416834377399</v>
+      </c>
+    </row>
+    <row r="6" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -968,7 +982,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L6">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M6">
         <v>68.015751583500688</v>
@@ -986,7 +1000,7 @@
         <v>6.4829231993965921</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -1021,7 +1035,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L7">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M7">
         <v>68.015751583500688</v>
@@ -1039,7 +1053,7 @@
         <v>6.4829231993965921</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -1074,7 +1088,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L8">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M8">
         <v>68.015751583500688</v>
@@ -1093,7 +1107,7 @@
       </c>
       <c r="R8">
         <f t="shared" ref="R8:R24" si="0">AA8</f>
-        <v>72.570716636937036</v>
+        <v>63.980350398411076</v>
       </c>
       <c r="S8" t="s">
         <v>70</v>
@@ -1112,14 +1126,14 @@
       </c>
       <c r="Z8">
         <f>((($U$4/$Y$22)*Y8)*$T$1)/$U$1</f>
-        <v>2.661780466724287</v>
+        <v>15.595839760113206</v>
       </c>
       <c r="AA8">
         <f>Z8+$U$2</f>
-        <v>72.570716636937036</v>
-      </c>
-    </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.35">
+        <v>63.980350398411076</v>
+      </c>
+    </row>
+    <row r="9" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -1154,7 +1168,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L9">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M9">
         <v>68.015751583500688</v>
@@ -1173,7 +1187,7 @@
       </c>
       <c r="R9">
         <f t="shared" si="0"/>
-        <v>71.074709722503158</v>
+        <v>55.214982852437224</v>
       </c>
       <c r="S9" t="s">
         <v>70</v>
@@ -1192,14 +1206,14 @@
       </c>
       <c r="Z9">
         <f t="shared" ref="Z9:Z24" si="1">((($U$4/$Y$22)*Y9)*$T$1)/$U$1</f>
-        <v>1.1657735522904062</v>
+        <v>6.8304722141393563</v>
       </c>
       <c r="AA9">
         <f t="shared" ref="AA9:AA24" si="2">Z9+$U$2</f>
-        <v>71.074709722503158</v>
-      </c>
-    </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.35">
+        <v>55.214982852437224</v>
+      </c>
+    </row>
+    <row r="10" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1234,7 +1248,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L10">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M10">
         <v>68.015751583500688</v>
@@ -1253,7 +1267,7 @@
       </c>
       <c r="R10">
         <f t="shared" si="0"/>
-        <v>70.338737380238683</v>
+        <v>50.902791497318645</v>
       </c>
       <c r="S10" t="s">
         <v>70</v>
@@ -1272,14 +1286,14 @@
       </c>
       <c r="Z10">
         <f t="shared" si="1"/>
-        <v>0.42980121002592919</v>
+        <v>2.5182808590207735</v>
       </c>
       <c r="AA10">
         <f t="shared" si="2"/>
-        <v>70.338737380238683</v>
-      </c>
-    </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.35">
+        <v>50.902791497318645</v>
+      </c>
+    </row>
+    <row r="11" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1314,7 +1328,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L11">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M11">
         <v>68.015751583500688</v>
@@ -1333,7 +1347,7 @@
       </c>
       <c r="R11">
         <f t="shared" si="0"/>
-        <v>70.936974199599092</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="S11" t="s">
         <v>70</v>
@@ -1348,18 +1362,18 @@
         <v>1239</v>
       </c>
       <c r="Y11">
-        <v>1993.9778328888817</v>
+        <v>1835.2610026544089</v>
       </c>
       <c r="Z11">
         <f t="shared" si="1"/>
-        <v>1.028038029386344</v>
+        <v>5.5439999999999996</v>
       </c>
       <c r="AA11">
         <f t="shared" si="2"/>
-        <v>70.936974199599092</v>
-      </c>
-    </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.35">
+        <v>53.928510638297865</v>
+      </c>
+    </row>
+    <row r="12" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1394,7 +1408,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L12">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M12">
         <v>68.015751583500688</v>
@@ -1413,7 +1427,7 @@
       </c>
       <c r="R12">
         <f t="shared" si="0"/>
-        <v>70.952739108847155</v>
+        <v>54.500335581634033</v>
       </c>
       <c r="S12" t="s">
         <v>70</v>
@@ -1432,14 +1446,14 @@
       </c>
       <c r="Z12">
         <f t="shared" si="1"/>
-        <v>1.0438029386343994</v>
+        <v>6.1158249433361638</v>
       </c>
       <c r="AA12">
         <f t="shared" si="2"/>
-        <v>70.952739108847155</v>
-      </c>
-    </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.35">
+        <v>54.500335581634033</v>
+      </c>
+    </row>
+    <row r="13" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -1474,7 +1488,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L13">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M13">
         <v>68.015751583500688</v>
@@ -1493,7 +1507,7 @@
       </c>
       <c r="R13">
         <f t="shared" si="0"/>
-        <v>73.345686386288818</v>
+        <v>68.521034418344286</v>
       </c>
       <c r="S13" t="s">
         <v>70</v>
@@ -1512,14 +1526,14 @@
       </c>
       <c r="Z13">
         <f t="shared" si="1"/>
-        <v>3.4367502160760592</v>
+        <v>20.136523780046414</v>
       </c>
       <c r="AA13">
         <f t="shared" si="2"/>
-        <v>73.345686386288818</v>
-      </c>
-    </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.35">
+        <v>68.521034418344286</v>
+      </c>
+    </row>
+    <row r="14" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -1554,7 +1568,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L14">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M14">
         <v>68.015751583500688</v>
@@ -1573,7 +1587,7 @@
       </c>
       <c r="R14">
         <f t="shared" si="0"/>
-        <v>72.625478953272392</v>
+        <v>64.301212438363535</v>
       </c>
       <c r="S14" t="s">
         <v>70</v>
@@ -1592,14 +1606,14 @@
       </c>
       <c r="Z14">
         <f t="shared" si="1"/>
-        <v>2.7165427830596371</v>
+        <v>15.916701800065661</v>
       </c>
       <c r="AA14">
         <f t="shared" si="2"/>
-        <v>72.625478953272392</v>
-      </c>
-    </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.35">
+        <v>64.301212438363535</v>
+      </c>
+    </row>
+    <row r="15" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -1634,7 +1648,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L15">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M15">
         <v>68.015751583500688</v>
@@ -1653,7 +1667,7 @@
       </c>
       <c r="R15">
         <f t="shared" si="0"/>
-        <v>73.091788374188553</v>
+        <v>67.03340132401928</v>
       </c>
       <c r="S15" t="s">
         <v>70</v>
@@ -1672,14 +1686,14 @@
       </c>
       <c r="Z15">
         <f t="shared" si="1"/>
-        <v>3.1828522039757998</v>
+        <v>18.648890685721405</v>
       </c>
       <c r="AA15">
         <f t="shared" si="2"/>
-        <v>73.091788374188553</v>
-      </c>
-    </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.35">
+        <v>67.03340132401928</v>
+      </c>
+    </row>
+    <row r="16" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -1714,7 +1728,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L16">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M16">
         <v>68.015751583500688</v>
@@ -1733,7 +1747,7 @@
       </c>
       <c r="R16">
         <f t="shared" si="0"/>
-        <v>71.636438330973348</v>
+        <v>58.506249534979816</v>
       </c>
       <c r="S16" t="s">
         <v>70</v>
@@ -1752,11 +1766,11 @@
       </c>
       <c r="Z16">
         <f t="shared" si="1"/>
-        <v>1.7275021607605878</v>
+        <v>10.121738896681949</v>
       </c>
       <c r="AA16">
         <f t="shared" si="2"/>
-        <v>71.636438330973348</v>
+        <v>58.506249534979816</v>
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.35">
@@ -1794,7 +1808,7 @@
         <v>67.958745558473652</v>
       </c>
       <c r="L17">
-        <v>67.958745558473652</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M17">
         <v>67.958745558473652</v>
@@ -1813,7 +1827,7 @@
       </c>
       <c r="R17">
         <f t="shared" si="0"/>
-        <v>71.316161753618118</v>
+        <v>56.629692755863957</v>
       </c>
       <c r="S17" t="s">
         <v>70</v>
@@ -1832,11 +1846,11 @@
       </c>
       <c r="Z17">
         <f t="shared" si="1"/>
-        <v>1.4072255834053586</v>
+        <v>8.2451821175660847</v>
       </c>
       <c r="AA17">
         <f t="shared" si="2"/>
-        <v>71.316161753618118</v>
+        <v>56.629692755863957</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.35">
@@ -1874,7 +1888,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L18">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M18">
         <v>68.015751583500688</v>
@@ -1893,7 +1907,7 @@
       </c>
       <c r="R18">
         <f t="shared" si="0"/>
-        <v>70.50800272163886</v>
+        <v>51.89454689353532</v>
       </c>
       <c r="S18" t="s">
         <v>70</v>
@@ -1912,11 +1926,11 @@
       </c>
       <c r="Z18">
         <f t="shared" si="1"/>
-        <v>0.5990665514261021</v>
+        <v>3.5100362552374489</v>
       </c>
       <c r="AA18">
         <f t="shared" si="2"/>
-        <v>70.50800272163886</v>
+        <v>51.89454689353532</v>
       </c>
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.35">
@@ -1954,7 +1968,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L19">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M19">
         <v>68.015751583500688</v>
@@ -1973,7 +1987,7 @@
       </c>
       <c r="R19">
         <f t="shared" si="0"/>
-        <v>72.320967285165224</v>
+        <v>62.51702503438549</v>
       </c>
       <c r="S19" t="s">
         <v>70</v>
@@ -1992,11 +2006,11 @@
       </c>
       <c r="Z19">
         <f t="shared" si="1"/>
-        <v>2.4120311149524638</v>
+        <v>14.132514396087624</v>
       </c>
       <c r="AA19">
         <f t="shared" si="2"/>
-        <v>72.320967285165224</v>
+        <v>62.51702503438549</v>
       </c>
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.35">
@@ -2034,7 +2048,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L20">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M20">
         <v>68.015751583500688</v>
@@ -2053,7 +2067,7 @@
       </c>
       <c r="R20">
         <f t="shared" si="0"/>
-        <v>73.521589584214482</v>
+        <v>69.551682183040043</v>
       </c>
       <c r="S20" t="s">
         <v>70</v>
@@ -2072,11 +2086,11 @@
       </c>
       <c r="Z20">
         <f t="shared" si="1"/>
-        <v>3.6126534140017288</v>
+        <v>21.167171544742178</v>
       </c>
       <c r="AA20">
         <f t="shared" si="2"/>
-        <v>73.521589584214482</v>
+        <v>69.551682183040043</v>
       </c>
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.35">
@@ -2114,7 +2128,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L21">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M21">
         <v>68.015751583500688</v>
@@ -2133,7 +2147,7 @@
       </c>
       <c r="R21">
         <f t="shared" si="0"/>
-        <v>73.521589584214482</v>
+        <v>69.551682183040043</v>
       </c>
       <c r="S21" t="s">
         <v>70</v>
@@ -2152,11 +2166,11 @@
       </c>
       <c r="Z21">
         <f t="shared" si="1"/>
-        <v>3.6126534140017288</v>
+        <v>21.167171544742178</v>
       </c>
       <c r="AA21">
         <f t="shared" si="2"/>
-        <v>73.521589584214482</v>
+        <v>69.551682183040043</v>
       </c>
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.35">
@@ -2194,7 +2208,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L22">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M22">
         <v>68.015751583500688</v>
@@ -2213,7 +2227,7 @@
       </c>
       <c r="R22">
         <f t="shared" si="0"/>
-        <v>72.78893617021275</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="S22" t="s">
         <v>70</v>
@@ -2228,15 +2242,15 @@
         <v>3471</v>
       </c>
       <c r="Y22">
-        <v>5586.0347521850754</v>
+        <v>1835.2610026544089</v>
       </c>
       <c r="Z22">
         <f>((($U$4/$Y$22)*Y22)*$T$1)/$U$1</f>
-        <v>2.88</v>
+        <v>5.5439999999999996</v>
       </c>
       <c r="AA22">
         <f t="shared" si="2"/>
-        <v>72.78893617021275</v>
+        <v>53.928510638297865</v>
       </c>
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.35">
@@ -2274,7 +2288,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L23">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M23">
         <v>68.015751583500688</v>
@@ -2293,7 +2307,7 @@
       </c>
       <c r="R23">
         <f t="shared" si="0"/>
-        <v>72.405599955865299</v>
+        <v>63.012902732493828</v>
       </c>
       <c r="S23" t="s">
         <v>70</v>
@@ -2312,11 +2326,11 @@
       </c>
       <c r="Z23">
         <f t="shared" si="1"/>
-        <v>2.49666378565255</v>
+        <v>14.628392094195959</v>
       </c>
       <c r="AA23">
         <f t="shared" si="2"/>
-        <v>72.405599955865299</v>
+        <v>63.012902732493828</v>
       </c>
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.35">
@@ -2354,7 +2368,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L24">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M24">
         <v>68.015751583500688</v>
@@ -2373,7 +2387,7 @@
       </c>
       <c r="R24">
         <f t="shared" si="0"/>
-        <v>73.471805660273262</v>
+        <v>69.25998941944691</v>
       </c>
       <c r="S24" t="s">
         <v>70</v>
@@ -2392,11 +2406,11 @@
       </c>
       <c r="Z24">
         <f t="shared" si="1"/>
-        <v>3.5628694900605016</v>
+        <v>20.875478781149038</v>
       </c>
       <c r="AA24">
         <f t="shared" si="2"/>
-        <v>73.471805660273262</v>
+        <v>69.25998941944691</v>
       </c>
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.35">
@@ -2434,7 +2448,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L25">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M25">
         <v>68.015751583500688</v>
@@ -2453,7 +2467,7 @@
       </c>
       <c r="R25">
         <f>AVERAGE(R8:R24)</f>
-        <v>72.142818929885323</v>
+        <v>60.778523560229964</v>
       </c>
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.35">
@@ -2491,7 +2505,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L26">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M26">
         <v>68.015751583500688</v>
@@ -2510,7 +2524,7 @@
       </c>
       <c r="Y26">
         <f>7.8/Y22</f>
-        <v>1.3963393258426995E-3</v>
+        <v>4.250076685941977E-3</v>
       </c>
     </row>
     <row r="27" spans="1:27" x14ac:dyDescent="0.35">
@@ -2548,7 +2562,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L27">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M27">
         <v>68.015751583500688</v>
@@ -2607,7 +2621,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L28">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M28">
         <v>68.015751583500688</v>
@@ -2629,7 +2643,7 @@
       </c>
       <c r="Y28">
         <f>Y27*Y26</f>
-        <v>1.3963393258426995</v>
+        <v>4.250076685941977</v>
       </c>
     </row>
     <row r="29" spans="1:27" x14ac:dyDescent="0.35">
@@ -2667,7 +2681,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L29">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M29">
         <v>68.015751583500688</v>
@@ -2720,7 +2734,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L30">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M30">
         <v>68.015751583500688</v>
@@ -2773,7 +2787,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L31">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M31">
         <v>68.015751583500688</v>
@@ -2834,7 +2848,7 @@
         <v>68.072757608527724</v>
       </c>
       <c r="L32">
-        <v>68.072757608527724</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M32">
         <v>68.072757608527724</v>
@@ -2887,7 +2901,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L33">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M33">
         <v>68.015751583500688</v>
@@ -2940,7 +2954,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L34">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M34">
         <v>68.015751583500688</v>
@@ -2993,7 +3007,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L35">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M35">
         <v>68.015751583500688</v>
@@ -3046,7 +3060,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L36">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M36">
         <v>68.015751583500688</v>
@@ -3099,7 +3113,7 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L37">
-        <v>68.015751583500688</v>
+        <v>53.928510638297865</v>
       </c>
       <c r="M37">
         <v>68.015751583500688</v>

</xml_diff>

<commit_message>
update LNG import emissions from TN
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
+++ b/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD580442-770A-48A5-AFA9-BADEAD102BAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3E25FDE-A2D7-4255-8A37-70C7DED942EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BAA9D55F-0FEB-4558-AFDF-92239B956412}"/>
   </bookViews>
@@ -722,10 +722,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L2">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M2">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N2">
         <v>68.015751583500688</v>
@@ -740,16 +740,16 @@
         <v>6.4829231993965921</v>
       </c>
       <c r="S2">
-        <f>U5-U4</f>
-        <v>13.440141843971631</v>
+        <f>U5</f>
+        <v>14.98014184397163</v>
       </c>
       <c r="T2">
         <f>S2*T1</f>
-        <v>48384510.638297871</v>
+        <v>53928510.638297871</v>
       </c>
       <c r="U2">
         <f>T2/U1</f>
-        <v>48.384510638297868</v>
+        <v>53.928510638297873</v>
       </c>
     </row>
     <row r="3" spans="1:29" x14ac:dyDescent="0.35">
@@ -787,10 +787,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L3">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M3">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N3">
         <v>68.015751583500688</v>
@@ -805,7 +805,7 @@
         <v>6.4829231993965921</v>
       </c>
       <c r="AC3">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.35">
@@ -843,10 +843,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L4">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M4">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N4">
         <v>68.015751583500688</v>
@@ -865,18 +865,18 @@
         <v>1.7463157894736843</v>
       </c>
       <c r="U4">
-        <v>1.54</v>
+        <v>1.43</v>
       </c>
       <c r="X4">
         <f>(15.4+12.8)/2</f>
         <v>14.100000000000001</v>
       </c>
       <c r="AA4">
-        <v>1835.2610026544089</v>
+        <v>1017.950789285221</v>
       </c>
       <c r="AC4">
         <f>AC3*(AA4/AA5)</f>
-        <v>1.5430393455280786</v>
+        <v>1.42644390217217</v>
       </c>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.35">
@@ -914,10 +914,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L5">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M5">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N5">
         <v>68.015751583500688</v>
@@ -982,10 +982,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L6">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M6">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N6">
         <v>68.015751583500688</v>
@@ -1035,10 +1035,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L7">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M7">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N7">
         <v>68.015751583500688</v>
@@ -1088,10 +1088,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L8">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M8">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N8">
         <v>68.015751583500688</v>
@@ -1107,7 +1107,7 @@
       </c>
       <c r="R8">
         <f t="shared" ref="R8:R24" si="0">AA8</f>
-        <v>63.980350398411076</v>
+        <v>68.410361844117276</v>
       </c>
       <c r="S8" t="s">
         <v>70</v>
@@ -1126,11 +1126,11 @@
       </c>
       <c r="Z8">
         <f>((($U$4/$Y$22)*Y8)*$T$1)/$U$1</f>
-        <v>15.595839760113206</v>
+        <v>14.481851205819403</v>
       </c>
       <c r="AA8">
         <f>Z8+$U$2</f>
-        <v>63.980350398411076</v>
+        <v>68.410361844117276</v>
       </c>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.35">
@@ -1168,10 +1168,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L9">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M9">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N9">
         <v>68.015751583500688</v>
@@ -1187,7 +1187,7 @@
       </c>
       <c r="R9">
         <f t="shared" si="0"/>
-        <v>55.214982852437224</v>
+        <v>60.271091979998701</v>
       </c>
       <c r="S9" t="s">
         <v>70</v>
@@ -1206,11 +1206,11 @@
       </c>
       <c r="Z9">
         <f t="shared" ref="Z9:Z24" si="1">((($U$4/$Y$22)*Y9)*$T$1)/$U$1</f>
-        <v>6.8304722141393563</v>
+        <v>6.3425813417008294</v>
       </c>
       <c r="AA9">
         <f t="shared" ref="AA9:AA24" si="2">Z9+$U$2</f>
-        <v>55.214982852437224</v>
+        <v>60.271091979998701</v>
       </c>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.35">
@@ -1248,10 +1248,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L10">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M10">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N10">
         <v>68.015751583500688</v>
@@ -1267,7 +1267,7 @@
       </c>
       <c r="R10">
         <f t="shared" si="0"/>
-        <v>50.902791497318645</v>
+        <v>56.266914293102879</v>
       </c>
       <c r="S10" t="s">
         <v>70</v>
@@ -1286,11 +1286,11 @@
       </c>
       <c r="Z10">
         <f t="shared" si="1"/>
-        <v>2.5182808590207735</v>
+        <v>2.3384036548050036</v>
       </c>
       <c r="AA10">
         <f t="shared" si="2"/>
-        <v>50.902791497318645</v>
+        <v>56.266914293102879</v>
       </c>
     </row>
     <row r="11" spans="1:29" x14ac:dyDescent="0.35">
@@ -1328,10 +1328,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L11">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M11">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N11">
         <v>68.015751583500688</v>
@@ -1347,7 +1347,7 @@
       </c>
       <c r="R11">
         <f t="shared" si="0"/>
-        <v>53.928510638297865</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="S11" t="s">
         <v>70</v>
@@ -1366,11 +1366,11 @@
       </c>
       <c r="Z11">
         <f t="shared" si="1"/>
-        <v>5.5439999999999996</v>
+        <v>5.1479999999999997</v>
       </c>
       <c r="AA11">
         <f t="shared" si="2"/>
-        <v>53.928510638297865</v>
+        <v>59.076510638297876</v>
       </c>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.35">
@@ -1408,10 +1408,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L12">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M12">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N12">
         <v>68.015751583500688</v>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="R12">
         <f t="shared" si="0"/>
-        <v>54.500335581634033</v>
+        <v>59.607490942824313</v>
       </c>
       <c r="S12" t="s">
         <v>70</v>
@@ -1446,11 +1446,11 @@
       </c>
       <c r="Z12">
         <f t="shared" si="1"/>
-        <v>6.1158249433361638</v>
+        <v>5.6789803045264371</v>
       </c>
       <c r="AA12">
         <f t="shared" si="2"/>
-        <v>54.500335581634033</v>
+        <v>59.607490942824313</v>
       </c>
     </row>
     <row r="13" spans="1:29" x14ac:dyDescent="0.35">
@@ -1488,10 +1488,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L13">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M13">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N13">
         <v>68.015751583500688</v>
@@ -1507,7 +1507,7 @@
       </c>
       <c r="R13">
         <f t="shared" si="0"/>
-        <v>68.521034418344286</v>
+        <v>72.62671129119812</v>
       </c>
       <c r="S13" t="s">
         <v>70</v>
@@ -1526,11 +1526,11 @@
       </c>
       <c r="Z13">
         <f t="shared" si="1"/>
-        <v>20.136523780046414</v>
+        <v>18.69820065290024</v>
       </c>
       <c r="AA13">
         <f t="shared" si="2"/>
-        <v>68.521034418344286</v>
+        <v>72.62671129119812</v>
       </c>
     </row>
     <row r="14" spans="1:29" x14ac:dyDescent="0.35">
@@ -1568,10 +1568,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L14">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M14">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N14">
         <v>68.015751583500688</v>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="R14">
         <f t="shared" si="0"/>
-        <v>64.301212438363535</v>
+        <v>68.708305166930273</v>
       </c>
       <c r="S14" t="s">
         <v>70</v>
@@ -1606,11 +1606,11 @@
       </c>
       <c r="Z14">
         <f t="shared" si="1"/>
-        <v>15.916701800065661</v>
+        <v>14.779794528632396</v>
       </c>
       <c r="AA14">
         <f t="shared" si="2"/>
-        <v>64.301212438363535</v>
+        <v>68.708305166930273</v>
       </c>
     </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.35">
@@ -1648,10 +1648,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L15">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M15">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N15">
         <v>68.015751583500688</v>
@@ -1667,7 +1667,7 @@
       </c>
       <c r="R15">
         <f t="shared" si="0"/>
-        <v>67.03340132401928</v>
+        <v>71.245337703610602</v>
       </c>
       <c r="S15" t="s">
         <v>70</v>
@@ -1686,11 +1686,11 @@
       </c>
       <c r="Z15">
         <f t="shared" si="1"/>
-        <v>18.648890685721405</v>
+        <v>17.316827065312733</v>
       </c>
       <c r="AA15">
         <f t="shared" si="2"/>
-        <v>67.03340132401928</v>
+        <v>71.245337703610602</v>
       </c>
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.35">
@@ -1728,10 +1728,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L16">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M16">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N16">
         <v>68.015751583500688</v>
@@ -1747,7 +1747,7 @@
       </c>
       <c r="R16">
         <f t="shared" si="0"/>
-        <v>58.506249534979816</v>
+        <v>63.327268185216823</v>
       </c>
       <c r="S16" t="s">
         <v>70</v>
@@ -1766,11 +1766,11 @@
       </c>
       <c r="Z16">
         <f t="shared" si="1"/>
-        <v>10.121738896681949</v>
+        <v>9.3987575469189508</v>
       </c>
       <c r="AA16">
         <f t="shared" si="2"/>
-        <v>58.506249534979816</v>
+        <v>63.327268185216823</v>
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.35">
@@ -1808,10 +1808,10 @@
         <v>67.958745558473652</v>
       </c>
       <c r="L17">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M17">
-        <v>67.958745558473652</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N17">
         <v>67.958745558473652</v>
@@ -1827,7 +1827,7 @@
       </c>
       <c r="R17">
         <f t="shared" si="0"/>
-        <v>56.629692755863957</v>
+        <v>61.584751176037805</v>
       </c>
       <c r="S17" t="s">
         <v>70</v>
@@ -1846,11 +1846,11 @@
       </c>
       <c r="Z17">
         <f t="shared" si="1"/>
-        <v>8.2451821175660847</v>
+        <v>7.6562405377399356</v>
       </c>
       <c r="AA17">
         <f t="shared" si="2"/>
-        <v>56.629692755863957</v>
+        <v>61.584751176037805</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.35">
@@ -1888,10 +1888,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L18">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M18">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N18">
         <v>68.015751583500688</v>
@@ -1907,7 +1907,7 @@
       </c>
       <c r="R18">
         <f t="shared" si="0"/>
-        <v>51.89454689353532</v>
+        <v>57.187830018161215</v>
       </c>
       <c r="S18" t="s">
         <v>70</v>
@@ -1926,11 +1926,11 @@
       </c>
       <c r="Z18">
         <f t="shared" si="1"/>
-        <v>3.5100362552374489</v>
+        <v>3.2593193798633444</v>
       </c>
       <c r="AA18">
         <f t="shared" si="2"/>
-        <v>51.89454689353532</v>
+        <v>57.187830018161215</v>
       </c>
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.35">
@@ -1968,10 +1968,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L19">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M19">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N19">
         <v>68.015751583500688</v>
@@ -1987,7 +1987,7 @@
       </c>
       <c r="R19">
         <f t="shared" si="0"/>
-        <v>62.51702503438549</v>
+        <v>67.051559720379231</v>
       </c>
       <c r="S19" t="s">
         <v>70</v>
@@ -2006,11 +2006,11 @@
       </c>
       <c r="Z19">
         <f t="shared" si="1"/>
-        <v>14.132514396087624</v>
+        <v>13.123049082081362</v>
       </c>
       <c r="AA19">
         <f t="shared" si="2"/>
-        <v>62.51702503438549</v>
+        <v>67.051559720379231</v>
       </c>
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.35">
@@ -2048,10 +2048,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L20">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M20">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N20">
         <v>68.015751583500688</v>
@@ -2067,7 +2067,7 @@
       </c>
       <c r="R20">
         <f t="shared" si="0"/>
-        <v>69.551682183040043</v>
+        <v>73.583741358415608</v>
       </c>
       <c r="S20" t="s">
         <v>70</v>
@@ -2086,11 +2086,11 @@
       </c>
       <c r="Z20">
         <f t="shared" si="1"/>
-        <v>21.167171544742178</v>
+        <v>19.655230720117729</v>
       </c>
       <c r="AA20">
         <f t="shared" si="2"/>
-        <v>69.551682183040043</v>
+        <v>73.583741358415608</v>
       </c>
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.35">
@@ -2128,10 +2128,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L21">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M21">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N21">
         <v>68.015751583500688</v>
@@ -2147,7 +2147,7 @@
       </c>
       <c r="R21">
         <f t="shared" si="0"/>
-        <v>69.551682183040043</v>
+        <v>73.583741358415608</v>
       </c>
       <c r="S21" t="s">
         <v>70</v>
@@ -2166,11 +2166,11 @@
       </c>
       <c r="Z21">
         <f t="shared" si="1"/>
-        <v>21.167171544742178</v>
+        <v>19.655230720117729</v>
       </c>
       <c r="AA21">
         <f t="shared" si="2"/>
-        <v>69.551682183040043</v>
+        <v>73.583741358415608</v>
       </c>
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.35">
@@ -2208,10 +2208,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L22">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M22">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N22">
         <v>68.015751583500688</v>
@@ -2227,7 +2227,7 @@
       </c>
       <c r="R22">
         <f t="shared" si="0"/>
-        <v>53.928510638297865</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="S22" t="s">
         <v>70</v>
@@ -2246,11 +2246,11 @@
       </c>
       <c r="Z22">
         <f>((($U$4/$Y$22)*Y22)*$T$1)/$U$1</f>
-        <v>5.5439999999999996</v>
+        <v>5.1479999999999997</v>
       </c>
       <c r="AA22">
         <f t="shared" si="2"/>
-        <v>53.928510638297865</v>
+        <v>59.076510638297876</v>
       </c>
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.35">
@@ -2288,10 +2288,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L23">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M23">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N23">
         <v>68.015751583500688</v>
@@ -2307,7 +2307,7 @@
       </c>
       <c r="R23">
         <f t="shared" si="0"/>
-        <v>63.012902732493828</v>
+        <v>67.512017582908399</v>
       </c>
       <c r="S23" t="s">
         <v>70</v>
@@ -2326,11 +2326,11 @@
       </c>
       <c r="Z23">
         <f t="shared" si="1"/>
-        <v>14.628392094195959</v>
+        <v>13.583506944610532</v>
       </c>
       <c r="AA23">
         <f t="shared" si="2"/>
-        <v>63.012902732493828</v>
+        <v>67.512017582908399</v>
       </c>
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.35">
@@ -2368,10 +2368,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L24">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M24">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N24">
         <v>68.015751583500688</v>
@@ -2387,7 +2387,7 @@
       </c>
       <c r="R24">
         <f t="shared" si="0"/>
-        <v>69.25998941944691</v>
+        <v>73.312883792221967</v>
       </c>
       <c r="S24" t="s">
         <v>70</v>
@@ -2406,11 +2406,11 @@
       </c>
       <c r="Z24">
         <f t="shared" si="1"/>
-        <v>20.875478781149038</v>
+        <v>19.384373153924098</v>
       </c>
       <c r="AA24">
         <f t="shared" si="2"/>
-        <v>69.25998941944691</v>
+        <v>73.312883792221967</v>
       </c>
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.35">
@@ -2448,10 +2448,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L25">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M25">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N25">
         <v>68.015751583500688</v>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="R25">
         <f>AVERAGE(R8:R24)</f>
-        <v>60.778523560229964</v>
+        <v>65.437236922949097</v>
       </c>
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.35">
@@ -2505,10 +2505,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L26">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M26">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N26">
         <v>68.015751583500688</v>
@@ -2562,10 +2562,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L27">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M27">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N27">
         <v>68.015751583500688</v>
@@ -2621,10 +2621,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L28">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M28">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N28">
         <v>68.015751583500688</v>
@@ -2681,10 +2681,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L29">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M29">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N29">
         <v>68.015751583500688</v>
@@ -2734,10 +2734,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L30">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M30">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N30">
         <v>68.015751583500688</v>
@@ -2787,10 +2787,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L31">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M31">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N31">
         <v>68.015751583500688</v>
@@ -2848,10 +2848,10 @@
         <v>68.072757608527724</v>
       </c>
       <c r="L32">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M32">
-        <v>68.072757608527724</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N32">
         <v>68.072757608527724</v>
@@ -2901,10 +2901,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L33">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M33">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N33">
         <v>68.015751583500688</v>
@@ -2954,10 +2954,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L34">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M34">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N34">
         <v>68.015751583500688</v>
@@ -3007,10 +3007,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L35">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M35">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N35">
         <v>68.015751583500688</v>
@@ -3060,10 +3060,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L36">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M36">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N36">
         <v>68.015751583500688</v>
@@ -3113,10 +3113,10 @@
         <v>68.015751583500688</v>
       </c>
       <c r="L37">
-        <v>53.928510638297865</v>
+        <v>59.472510638297869</v>
       </c>
       <c r="M37">
-        <v>68.015751583500688</v>
+        <v>59.076510638297876</v>
       </c>
       <c r="N37">
         <v>68.015751583500688</v>

</xml_diff>

<commit_message>
update LNG import emissions from MA
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
+++ b/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3E25FDE-A2D7-4255-8A37-70C7DED942EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{750AA016-7DC5-437F-AF69-47D5C8E6FB30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BAA9D55F-0FEB-4558-AFDF-92239B956412}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="53">
   <si>
     <t>AL</t>
   </si>
@@ -196,60 +196,6 @@
   </si>
   <si>
     <t>Node</t>
-  </si>
-  <si>
-    <t>BE_LNG</t>
-  </si>
-  <si>
-    <t>FR_LNG</t>
-  </si>
-  <si>
-    <t>EL_LNG</t>
-  </si>
-  <si>
-    <t>IT_LNG</t>
-  </si>
-  <si>
-    <t>HR_LNG</t>
-  </si>
-  <si>
-    <t>LT_LNG</t>
-  </si>
-  <si>
-    <t>NL_LNG</t>
-  </si>
-  <si>
-    <t>PL_LNG</t>
-  </si>
-  <si>
-    <t>PT_LNG</t>
-  </si>
-  <si>
-    <t>ES_LNG</t>
-  </si>
-  <si>
-    <t>TR_LNG</t>
-  </si>
-  <si>
-    <t>UK_LNG</t>
-  </si>
-  <si>
-    <t>EE_LNG</t>
-  </si>
-  <si>
-    <t>FI_LNG</t>
-  </si>
-  <si>
-    <t>DE_LNG</t>
-  </si>
-  <si>
-    <t>IE_LNG</t>
-  </si>
-  <si>
-    <t>LV_LNG</t>
-  </si>
-  <si>
-    <t>EG_LNG</t>
   </si>
 </sst>
 </file>
@@ -621,13 +567,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6177B6A9-4CD7-49C9-8407-62B26396811D}">
-  <dimension ref="A1:AC37"/>
+  <dimension ref="A1:Q37"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="26" max="26" width="11.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>52</v>
       </c>
@@ -679,15 +625,8 @@
       <c r="Q1" t="s">
         <v>22</v>
       </c>
-      <c r="T1">
-        <v>3600000</v>
-      </c>
-      <c r="U1">
-        <f>1000*1000</f>
-        <v>1000000</v>
-      </c>
-    </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -728,7 +667,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N2">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O2">
         <v>72.142818929885323</v>
@@ -739,20 +678,8 @@
       <c r="Q2">
         <v>6.4829231993965921</v>
       </c>
-      <c r="S2">
-        <f>U5</f>
-        <v>14.98014184397163</v>
-      </c>
-      <c r="T2">
-        <f>S2*T1</f>
-        <v>53928510.638297871</v>
-      </c>
-      <c r="U2">
-        <f>T2/U1</f>
-        <v>53.928510638297873</v>
-      </c>
-    </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -793,7 +720,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N3">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O3">
         <v>72.142818929885323</v>
@@ -804,11 +731,8 @@
       <c r="Q3">
         <v>6.4829231993965921</v>
       </c>
-      <c r="AC3">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -849,7 +773,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N4">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O4">
         <v>72.570716636937036</v>
@@ -860,26 +784,8 @@
       <c r="Q4">
         <v>6.5604478724514799</v>
       </c>
-      <c r="S4">
-        <f>(2.1/9500)*7900</f>
-        <v>1.7463157894736843</v>
-      </c>
-      <c r="U4">
-        <v>1.43</v>
-      </c>
-      <c r="X4">
-        <f>(15.4+12.8)/2</f>
-        <v>14.100000000000001</v>
-      </c>
-      <c r="AA4">
-        <v>1017.950789285221</v>
-      </c>
-      <c r="AC4">
-        <f>AC3*(AA4/AA5)</f>
-        <v>1.42644390217217</v>
-      </c>
-    </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -920,7 +826,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N5">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O5">
         <v>72.142818929885323</v>
@@ -931,23 +837,8 @@
       <c r="Q5">
         <v>6.4829231993965921</v>
       </c>
-      <c r="U5">
-        <f>1+V5</f>
-        <v>14.98014184397163</v>
-      </c>
-      <c r="V5">
-        <f>19.2*(X5/X4)</f>
-        <v>13.98014184397163</v>
-      </c>
-      <c r="X5">
-        <f>(8.9+8.3+13.6)/3</f>
-        <v>10.266666666666667</v>
-      </c>
-      <c r="AA5">
-        <v>356.81416834377399</v>
-      </c>
-    </row>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -988,7 +879,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N6">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O6">
         <v>72.142818929885323</v>
@@ -1000,7 +891,7 @@
         <v>6.4829231993965921</v>
       </c>
     </row>
-    <row r="7" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -1041,7 +932,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N7">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O7">
         <v>70.952739108847155</v>
@@ -1053,7 +944,7 @@
         <v>6.4829231993965921</v>
       </c>
     </row>
-    <row r="8" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -1094,7 +985,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N8">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O8">
         <v>72.142818929885323</v>
@@ -1105,35 +996,8 @@
       <c r="Q8">
         <v>6.4829231993965921</v>
       </c>
-      <c r="R8">
-        <f t="shared" ref="R8:R24" si="0">AA8</f>
-        <v>68.410361844117276</v>
-      </c>
-      <c r="S8" t="s">
-        <v>70</v>
-      </c>
-      <c r="T8" t="s">
-        <v>53</v>
-      </c>
-      <c r="W8">
-        <v>0</v>
-      </c>
-      <c r="X8">
-        <v>3208</v>
-      </c>
-      <c r="Y8">
-        <v>5162.7771492393322</v>
-      </c>
-      <c r="Z8">
-        <f>((($U$4/$Y$22)*Y8)*$T$1)/$U$1</f>
-        <v>14.481851205819403</v>
-      </c>
-      <c r="AA8">
-        <f>Z8+$U$2</f>
-        <v>68.410361844117276</v>
-      </c>
-    </row>
-    <row r="9" spans="1:29" x14ac:dyDescent="0.35">
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -1174,7 +1038,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N9">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O9">
         <v>72.142818929885323</v>
@@ -1185,35 +1049,8 @@
       <c r="Q9">
         <v>6.0724198318715077</v>
       </c>
-      <c r="R9">
-        <f t="shared" si="0"/>
-        <v>60.271091979998701</v>
-      </c>
-      <c r="S9" t="s">
-        <v>70</v>
-      </c>
-      <c r="T9" t="s">
-        <v>54</v>
-      </c>
-      <c r="W9">
-        <v>0</v>
-      </c>
-      <c r="X9">
-        <v>1405</v>
-      </c>
-      <c r="Y9">
-        <v>2261.1290195390466</v>
-      </c>
-      <c r="Z9">
-        <f t="shared" ref="Z9:Z24" si="1">((($U$4/$Y$22)*Y9)*$T$1)/$U$1</f>
-        <v>6.3425813417008294</v>
-      </c>
-      <c r="AA9">
-        <f t="shared" ref="AA9:AA24" si="2">Z9+$U$2</f>
-        <v>60.271091979998701</v>
-      </c>
-    </row>
-    <row r="10" spans="1:29" x14ac:dyDescent="0.35">
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1254,7 +1091,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N10">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O10">
         <v>73.521589584214482</v>
@@ -1265,35 +1102,8 @@
       <c r="Q10">
         <v>6.4829231993965921</v>
       </c>
-      <c r="R10">
-        <f t="shared" si="0"/>
-        <v>56.266914293102879</v>
-      </c>
-      <c r="S10" t="s">
-        <v>70</v>
-      </c>
-      <c r="T10" t="s">
-        <v>55</v>
-      </c>
-      <c r="W10">
-        <v>0</v>
-      </c>
-      <c r="X10">
-        <v>518</v>
-      </c>
-      <c r="Y10">
-        <v>833.64044990834611</v>
-      </c>
-      <c r="Z10">
-        <f t="shared" si="1"/>
-        <v>2.3384036548050036</v>
-      </c>
-      <c r="AA10">
-        <f t="shared" si="2"/>
-        <v>56.266914293102879</v>
-      </c>
-    </row>
-    <row r="11" spans="1:29" x14ac:dyDescent="0.35">
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1334,7 +1144,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N11">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O11">
         <v>73.521589584214482</v>
@@ -1345,35 +1155,8 @@
       <c r="Q11">
         <v>6.4829231993965921</v>
       </c>
-      <c r="R11">
-        <f t="shared" si="0"/>
-        <v>59.076510638297876</v>
-      </c>
-      <c r="S11" t="s">
-        <v>70</v>
-      </c>
-      <c r="T11" t="s">
-        <v>56</v>
-      </c>
-      <c r="W11">
-        <v>0</v>
-      </c>
-      <c r="X11">
-        <v>1239</v>
-      </c>
-      <c r="Y11">
-        <v>1835.2610026544089</v>
-      </c>
-      <c r="Z11">
-        <f t="shared" si="1"/>
-        <v>5.1479999999999997</v>
-      </c>
-      <c r="AA11">
-        <f t="shared" si="2"/>
-        <v>59.076510638297876</v>
-      </c>
-    </row>
-    <row r="12" spans="1:29" x14ac:dyDescent="0.35">
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1414,7 +1197,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N12">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O12">
         <v>71.074709722503158</v>
@@ -1425,35 +1208,8 @@
       <c r="Q12">
         <v>6.9190068562697657</v>
       </c>
-      <c r="R12">
-        <f t="shared" si="0"/>
-        <v>59.607490942824313</v>
-      </c>
-      <c r="S12" t="s">
-        <v>70</v>
-      </c>
-      <c r="T12" t="s">
-        <v>57</v>
-      </c>
-      <c r="W12">
-        <v>0</v>
-      </c>
-      <c r="X12">
-        <v>1258</v>
-      </c>
-      <c r="Y12">
-        <v>2024.5553783488403</v>
-      </c>
-      <c r="Z12">
-        <f t="shared" si="1"/>
-        <v>5.6789803045264371</v>
-      </c>
-      <c r="AA12">
-        <f t="shared" si="2"/>
-        <v>59.607490942824313</v>
-      </c>
-    </row>
-    <row r="13" spans="1:29" x14ac:dyDescent="0.35">
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -1494,7 +1250,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N13">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O13">
         <v>72.78893617021275</v>
@@ -1505,35 +1261,8 @@
       <c r="Q13">
         <v>6.48</v>
       </c>
-      <c r="R13">
-        <f t="shared" si="0"/>
-        <v>72.62671129119812</v>
-      </c>
-      <c r="S13" t="s">
-        <v>70</v>
-      </c>
-      <c r="T13" t="s">
-        <v>58</v>
-      </c>
-      <c r="W13">
-        <v>0</v>
-      </c>
-      <c r="X13">
-        <v>4142</v>
-      </c>
-      <c r="Y13">
-        <v>6665.9049102709832</v>
-      </c>
-      <c r="Z13">
-        <f t="shared" si="1"/>
-        <v>18.69820065290024</v>
-      </c>
-      <c r="AA13">
-        <f t="shared" si="2"/>
-        <v>72.62671129119812</v>
-      </c>
-    </row>
-    <row r="14" spans="1:29" x14ac:dyDescent="0.35">
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -1574,7 +1303,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N14">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O14">
         <v>70.338737380238683</v>
@@ -1585,35 +1314,8 @@
       <c r="Q14">
         <v>6.4829231993965921</v>
       </c>
-      <c r="R14">
-        <f t="shared" si="0"/>
-        <v>68.708305166930273</v>
-      </c>
-      <c r="S14" t="s">
-        <v>70</v>
-      </c>
-      <c r="T14" t="s">
-        <v>59</v>
-      </c>
-      <c r="W14">
-        <v>0</v>
-      </c>
-      <c r="X14">
-        <v>3274</v>
-      </c>
-      <c r="Y14">
-        <v>5268.9938861002411</v>
-      </c>
-      <c r="Z14">
-        <f t="shared" si="1"/>
-        <v>14.779794528632396</v>
-      </c>
-      <c r="AA14">
-        <f t="shared" si="2"/>
-        <v>68.708305166930273</v>
-      </c>
-    </row>
-    <row r="15" spans="1:29" x14ac:dyDescent="0.35">
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -1654,7 +1356,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N15">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O15">
         <v>72.142818929885323</v>
@@ -1665,35 +1367,8 @@
       <c r="Q15">
         <v>6.4829231993965921</v>
       </c>
-      <c r="R15">
-        <f t="shared" si="0"/>
-        <v>71.245337703610602</v>
-      </c>
-      <c r="S15" t="s">
-        <v>70</v>
-      </c>
-      <c r="T15" t="s">
-        <v>60</v>
-      </c>
-      <c r="W15">
-        <v>0</v>
-      </c>
-      <c r="X15">
-        <v>3836</v>
-      </c>
-      <c r="Y15">
-        <v>6173.4454939158604</v>
-      </c>
-      <c r="Z15">
-        <f t="shared" si="1"/>
-        <v>17.316827065312733</v>
-      </c>
-      <c r="AA15">
-        <f t="shared" si="2"/>
-        <v>71.245337703610602</v>
-      </c>
-    </row>
-    <row r="16" spans="1:29" x14ac:dyDescent="0.35">
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -1734,7 +1409,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N16">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O16">
         <v>72.405599955865299</v>
@@ -1745,35 +1420,8 @@
       <c r="Q16">
         <v>6.4829231993965921</v>
       </c>
-      <c r="R16">
-        <f t="shared" si="0"/>
-        <v>63.327268185216823</v>
-      </c>
-      <c r="S16" t="s">
-        <v>70</v>
-      </c>
-      <c r="T16" t="s">
-        <v>61</v>
-      </c>
-      <c r="W16">
-        <v>0</v>
-      </c>
-      <c r="X16">
-        <v>2082</v>
-      </c>
-      <c r="Y16">
-        <v>3350.6552446123096</v>
-      </c>
-      <c r="Z16">
-        <f t="shared" si="1"/>
-        <v>9.3987575469189508</v>
-      </c>
-      <c r="AA16">
-        <f t="shared" si="2"/>
-        <v>63.327268185216823</v>
-      </c>
-    </row>
-    <row r="17" spans="1:27" x14ac:dyDescent="0.35">
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -1814,7 +1462,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N17">
-        <v>67.958745558473652</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O17">
         <v>70.936974199599092</v>
@@ -1825,35 +1473,8 @@
       <c r="Q17">
         <v>6.4829231993965921</v>
       </c>
-      <c r="R17">
-        <f t="shared" si="0"/>
-        <v>61.584751176037805</v>
-      </c>
-      <c r="S17" t="s">
-        <v>70</v>
-      </c>
-      <c r="T17" t="s">
-        <v>62</v>
-      </c>
-      <c r="W17">
-        <v>0</v>
-      </c>
-      <c r="X17">
-        <v>1696</v>
-      </c>
-      <c r="Y17">
-        <v>2729.4482684257819</v>
-      </c>
-      <c r="Z17">
-        <f t="shared" si="1"/>
-        <v>7.6562405377399356</v>
-      </c>
-      <c r="AA17">
-        <f t="shared" si="2"/>
-        <v>61.584751176037805</v>
-      </c>
-    </row>
-    <row r="18" spans="1:27" x14ac:dyDescent="0.35">
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -1894,7 +1515,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N18">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O18">
         <v>73.471805660273262</v>
@@ -1905,35 +1526,8 @@
       <c r="Q18">
         <v>6.4829231993965921</v>
       </c>
-      <c r="R18">
-        <f t="shared" si="0"/>
-        <v>57.187830018161215</v>
-      </c>
-      <c r="S18" t="s">
-        <v>70</v>
-      </c>
-      <c r="T18" t="s">
-        <v>63</v>
-      </c>
-      <c r="W18">
-        <v>0</v>
-      </c>
-      <c r="X18">
-        <v>722</v>
-      </c>
-      <c r="Y18">
-        <v>1161.9467274784283</v>
-      </c>
-      <c r="Z18">
-        <f t="shared" si="1"/>
-        <v>3.2593193798633444</v>
-      </c>
-      <c r="AA18">
-        <f t="shared" si="2"/>
-        <v>57.187830018161215</v>
-      </c>
-    </row>
-    <row r="19" spans="1:27" x14ac:dyDescent="0.35">
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>17</v>
       </c>
@@ -1974,7 +1568,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N19">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O19">
         <v>73.345686386288818</v>
@@ -1985,35 +1579,8 @@
       <c r="Q19">
         <v>6.4829231993965921</v>
       </c>
-      <c r="R19">
-        <f t="shared" si="0"/>
-        <v>67.051559720379231</v>
-      </c>
-      <c r="S19" t="s">
-        <v>70</v>
-      </c>
-      <c r="T19" t="s">
-        <v>64</v>
-      </c>
-      <c r="W19">
-        <v>0</v>
-      </c>
-      <c r="X19">
-        <v>2907</v>
-      </c>
-      <c r="Y19">
-        <v>4678.3644553736722</v>
-      </c>
-      <c r="Z19">
-        <f t="shared" si="1"/>
-        <v>13.123049082081362</v>
-      </c>
-      <c r="AA19">
-        <f t="shared" si="2"/>
-        <v>67.051559720379231</v>
-      </c>
-    </row>
-    <row r="20" spans="1:27" x14ac:dyDescent="0.35">
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>18</v>
       </c>
@@ -2054,7 +1621,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N20">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O20">
         <v>72.142818929885323</v>
@@ -2065,35 +1632,8 @@
       <c r="Q20">
         <v>6.4829231993965921</v>
       </c>
-      <c r="R20">
-        <f t="shared" si="0"/>
-        <v>73.583741358415608</v>
-      </c>
-      <c r="S20" t="s">
-        <v>70</v>
-      </c>
-      <c r="T20" t="s">
-        <v>65</v>
-      </c>
-      <c r="W20">
-        <v>0</v>
-      </c>
-      <c r="X20">
-        <v>4354</v>
-      </c>
-      <c r="Y20">
-        <v>7007.085943824206</v>
-      </c>
-      <c r="Z20">
-        <f t="shared" si="1"/>
-        <v>19.655230720117729</v>
-      </c>
-      <c r="AA20">
-        <f t="shared" si="2"/>
-        <v>73.583741358415608</v>
-      </c>
-    </row>
-    <row r="21" spans="1:27" x14ac:dyDescent="0.35">
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -2134,7 +1674,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N21">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O21">
         <v>72.142818929885323</v>
@@ -2145,35 +1685,8 @@
       <c r="Q21">
         <v>6.4829231993965921</v>
       </c>
-      <c r="R21">
-        <f t="shared" si="0"/>
-        <v>73.583741358415608</v>
-      </c>
-      <c r="S21" t="s">
-        <v>70</v>
-      </c>
-      <c r="T21" t="s">
-        <v>66</v>
-      </c>
-      <c r="W21">
-        <v>0</v>
-      </c>
-      <c r="X21">
-        <v>4354</v>
-      </c>
-      <c r="Y21">
-        <v>7007.085943824206</v>
-      </c>
-      <c r="Z21">
-        <f t="shared" si="1"/>
-        <v>19.655230720117729</v>
-      </c>
-      <c r="AA21">
-        <f t="shared" si="2"/>
-        <v>73.583741358415608</v>
-      </c>
-    </row>
-    <row r="22" spans="1:27" x14ac:dyDescent="0.35">
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -2214,7 +1727,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N22">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O22">
         <v>72.625478953272392</v>
@@ -2225,35 +1738,8 @@
       <c r="Q22">
         <v>6.4181490433991044</v>
       </c>
-      <c r="R22">
-        <f t="shared" si="0"/>
-        <v>59.076510638297876</v>
-      </c>
-      <c r="S22" t="s">
-        <v>70</v>
-      </c>
-      <c r="T22" t="s">
-        <v>67</v>
-      </c>
-      <c r="W22">
-        <v>0</v>
-      </c>
-      <c r="X22">
-        <v>3471</v>
-      </c>
-      <c r="Y22">
-        <v>1835.2610026544089</v>
-      </c>
-      <c r="Z22">
-        <f>((($U$4/$Y$22)*Y22)*$T$1)/$U$1</f>
-        <v>5.1479999999999997</v>
-      </c>
-      <c r="AA22">
-        <f t="shared" si="2"/>
-        <v>59.076510638297876</v>
-      </c>
-    </row>
-    <row r="23" spans="1:27" x14ac:dyDescent="0.35">
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -2294,7 +1780,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N23">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O23">
         <v>72.142818929885323</v>
@@ -2305,35 +1791,8 @@
       <c r="Q23">
         <v>6.4829231993965921</v>
       </c>
-      <c r="R23">
-        <f t="shared" si="0"/>
-        <v>67.512017582908399</v>
-      </c>
-      <c r="S23" t="s">
-        <v>70</v>
-      </c>
-      <c r="T23" t="s">
-        <v>68</v>
-      </c>
-      <c r="W23">
-        <v>0</v>
-      </c>
-      <c r="X23">
-        <v>3009</v>
-      </c>
-      <c r="Y23">
-        <v>4842.5175941587131</v>
-      </c>
-      <c r="Z23">
-        <f t="shared" si="1"/>
-        <v>13.583506944610532</v>
-      </c>
-      <c r="AA23">
-        <f t="shared" si="2"/>
-        <v>67.512017582908399</v>
-      </c>
-    </row>
-    <row r="24" spans="1:27" x14ac:dyDescent="0.35">
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>22</v>
       </c>
@@ -2374,7 +1833,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N24">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O24">
         <v>72.142818929885323</v>
@@ -2385,35 +1844,8 @@
       <c r="Q24">
         <v>5.4</v>
       </c>
-      <c r="R24">
-        <f t="shared" si="0"/>
-        <v>73.312883792221967</v>
-      </c>
-      <c r="S24" t="s">
-        <v>70</v>
-      </c>
-      <c r="T24" t="s">
-        <v>69</v>
-      </c>
-      <c r="W24">
-        <v>0</v>
-      </c>
-      <c r="X24">
-        <v>4294</v>
-      </c>
-      <c r="Y24">
-        <v>6910.5252739506523</v>
-      </c>
-      <c r="Z24">
-        <f t="shared" si="1"/>
-        <v>19.384373153924098</v>
-      </c>
-      <c r="AA24">
-        <f t="shared" si="2"/>
-        <v>73.312883792221967</v>
-      </c>
-    </row>
-    <row r="25" spans="1:27" x14ac:dyDescent="0.35">
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -2454,7 +1886,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N25">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O25">
         <v>73.091788374188553</v>
@@ -2465,12 +1897,8 @@
       <c r="Q25">
         <v>6.4829231993965921</v>
       </c>
-      <c r="R25">
-        <f>AVERAGE(R8:R24)</f>
-        <v>65.437236922949097</v>
-      </c>
-    </row>
-    <row r="26" spans="1:27" x14ac:dyDescent="0.35">
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>24</v>
       </c>
@@ -2511,7 +1939,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N26">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O26">
         <v>71.636438330973348</v>
@@ -2522,12 +1950,8 @@
       <c r="Q26">
         <v>6.4829231993965921</v>
       </c>
-      <c r="Y26">
-        <f>7.8/Y22</f>
-        <v>4.250076685941977E-3</v>
-      </c>
-    </row>
-    <row r="27" spans="1:27" x14ac:dyDescent="0.35">
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>25</v>
       </c>
@@ -2568,7 +1992,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N27">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O27">
         <v>72.142818929885323</v>
@@ -2579,14 +2003,8 @@
       <c r="Q27">
         <v>6.4829231993965921</v>
       </c>
-      <c r="U27">
-        <v>3681.0367786032052</v>
-      </c>
-      <c r="Y27">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="28" spans="1:27" x14ac:dyDescent="0.35">
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>26</v>
       </c>
@@ -2627,7 +2045,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N28">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O28">
         <v>72.142818929885323</v>
@@ -2638,15 +2056,8 @@
       <c r="Q28">
         <v>6.4829231993965921</v>
       </c>
-      <c r="U28">
-        <v>599.30727457358682</v>
-      </c>
-      <c r="Y28">
-        <f>Y27*Y26</f>
-        <v>4.250076685941977</v>
-      </c>
-    </row>
-    <row r="29" spans="1:27" x14ac:dyDescent="0.35">
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>27</v>
       </c>
@@ -2687,7 +2098,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N29">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O29">
         <v>72.142818929885323</v>
@@ -2699,7 +2110,7 @@
         <v>6.4829231993965921</v>
       </c>
     </row>
-    <row r="30" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>28</v>
       </c>
@@ -2740,7 +2151,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N30">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O30">
         <v>72.142818929885323</v>
@@ -2752,7 +2163,7 @@
         <v>6.4829231993965921</v>
       </c>
     </row>
-    <row r="31" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>29</v>
       </c>
@@ -2793,7 +2204,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N31">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O31">
         <v>72.142818929885323</v>
@@ -2804,16 +2215,8 @@
       <c r="Q31">
         <v>6.4829231993965921</v>
       </c>
-      <c r="S31">
-        <f>(Q36+Q22+Q13+Q12+Q9+Q4)/6</f>
-        <v>6.4829231993965921</v>
-      </c>
-      <c r="U31">
-        <f>SUM(U27:U29)</f>
-        <v>4280.3440531767919</v>
-      </c>
-    </row>
-    <row r="32" spans="1:27" x14ac:dyDescent="0.35">
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>30</v>
       </c>
@@ -2854,7 +2257,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N32">
-        <v>68.072757608527724</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O32">
         <v>71.316161753618118</v>
@@ -2907,7 +2310,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N33">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O33">
         <v>72.142818929885323</v>
@@ -2960,7 +2363,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N34">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O34">
         <v>72.142818929885323</v>
@@ -3013,7 +2416,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N35">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O35">
         <v>70.50800272163886</v>
@@ -3066,7 +2469,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N36">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O36">
         <v>72.320967285165224</v>
@@ -3119,7 +2522,7 @@
         <v>59.076510638297876</v>
       </c>
       <c r="N37">
-        <v>68.015751583500688</v>
+        <v>58.860510638297875</v>
       </c>
       <c r="O37">
         <v>72.142818929885323</v>

</xml_diff>

<commit_message>
add sources for the emission factors
as separate sheet in the input data file
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
+++ b/01_data/01_input_data/02_processed/emission_factors_natural_gas.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{750AA016-7DC5-437F-AF69-47D5C8E6FB30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC3C1942-7EDC-42BA-931F-C16B206DD942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BAA9D55F-0FEB-4558-AFDF-92239B956412}"/>
   </bookViews>
   <sheets>
     <sheet name="Emission_Factors_Import" sheetId="1" r:id="rId1"/>
     <sheet name="Emission_Factors_Domestic" sheetId="2" r:id="rId2"/>
+    <sheet name="Sources" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="70">
   <si>
     <t>AL</t>
   </si>
@@ -196,6 +197,57 @@
   </si>
   <si>
     <t>Node</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>https://www.umweltbundesamt.de/sites/default/files/medien/1410/publikationen/cc_61-2021_emissionsfaktoren-stromerzeugung_bf.pdf</t>
+  </si>
+  <si>
+    <t>Domestic and Russian factor, excluding national (within Germany) part</t>
+  </si>
+  <si>
+    <t>https://www.ifeu.de/fileadmin/uploads/Publikationen/WPKS-Study_Analysis_of_the_greenhouse_gas_intensities_of_LNG_imports_to_Germany.pdf</t>
+  </si>
+  <si>
+    <t>LNG imports, adjusted for distances to different European ports</t>
+  </si>
+  <si>
+    <t>https://www.dcceew.gov.au/sites/default/files/documents/national-greenhouse-account-factors-2023.pdf</t>
+  </si>
+  <si>
+    <t>https://www.publish.csiro.au/EP/EP24202</t>
+  </si>
+  <si>
+    <t>Upstream emissions within Australia</t>
+  </si>
+  <si>
+    <t>https://cleanshipping.org/wp-content/uploads/2025/02/MEPC-83-7-28-Key-considerations-to-determine-the-well-to-tank-WtT-emission-factor-for-liquefied-natur.-Pacific-Environment-CSC.pdf</t>
+  </si>
+  <si>
+    <t>upstream emissions Trinidad and Tobago</t>
+  </si>
+  <si>
+    <t>https://enveurope.springeropen.com/articles/10.1007/s12302-010-0125-6</t>
+  </si>
+  <si>
+    <t>UK and DK are comparable</t>
+  </si>
+  <si>
+    <t>Wie klimafreundlich ist LNG? Kurzstudie zur Bewertung der Vorkettenemissionen bei Nutzung von verflüssigtem Erdgas (LNG)</t>
+  </si>
+  <si>
+    <t>Further factors for LNG imports</t>
+  </si>
+  <si>
+    <t>Upstream Emissions of Fossil Fuel Feedstocks for Transport Fuels Consumed in the EU,  International Council on Clean Transportation (ICCT), 2014</t>
+  </si>
+  <si>
+    <t>Values to scale the factors for further African nodes compared to Algerian emission factor</t>
   </si>
 </sst>
 </file>
@@ -2835,4 +2887,86 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9DE33F9-34E8-4544-981B-AD0FE1A4EE5C}">
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B8" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>68</v>
+      </c>
+      <c r="B9" t="s">
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>